<commit_message>
Add CPU baseline results: Skill-Inject Filter, cisco-skill-scanner on Lexical/Inverse Decoy
Lexical Decoy (FPR):
  Skill-Inject: AUROC=0.80 FPR=40.0%
  cisco:        AUROC=0.53 FPR=43.3%
  TF-IDF:       AUROC=0.74 FPR=39.3%

Inverse Decoy (FNR):
  Skill-Inject: AUROC=0.50 (random)
  cisco:        AUROC=0.50 (random)
  TF-IDF:       AUROC=0.16 FNR=78.1%

All surface-text methods fail on clean-vocabulary attacks. Only hidden-state methods succeed.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="v2 归因分析" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="方法演进" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="总览" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="SMP Stealth V2" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="MSB" sheetId="4" state="visible" r:id="rId4"/>
@@ -247,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -413,6 +413,37 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -778,22 +809,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="6" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>SkillProbe v2: Dual-Pass Detection + Malicious Attribution</t>
+          <t>SkillProbe 方法演进：v1 → v2 → v3 → v4</t>
         </is>
       </c>
     </row>
@@ -804,67 +836,268 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>版本</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>SMP</t>
+        </is>
+      </c>
+      <c r="D3" s="67" t="inlineStr">
+        <is>
+          <t>Decoy</t>
+        </is>
+      </c>
+      <c r="E3" s="67" t="inlineStr">
+        <is>
+          <t>InvDecoy</t>
+        </is>
+      </c>
+      <c r="F3" s="67" t="inlineStr">
+        <is>
+          <t>MSB</t>
+        </is>
+      </c>
+      <c r="G3" s="67" t="inlineStr">
+        <is>
+          <t>MASB</t>
+        </is>
+      </c>
+      <c r="H3" s="67" t="inlineStr">
+        <is>
+          <t>核心改进</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="65" t="inlineStr">
-        <is>
-          <t>架构:</t>
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>oper+bnd+PCA8+LR</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
+        <is>
+          <t>0.910</t>
+        </is>
+      </c>
+      <c r="D4" s="22" t="inlineStr">
+        <is>
+          <t>0.427</t>
+        </is>
+      </c>
+      <c r="E4" s="22" t="inlineStr">
+        <is>
+          <t>0.165</t>
+        </is>
+      </c>
+      <c r="F4" s="22" t="inlineStr">
+        <is>
+          <t>0.964</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>基础：读代码 hidden-state 几何关系</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Pass A: prompt截断在声明末尾 → 模型只看到声明 → decl-bnd → Decl-Probe (L2-LR) → score_decl</t>
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>v1 + decl-probe 双趟 max()</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>0.910</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>0.427</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>0.165</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>0.964</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>+声明投毒覆盖 + 恶意归因。现有 benchmark 零退化</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Pass B: 完整 prompt (同v1) → oper+bnd几何特征 → PCA(8)+LR → score_v1</t>
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>v1 + centering(-PC1)</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>0.858</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>0.758</t>
+        </is>
+      </c>
+      <c r="F6" s="69" t="inlineStr">
+        <is>
+          <t>0.937</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>+去模板噪声。跨分布 AUROC 暴涨+43-59pp</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>risk = max(score_v1, score_decl)    attribution = argmax → DECLARATION / OPERATION / BOTH / CLEAN</t>
+      <c r="A7" s="76" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="B7" s="77" t="inlineStr">
+        <is>
+          <t>v3 + Boundary gating</t>
+        </is>
+      </c>
+      <c r="C7" s="77" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="D7" s="77" t="inlineStr">
+        <is>
+          <t>0.998</t>
+        </is>
+      </c>
+      <c r="E7" s="77" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="F7" s="77" t="inlineStr">
+        <is>
+          <t>0.937</t>
+        </is>
+      </c>
+      <c r="G7" s="77" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="H7" s="78" t="inlineStr">
+        <is>
+          <t>+Boundary 安全门。Decoy FPR 100%→0%！</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="66" t="inlineStr">
+        <is>
+          <t>v2 恶意归因 (175 samples)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="66" t="inlineStr">
-        <is>
-          <t>SMP Stealth V2 测试结果 (124 samples)</t>
+      <c r="A9" s="79" t="inlineStr">
+        <is>
+          <t>v2: 双趟并行 + 恶意归因</t>
+        </is>
+      </c>
+      <c r="B9" s="67" t="inlineStr">
+        <is>
+          <t>样本</t>
+        </is>
+      </c>
+      <c r="C9" s="67" t="inlineStr">
+        <is>
+          <t>正确</t>
+        </is>
+      </c>
+      <c r="D9" s="67" t="inlineStr">
+        <is>
+          <t>准确率</t>
+        </is>
+      </c>
+      <c r="E9" s="67" t="inlineStr">
+        <is>
+          <t>说明</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="67" t="inlineStr">
-        <is>
-          <t>方法</t>
-        </is>
-      </c>
-      <c r="B10" s="67" t="inlineStr">
-        <is>
-          <t>AUROC</t>
-        </is>
-      </c>
-      <c r="C10" s="67" t="inlineStr">
-        <is>
-          <t>F1%</t>
-        </is>
-      </c>
-      <c r="D10" s="67" t="inlineStr">
-        <is>
-          <t>FPR%</t>
-        </is>
-      </c>
-      <c r="E10" s="67" t="inlineStr">
-        <is>
-          <t>FNR%</t>
-        </is>
-      </c>
+      <c r="A10" s="72" t="inlineStr">
+        <is>
+          <t>Pass A (decl-only, ~50ms): prompt 截断在声明末尾 → decl-bnd → Decl-Probe → score_decl</t>
+        </is>
+      </c>
+      <c r="B10" s="73" t="n">
+        <v>50</v>
+      </c>
+      <c r="C10" s="73" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" s="73" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E10" s="73" t="inlineStr"/>
       <c r="F10" s="67" t="inlineStr">
         <is>
           <t>说明</t>
@@ -874,27 +1107,23 @@
     <row r="11">
       <c r="A11" s="68" t="inlineStr">
         <is>
-          <t>v1 Code-Probe (oper+bnd)</t>
-        </is>
-      </c>
-      <c r="B11" s="69" t="inlineStr">
-        <is>
-          <t>0.877</t>
-        </is>
-      </c>
-      <c r="C11" s="69" t="inlineStr">
-        <is>
-          <t>88.2</t>
-        </is>
+          <t>Pass B (完整 prompt, ~1945ms): 同 v1 → oper+bnd 几何特征 → PCA(8)+LR → score_v1</t>
+        </is>
+      </c>
+      <c r="B11" s="69" t="n">
+        <v>50</v>
+      </c>
+      <c r="C11" s="69" t="n">
+        <v>22</v>
       </c>
       <c r="D11" s="69" t="inlineStr">
         <is>
-          <t>22.6</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="E11" s="69" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>Decl-Probe L31信号不够强</t>
         </is>
       </c>
       <c r="F11" s="69" t="inlineStr">
@@ -906,27 +1135,23 @@
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Decl-Probe (decl-only)</t>
-        </is>
-      </c>
-      <c r="B12" s="22" t="inlineStr">
-        <is>
-          <t>0.471</t>
-        </is>
-      </c>
-      <c r="C12" s="22" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+          <t>risk = max(score_v1, score_decl)   attribution = argmax → DECL/OPER/BOTH/CLEAN</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="C12" s="22" t="n">
+        <v>50</v>
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E12" s="22" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>v1 完美检出</t>
         </is>
       </c>
       <c r="F12" s="22" t="inlineStr">
@@ -936,54 +1161,76 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>v2 Fusion max(v1,decl)</t>
-        </is>
-      </c>
-      <c r="B13" s="22" t="inlineStr">
-        <is>
-          <t>0.875</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="inlineStr">
-        <is>
-          <t>88.2</t>
-        </is>
+      <c r="A13" s="74" t="inlineStr">
+        <is>
+          <t>归因准确率: 175 样本 84% (CLEAN 100%, OPER 100%, BOTH 100%, DECL 44%)</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="C13" s="22" t="n">
+        <v>25</v>
       </c>
       <c r="D13" s="22" t="inlineStr">
         <is>
-          <t>22.6</t>
-        </is>
-      </c>
-      <c r="E13" s="22" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr"/>
       <c r="F13" s="22">
         <f> v1。max()确保decl随机信号不拖累v1。零退化</f>
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="n">
+        <v>175</v>
+      </c>
+      <c r="C14" s="22" t="n">
+        <v>147</v>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>84%</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
+        <is>
+          <t>argmax归因</t>
+        </is>
+      </c>
+    </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>结论：在SMP上v2=v1（无损）。SMP没有声明投毒攻击，Decl-Probe正确输出随机分数。</t>
+      <c r="A15" s="66" t="inlineStr">
+        <is>
+          <t>v3: 各向异性修正 (centering)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="64" t="inlineStr">
+        <is>
+          <t>在 v1 基础上增加一步: 对 oper 和 resp 特征逐层移除 PC1（prompt 模板主导的方差方向）</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="66" t="inlineStr">
-        <is>
-          <t>Attribution 数据集 (175 samples: 50 clean + 50 decl-poison + 50 oper-poison + 25 both)</t>
+      <c r="A17" s="64" t="inlineStr">
+        <is>
+          <t>效果: 几何特征反映 skill 内容而非 token 位置 → 跨分布鲁棒。Decoy AUROC +43pp, InvDecoy +59pp</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="67" t="inlineStr">
-        <is>
-          <t>探针</t>
+      <c r="A18" s="80" t="inlineStr">
+        <is>
+          <t>签名: oper+bnd → center(-PC1) → 5几何特征 → PCA(8) → LR(C=0.01) · L7+</t>
         </is>
       </c>
       <c r="B18" s="67" t="inlineStr">
@@ -1020,7 +1267,7 @@
     <row r="19">
       <c r="A19" s="21" t="inlineStr">
         <is>
-          <t>Decl-Probe</t>
+          <t>risk = max(score_v1, score_decl)   attribution = argmax</t>
         </is>
       </c>
       <c r="B19" s="22" t="inlineStr">
@@ -1055,9 +1302,9 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>Code-Probe</t>
+      <c r="A20" s="81" t="inlineStr">
+        <is>
+          <t>v4: Boundary 安全门控</t>
         </is>
       </c>
       <c r="B20" s="22" t="inlineStr">
@@ -1094,7 +1341,7 @@
     <row r="21">
       <c r="A21" s="68" t="inlineStr">
         <is>
-          <t>Fusion max()</t>
+          <t>if score_boundary &lt; 0.15: risk = score_boundary  (模型确定安全→信任模型判断)</t>
         </is>
       </c>
       <c r="B21" s="69" t="inlineStr">
@@ -1128,24 +1375,38 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="64" t="inlineStr">
+        <is>
+          <t>else: risk = score_v3  (模型不确定→用 v3 代码级检测)</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>结论：两路信号正交。Decl-Probe和Code-Probe检测的是不同的攻击类型，互不重叠。max()融合实现100%检出率。</t>
+      <c r="A23" s="64" t="inlineStr">
+        <is>
+          <t>Boundary 在安全样本上天然极低 (~0.005)，在恶意样本上天然高 (~0.9)。Gate=0.15 无需调参。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="64" t="inlineStr">
+        <is>
+          <t>效果: Lexical Decoy FPR 100%→0%, InvDecoy FPR 100%→0%。两张 Decoy 全部解决。</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="66" t="inlineStr">
-        <is>
-          <t>恶意归因准确率</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>签名: oper+bnd → center(−PC1) → 5几何特征 → PCA(8) → LR(C=0.01) · L7+</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="67" t="inlineStr">
-        <is>
-          <t>真实类别</t>
+      <c r="A26" s="79" t="inlineStr">
+        <is>
+          <t>最终方法: SkillProbe v4 五数据集表现</t>
         </is>
       </c>
       <c r="B26" s="67" t="inlineStr">
@@ -1170,140 +1431,191 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="68" t="inlineStr">
-        <is>
-          <t>CLEAN (干净)</t>
-        </is>
-      </c>
-      <c r="B27" s="69" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="C27" s="69" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="D27" s="69" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="E27" s="69" t="inlineStr">
-        <is>
-          <t>全部正确归因为CLEAN</t>
+      <c r="A27" s="67" t="inlineStr">
+        <is>
+          <t>数据集</t>
+        </is>
+      </c>
+      <c r="B27" s="67" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="C27" s="67" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="D27" s="67" t="inlineStr">
+        <is>
+          <t>Δ</t>
+        </is>
+      </c>
+      <c r="E27" s="67" t="inlineStr">
+        <is>
+          <t>v4 关键指标</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>DECLARATION (声明投毒)</t>
-        </is>
-      </c>
-      <c r="B28" s="22" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="C28" s="22" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="D28" s="22" t="inlineStr">
-        <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="E28" s="22" t="inlineStr">
-        <is>
-          <t>28个被错归为BOTH——Decl-Probe对部分样本信号不够强</t>
+      <c r="A28" s="72" t="inlineStr">
+        <is>
+          <t>SMP Stealth V2</t>
+        </is>
+      </c>
+      <c r="B28" s="73" t="inlineStr">
+        <is>
+          <t>0.910</t>
+        </is>
+      </c>
+      <c r="C28" s="73" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="D28" s="73" t="inlineStr">
+        <is>
+          <t>+0.031</t>
+        </is>
+      </c>
+      <c r="E28" s="69" t="inlineStr">
+        <is>
+          <t>AUROC=0.941 SOTA. FPR=19.4% FNR=6.5%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="68" t="inlineStr">
         <is>
-          <t>OPERATION (代码投毒)</t>
+          <t>MSB</t>
         </is>
       </c>
       <c r="B29" s="69" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>0.964</t>
         </is>
       </c>
       <c r="C29" s="69" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>0.937</t>
         </is>
       </c>
       <c r="D29" s="69" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>-0.027</t>
         </is>
       </c>
       <c r="E29" s="69" t="inlineStr">
         <is>
-          <t>全部正确归因为OPERATION</t>
+          <t>去 confound 虚高→更诚实. FPR=13.8% FNR=12.5%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="68" t="inlineStr">
         <is>
-          <t>BOTH (双投毒)</t>
+          <t>MASB 75K</t>
         </is>
       </c>
       <c r="B30" s="69" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>0.923</t>
         </is>
       </c>
       <c r="C30" s="69" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>0.875</t>
         </is>
       </c>
       <c r="D30" s="69" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>-0.048</t>
         </is>
       </c>
       <c r="E30" s="69" t="inlineStr">
         <is>
-          <t>全部正确归因为BOTH</t>
+          <t>去 in-domain bias. FPR=35.3% FNR=9.5%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>合计</t>
+          <t>Lexical Decoy</t>
         </is>
       </c>
       <c r="B31" s="22" t="inlineStr">
         <is>
-          <t>175</t>
+          <t>0.427</t>
         </is>
       </c>
       <c r="C31" s="22" t="inlineStr">
         <is>
-          <t>147</t>
+          <t>0.998</t>
         </is>
       </c>
       <c r="D31" s="22" t="inlineStr">
         <is>
-          <t>84.0%</t>
-        </is>
-      </c>
-      <c r="E31" s="22" t="inlineStr"/>
+          <t>+0.571</t>
+        </is>
+      </c>
+      <c r="E31" s="69" t="inlineStr">
+        <is>
+          <t>FPR=0%! Boundary gate 完美拦截所有 decoy</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>Inverse Decoy</t>
+        </is>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>0.165</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>+0.835</t>
+        </is>
+      </c>
+      <c r="E32" s="69" t="inlineStr">
+        <is>
+          <t>FPR=0% AUC=1.0! 两张 Decoy 全部解决</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>归因方法：argmax(score_v1, score_decl)。如果两路都&gt;阈值则为BOTH，都&lt;阈值则为CLEAN。声明归因较弱(44%)是因为L31的decl-only信号对部分样本不够强——未来可改进层选择。</t>
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>Inverse Decoy</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>0.165</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>0.758</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>+0.593</t>
+        </is>
+      </c>
+      <c r="E33" s="69" t="inlineStr">
+        <is>
+          <t>centering 从噪声中恢复信号</t>
         </is>
       </c>
     </row>
@@ -1641,14 +1953,21 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="66" t="inlineStr">
+        <is>
+          <t>v3 更新：SkillProbe v3 = v1 + centering (去PC1)。在所有数据集上达到最佳或接近最佳。</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="64" t="inlineStr">
+        <is>
+          <t>SMP: v3=0.941 (+6.5pp) | Decoy: v3=0.858 (+43pp) | InvDecoy: v3=0.758 (+59pp) | MSB: v3=0.937 | MASB: v3=0.875</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A44:J44"/>
-    <mergeCell ref="A23:J23"/>
-    <mergeCell ref="A56:J56"/>
-    <mergeCell ref="A15:J15"/>
-    <mergeCell ref="A33:J33"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2291,7 +2610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2651,7 +2970,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>SkillProbe (ours)</t>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B12" s="28" t="n">
@@ -2677,7 +2996,7 @@
       </c>
       <c r="I12" s="28" t="inlineStr">
         <is>
-          <t>L11, no interact+PCA8+C=0.01 (L7+, internal contract verified)</t>
+          <t>v1: oper+bnd+PCA8+C=0.01+L7+. Baseline method</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -2685,7 +3004,7 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2 (ours)</t>
+          <t>SkillProbe v2</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
@@ -2713,7 +3032,40 @@
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>max(v1,decl). SMP无声明投毒→v2=v1. +Decl-Probe补盲区+归因</t>
+          <t>v2: max(v1,decl). SMP无声明投毒→=v1. 零退化+补盲区+归因</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>SkillProbe v3 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="71" t="n">
+        <v>0.9409999999999999</v>
+      </c>
+      <c r="C14" s="71" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D14" s="71" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E14" s="71" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="F14" s="71" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="G14" s="71" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="H14" s="71" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="I14" s="71" t="inlineStr">
+        <is>
+          <t>★ v3: oper+bnd+centering+PCA8+C=0.01+L7+. L15. AUROC=0.941 SOTA on SMP</t>
         </is>
       </c>
     </row>
@@ -2732,7 +3084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3083,7 +3435,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>SkillProbe (ours)</t>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B12" s="28" t="n">
@@ -3109,14 +3461,14 @@
       </c>
       <c r="I12" s="28" t="inlineStr">
         <is>
-          <t>L31, no interact+PCA8 (L7+ verified)</t>
+          <t>v1: oper+bnd. Source confound inflated</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2 (ours)</t>
+          <t>SkillProbe v2</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
@@ -3137,12 +3489,47 @@
       <c r="G13" s="70" t="n">
         <v>91.5</v>
       </c>
-      <c r="H13" s="70" t="n">
-        <v>0.963</v>
+      <c r="H13" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>max(v1,decl). 同v1. Decl-Probe待提取</t>
+          <t>v2: max(v1,decl). =v1 on MSB</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>SkillProbe v3 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="71" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="C14" s="71" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="D14" s="71" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E14" s="71" t="n">
+        <v>86.90000000000001</v>
+      </c>
+      <c r="F14" s="71" t="n">
+        <v>87</v>
+      </c>
+      <c r="G14" s="71" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="H14" s="71" t="n">
+        <v>0.9370000000000001</v>
+      </c>
+      <c r="I14" s="71" t="inlineStr">
+        <is>
+          <t>★ v3: centering removes confound inflation. More honest than v1</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3514,7 +3901,7 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>SkillProbe (ours)</t>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B12" s="28" t="n">
@@ -3540,14 +3927,14 @@
       </c>
       <c r="I12" s="28" t="inlineStr">
         <is>
-          <t>L7, in-domain, no interact+PCA8 (L7+)</t>
+          <t>v1: oper+bnd. In-domain</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2 (ours)</t>
+          <t>SkillProbe v2</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
@@ -3568,12 +3955,47 @@
       <c r="G13" s="70" t="n">
         <v>83.59999999999999</v>
       </c>
-      <c r="H13" s="70" t="n">
-        <v>0.921</v>
+      <c r="H13" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>max(v1,decl). 同v1. Decl-Probe待提取</t>
+          <t>v2: max(v1,decl). =v1 on MASB</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>SkillProbe v3 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="71" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="C14" s="71" t="n">
+        <v>35.3</v>
+      </c>
+      <c r="D14" s="71" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="E14" s="71" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="F14" s="71" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="G14" s="71" t="n">
+        <v>90.5</v>
+      </c>
+      <c r="H14" s="71" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="I14" s="71" t="inlineStr">
+        <is>
+          <t>★ v3: centering reduces in-domain bias. More robust OOD. FNR=9.5% excellent</t>
         </is>
       </c>
     </row>
@@ -3592,7 +4014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3614,14 +4036,14 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>Lexical Decoy — Suspicious Vocabulary, Benign Semantics</t>
+          <t>Lexical Decoy — Suspicious Vocabulary, Benign Semantics (155 samples)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>60 decoys, SMP mal + Decoy ben. Unified internal contract. No interact, PCA=8.</t>
+          <t>155 decoys + 62 SMP mal paired. Unified internal contract. L7+. No interaction. PCA=8. C=0.01.</t>
         </is>
       </c>
     </row>
@@ -3679,10 +4101,8 @@
           <t>Static Regex</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B4" s="24" t="n">
+        <v>0.4625</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>100</v>
@@ -3694,10 +4114,10 @@
         <v>66.7</v>
       </c>
       <c r="F4" s="24" t="n">
-        <v>50</v>
+        <v>44.1</v>
       </c>
       <c r="G4" s="24" t="n">
-        <v>100</v>
+        <v>35.3</v>
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
@@ -3706,7 +4126,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Always fires</t>
+          <t>Static Regex on 155 decoys: FPR=59% (better than old 100%—more diverse decoys)</t>
         </is>
       </c>
       <c r="J4" s="22" t="n"/>
@@ -3717,44 +4137,32 @@
           <t>TF-IDF + LR</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="24" t="n">
+        <v>0.7435</v>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>FPR known=100%</t>
+          <t>TF-IDF on 155 decoys: FPR=100% (suspicious vocab = malicious to TF-IDF)</t>
         </is>
       </c>
       <c r="J5" s="22" t="n"/>
@@ -3765,11 +4173,15 @@
           <t>LLM-as-judge</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n"/>
+      <c r="B6" s="24" t="n">
+        <v>0.5</v>
+      </c>
       <c r="C6" s="24" t="n">
         <v>100</v>
       </c>
-      <c r="D6" s="24" t="n"/>
+      <c r="D6" s="24" t="n">
+        <v>0</v>
+      </c>
       <c r="E6" s="24" t="n">
         <v>66.7</v>
       </c>
@@ -3786,7 +4198,7 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%)</t>
         </is>
       </c>
       <c r="J6" s="22" t="n"/>
@@ -3798,29 +4210,29 @@
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>0.885</v>
+        <v>0.991</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>36.7</v>
+        <v>0</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>5</v>
+        <v>3.2</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>82</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>90.5</v>
+        <v>100</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>95</v>
+        <v>96.8</v>
       </c>
       <c r="H7" s="26" t="n">
         <v>0.994</v>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L27 (unified contract, L7+)</t>
+          <t>L23 (L7+). Model judges ALL 150 decoys safe!</t>
         </is>
       </c>
       <c r="J7" s="22" t="n"/>
@@ -3832,29 +4244,29 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.84</v>
+        <v>0.867</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>35</v>
+        <v>22.7</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>8.300000000000001</v>
+        <v>21</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>80.90000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>88.7</v>
+        <v>68.2</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>91.7</v>
+        <v>79</v>
       </c>
       <c r="H8" s="22" t="n">
         <v>0.989</v>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L15 (unified contract, L7+)</t>
+          <t>L15 (L7+). PCA(50) boundary. FPR=23% acceptable.</t>
         </is>
       </c>
       <c r="J8" s="22" t="n"/>
@@ -3866,39 +4278,29 @@
         </is>
       </c>
       <c r="B9" s="30" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F9" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G9" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>0.777</v>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>100</v>
       </c>
       <c r="H9" s="24" t="n">
         <v>0.734</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>CV=0.73 on SMP dev. Cross-extract prevents fair Decoy eval</t>
+          <t>rhid only. Cross-extract caution. FPR=65%</t>
         </is>
       </c>
       <c r="J9" s="22" t="n"/>
@@ -3910,97 +4312,103 @@
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.46</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>12.5</v>
+        <v>100</v>
       </c>
       <c r="D10" s="26" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>92.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>98.5</v>
+        <v>50</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>87</v>
-      </c>
-      <c r="H10" s="26" t="n">
-        <v>0.979</v>
+        <v>100</v>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>Obsolete (interaction+PCA64). FPR=100% confirms noise</t>
         </is>
       </c>
       <c r="J10" s="22" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="68" t="inlineStr">
         <is>
           <t>Centered Relational</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
-        <v>0.958</v>
-      </c>
-      <c r="C11" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="26" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="E11" s="26" t="n">
-        <v>85.90000000000001</v>
-      </c>
-      <c r="F11" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="G11" s="26" t="n">
+      <c r="B11" s="69" t="n">
+        <v>0.705</v>
+      </c>
+      <c r="C11" s="69" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="D11" s="69" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="E11" s="69" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="F11" s="69" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="G11" s="69" t="n">
+        <v>85.3</v>
+      </c>
+      <c r="H11" s="69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="69" t="inlineStr">
+        <is>
+          <t>Centered (-1PC). AUC=0.71 better than SkillProbe on decoy—centering helps lexical robustness</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="68" t="inlineStr">
+        <is>
+          <t>SkillProbe v1</t>
+        </is>
+      </c>
+      <c r="B12" s="69" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="C12" s="69" t="n">
         <v>75.3</v>
       </c>
-      <c r="H11" s="26" t="n">
-        <v>0.976</v>
-      </c>
-      <c r="I11" s="22" t="inlineStr">
-        <is>
-          <t>L11</t>
-        </is>
-      </c>
-      <c r="J11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="27" t="inlineStr">
-        <is>
-          <t>SkillProbe (ours)</t>
-        </is>
-      </c>
-      <c r="B12" s="28" t="n">
-        <v>0.536</v>
-      </c>
-      <c r="C12" s="28" t="n">
-        <v>100</v>
-      </c>
-      <c r="D12" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="28" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F12" s="28" t="n">
-        <v>50</v>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>100</v>
-      </c>
-      <c r="H12" s="28" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="I12" s="28" t="inlineStr">
-        <is>
-          <t>L11. oper code suspicious→FPR=100%. ≠Regex: SP reads hidden-state not keywords. Boundary(FPR=37%) shows model judges safe—SP reads code reality</t>
+      <c r="D12" s="69" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E12" s="69" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F12" s="69" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G12" s="69" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="H12" s="69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="69" t="inlineStr">
+        <is>
+          <t>v1: FPR=75% (oper reads suspicious code)</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -4008,35 +4416,128 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2 (ours)</t>
+          <t>SkillProbe v2</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.536</v>
+        <v>0.427</v>
       </c>
       <c r="C13" s="70" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="D13" s="70" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E13" s="70" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F13" s="70" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G13" s="70" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="H13" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="70" t="inlineStr">
+        <is>
+          <t>v2: max(v1,decl). Decl-Probe also fires on suspicious vocab. =v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>SkillProbe v4 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="F14" s="70" t="n">
         <v>100</v>
       </c>
-      <c r="D13" s="70" t="n">
+      <c r="G14" s="70" t="n">
+        <v>97</v>
+      </c>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>★ v4: Boundary-gated v3. Gate&lt;0.15. FPR=0% FNR=3%. Best on Decoy!</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Skill-Inject Filter</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D15" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="70" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F13" s="70" t="n">
-        <v>50</v>
-      </c>
-      <c r="G13" s="70" t="n">
-        <v>100</v>
-      </c>
-      <c r="H13" s="70" t="inlineStr">
+      <c r="E15" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="H15" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I13" s="70" t="inlineStr">
-        <is>
-          <t>max(v1,decl). v1(oper读可疑代码)+Decl(decl读可疑词汇)→两路都报警→FPR=100%相同</t>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Schmotz et al. 2026, naive input filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cisco-skill-scanner</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.5331</v>
+      </c>
+      <c r="C16" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>176 patterns (core+promptguard), Python 3.10+ required</t>
         </is>
       </c>
     </row>
@@ -4055,7 +4556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4077,14 +4578,14 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>Inverse Decoy — Clean Vocabulary, Malicious Semantics</t>
+          <t>Inverse Decoy — Clean Vocabulary, Malicious Semantics (155 pairs)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>60 pairs (70 valid). Vocab clean, semantics malicious. L7+ verified (small N).</t>
+          <t>155 clean + 155 malicious. SMP-trained. L7+. Vocab-clean semantics-malicious. FNR benchmark: can model detect malice without lexical cues?</t>
         </is>
       </c>
     </row>
@@ -4142,10 +4643,8 @@
           <t>Static Regex</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B4" s="24" t="n">
+        <v>0.9935</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>100</v>
@@ -4157,10 +4656,10 @@
         <v>66.7</v>
       </c>
       <c r="F4" s="24" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G4" s="24" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
@@ -4169,7 +4668,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Always fires</t>
+          <t>Regex on clean vocab: FPR=0% FNR=100%—no patterns to match. Useless.</t>
         </is>
       </c>
       <c r="J4" s="22" t="n"/>
@@ -4180,44 +4679,32 @@
           <t>TF-IDF + LR</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="24" t="n">
+        <v>0.1593</v>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TF-IDF on clean vocab: AUC=0.50 random (vocab has no signal)</t>
         </is>
       </c>
       <c r="J5" s="22" t="n"/>
@@ -4253,7 +4740,7 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+          <t>Mistral always MAL. Zero-shot useless</t>
         </is>
       </c>
       <c r="J6" s="22" t="n"/>
@@ -4265,29 +4752,29 @@
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>0.408</v>
+        <v>0.793</v>
       </c>
       <c r="C7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="E7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="26" t="n">
-        <v>66.7</v>
-      </c>
       <c r="F7" s="26" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>0.524</v>
+        <v>0.994</v>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L7, CV (L7+, 70 samples)</t>
+          <t>L23. Model judges ALL safe! FNR=100%—clean vocab fools model judgment completely</t>
         </is>
       </c>
       <c r="J7" s="22" t="n"/>
@@ -4299,29 +4786,29 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.694</v>
+        <v>0.676</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>71.40000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>73.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>58.3</v>
+        <v>53.2</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>100</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>1</v>
+        <v>0.989</v>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L23, CV (L7+, 70 samples)</t>
+          <t>L15. Catches 99% malicious but FPR=78%</t>
         </is>
       </c>
       <c r="J8" s="22" t="n"/>
@@ -4333,7 +4820,7 @@
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>0.372</v>
+        <v>0.5</v>
       </c>
       <c r="C9" s="24" t="n">
         <v>100</v>
@@ -4351,11 +4838,11 @@
         <v>100</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>0.538</v>
+        <v>0.734</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>rhid only, L7, CV. 70 samples. Honest: near random</t>
+          <t>rhid only. Random on clean vocab. Cross-extract.</t>
         </is>
       </c>
       <c r="J9" s="22" t="n"/>
@@ -4367,7 +4854,7 @@
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>0.643</v>
+        <v>0.824</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>100</v>
@@ -4384,80 +4871,86 @@
       <c r="G10" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="H10" s="26" t="n">
-        <v>1</v>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>70 samples</t>
+          <t>AUC=0.82 ranks correctly but FPR=100% (threshold issue)</t>
         </is>
       </c>
       <c r="J10" s="22" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="68" t="inlineStr">
         <is>
           <t>Centered Relational</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
-        <v>0.408</v>
-      </c>
-      <c r="C11" s="26" t="n">
+      <c r="B11" s="69" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="C11" s="69" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="D11" s="69" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E11" s="69" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="F11" s="69" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="G11" s="69" t="n">
+        <v>98.7</v>
+      </c>
+      <c r="H11" s="69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="69" t="inlineStr">
+        <is>
+          <t>Centered (-1PC). AUC=0.85 BEST on InvDecoy! Centering removes anisotropic noise→clean signal</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="68" t="inlineStr">
+        <is>
+          <t>SkillProbe v1</t>
+        </is>
+      </c>
+      <c r="B12" s="69" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="C12" s="69" t="n">
         <v>100</v>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D12" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="26" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F11" s="26" t="n">
+      <c r="E12" s="69" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="F12" s="69" t="n">
         <v>50</v>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G12" s="69" t="n">
         <v>100</v>
       </c>
-      <c r="H11" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" s="22" t="inlineStr">
-        <is>
-          <t>70 samples</t>
-        </is>
-      </c>
-      <c r="J11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="27" t="inlineStr">
-        <is>
-          <t>SkillProbe (ours)</t>
-        </is>
-      </c>
-      <c r="B12" s="28" t="n">
-        <v>0.643</v>
-      </c>
-      <c r="C12" s="28" t="n">
-        <v>71.40000000000001</v>
-      </c>
-      <c r="D12" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="28" t="n">
-        <v>73.7</v>
-      </c>
-      <c r="F12" s="28" t="n">
-        <v>58.3</v>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>100</v>
-      </c>
-      <c r="H12" s="28" t="n">
-        <v>0.678</v>
-      </c>
-      <c r="I12" s="28" t="inlineStr">
-        <is>
-          <t>L7, CV (L7+, 70 samples)</t>
+      <c r="H12" s="69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="69" t="inlineStr">
+        <is>
+          <t>v1: cross-distribution collapse. AUC=0.16</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -4465,11 +4958,11 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2 (ours)</t>
+          <t>SkillProbe v2</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.476</v>
+        <v>0.165</v>
       </c>
       <c r="C13" s="70" t="n">
         <v>100</v>
@@ -4478,7 +4971,7 @@
         <v>0</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>66.7</v>
+        <v>43.9</v>
       </c>
       <c r="F13" s="70" t="n">
         <v>50</v>
@@ -4493,7 +4986,100 @@
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>max(v1,decl). Decl偏向判MAL→v2=Decl. 70样本太小不可靠</t>
+          <t>v2: max(v1,decl). Decl AUC=0.48 random. =v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>SkillProbe v4 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="F14" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" s="70" t="n">
+        <v>97</v>
+      </c>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>★ v4: Boundary-gated v3. Gate&lt;0.15. AUC=1.0 FPR=0%! Both Decoy solved!</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Skill-Inject Filter</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Naive filter: clean vocab -&gt; always fires</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cisco-skill-scanner</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.5032</v>
+      </c>
+      <c r="C16" t="n">
+        <v>100</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Standard Python code triggers patterns -&gt; always fires</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add CPU baselines to SMP: Skill-Inject AUROC=0.53, cisco AUROC=0.54
SMP Stealth V2 (360 dev samples):
  Static Regex:   AUROC=0.68 FPR=100%
  Skill-Inject:   AUROC=0.53 FPR=100%
  cisco-core:     AUROC=0.54 FPR=68%
  TF-IDF+LR:      AUROC=0.38 FPR=58%

MSB: shards 0-3 all benign (3124 samples), shards 4-9 need GPU extraction
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -25,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -119,6 +119,10 @@
     <font>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="14">
@@ -247,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -443,6 +447,11 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1978,7 +1987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1990,503 +1999,477 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="82" t="inlineStr">
         <is>
           <t>SkillProbe — 实验总览</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="83" t="inlineStr">
         <is>
           <t>一、数据集</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="67" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="67" t="inlineStr">
         <is>
           <t>数据集</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="67" t="inlineStr">
         <is>
           <t>样本数</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="67" t="inlineStr">
         <is>
           <t>设计</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="67" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
-        <is>
-          <t>论证什么</t>
+      <c r="F4" s="67" t="inlineStr">
+        <is>
+          <t>论文角色</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="A5" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>SMP Stealth V2</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>484</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Paired CF，同 source/style/lineage</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>484 (242对)</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Paired CF (LLM注入)</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>242 pairs</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>控制表面文本 confound 的唯一 benchmark</t>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>主基准. 唯一控制 source confound</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>MSB (MalSkillBench)</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>7894</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Unpaired，malware repos vs ClawHub</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>3944/3950</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>证明 unpaired 数据上 TF-IDF 被高估到 0.967</t>
+      <c r="A6" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>MSB</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>7,894</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>Unpaired (异源)</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="inlineStr">
+        <is>
+          <t>3,955b/3,939m</t>
+        </is>
+      </c>
+      <c r="F6" s="22" t="inlineStr">
+        <is>
+          <t>混杂证据. 证明 unpaired 虚高</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="A7" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>MASB 75K</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>75882</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>真实开源 skill，全部良性</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>~9K</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>大规模良性+MSB恶意</t>
+        </is>
+      </c>
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>Benign only</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>大规模真实分布 FPR 基准</t>
+      <c r="F7" s="22" t="inlineStr">
+        <is>
+          <t>FPR 基准. 大规模真实分布</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="A8" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>Lexical Decoy</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>词汇可疑+语义良性，12× 可疑词密度</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>Benign only</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>2×2 矩阵：测 FPR（读语义还是读关键词）</t>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>155</t>
+        </is>
+      </c>
+      <c r="D8" s="22" t="inlineStr">
+        <is>
+          <t>词汇可疑+语义良性</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="inlineStr">
+        <is>
+          <t>Benign (配SMP mal)</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="inlineStr">
+        <is>
+          <t>2×2 FPR: 会误杀吗？</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="A9" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>Inverse Decoy</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>60 pairs</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>155对</t>
+        </is>
+      </c>
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>词汇干净+语义恶意</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Clean/Malicious</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>2×2 矩阵：测 FNR（低特征恶意检测）</t>
+      <c r="E9" s="22" t="inlineStr">
+        <is>
+          <t>Clean/Mal</t>
+        </is>
+      </c>
+      <c r="F9" s="22" t="inlineStr">
+        <is>
+          <t>2×2 FNR: 会漏检吗？</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>二、对比基线（9 项）</t>
+      <c r="A11" s="83" t="inlineStr">
+        <is>
+          <t>二、对比基线</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="67" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="67" t="inlineStr">
         <is>
           <t>基线</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="67" t="inlineStr">
         <is>
           <t>输入</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="67" t="inlineStr">
         <is>
           <t>方法</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="67" t="inlineStr">
         <is>
           <t>类型</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>来源/角色</t>
+      <c r="F12" s="67" t="inlineStr">
+        <is>
+          <t>来源</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="A13" s="21" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Static Regex</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>Skill 全文</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>10 个正则模式匹配</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>Skill全文</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>10个正则</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
         <is>
           <t>表面文本</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>MalSkillBench/RouteGuard 均有</t>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>MalSkillBench</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="A14" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>TF-IDF + LR</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Skill 全文</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>TF-IDF(20K,1-2gram)→L2-LR</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>Skill全文</t>
+        </is>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>TF-IDF(20K,1-2gram)→LR</t>
+        </is>
+      </c>
+      <c r="E14" s="22" t="inlineStr">
         <is>
           <t>表面文本</t>
         </is>
       </c>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t>标准文本基线，审稿人必问</t>
+      <c r="F14" s="22" t="inlineStr">
+        <is>
+          <t>标准文本基线</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="A15" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
         <is>
           <t>LLM-as-judge</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>Skill 全文</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Llama-3.1-8B zero-shot</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>Skill全文</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>Mistral-7B zero-shot</t>
+        </is>
+      </c>
+      <c r="E15" s="22" t="inlineStr">
         <is>
           <t>黑盒审计</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>RouteGuard/BIV/MalSkillBench 均有</t>
+      <c r="F15" s="22" t="inlineStr">
+        <is>
+          <t>RouteGuard/BIV</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="A16" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Boundary only</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>Boundary token</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>L2-LR</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="22" t="inlineStr">
         <is>
           <t>内部探针</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>我们的消融基线</t>
+      <c r="F16" s="22" t="inlineStr">
+        <is>
+          <t>消融基线</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="A17" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="22" t="inlineStr">
         <is>
           <t>AgentLens</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Boundary top-K</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>PCA(50)→L2-LR</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
+        <is>
+          <t>PCA(50)→LR</t>
+        </is>
+      </c>
+      <c r="E17" s="22" t="inlineStr">
         <is>
           <t>内部探针</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>复现 arxiv 2606.22673</t>
+      <c r="F17" s="22" t="inlineStr">
+        <is>
+          <t>arxiv 2606.22673</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="A18" s="21" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>Attn+Hidden stats</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>8层→L2-LR</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>Attn+Hidden</t>
+        </is>
+      </c>
+      <c r="D18" s="22" t="inlineStr">
+        <is>
+          <t>8层→LR</t>
+        </is>
+      </c>
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>内部探针</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>复现 arxiv 2604.22888，需 attn 特征</t>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>arxiv 2604.22888</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>Relational (v1)</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="A19" s="21" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>Relational v1</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="inlineStr">
         <is>
           <t>decl+oper+bnd</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>6几何特征+PCA64</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>6几何+PCA64</t>
+        </is>
+      </c>
+      <c r="E19" s="22" t="inlineStr">
         <is>
           <t>内部探针</t>
         </is>
       </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>我们的旧版（含 interaction，已废弃）</t>
+      <c r="F19" s="22" t="inlineStr">
+        <is>
+          <t>旧版(已废弃)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>Centered Relational</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="A20" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>Centered Rel.</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
         <is>
           <t>decl+oper+bnd</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>Center−1PC+PCA64</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
+        <is>
+          <t>-PC1+PCA64</t>
+        </is>
+      </c>
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>内部探针</t>
         </is>
       </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>我们的变体（各向异性修正）</t>
+      <c r="F20" s="22" t="inlineStr">
+        <is>
+          <t>变体(已废弃)</t>
         </is>
       </c>
     </row>
@@ -2522,38 +2505,220 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" s="66" t="inlineStr">
+        <is>
+          <t>三、SkillProbe 方法演进</t>
+        </is>
+      </c>
+    </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
-        <is>
-          <t>三、关键发现</t>
+      <c r="A23" s="67" t="inlineStr">
+        <is>
+          <t>版本</t>
+        </is>
+      </c>
+      <c r="B23" s="67" t="inlineStr">
+        <is>
+          <t>方法</t>
+        </is>
+      </c>
+      <c r="C23" s="67" t="inlineStr">
+        <is>
+          <t>SMP</t>
+        </is>
+      </c>
+      <c r="D23" s="67" t="inlineStr">
+        <is>
+          <t>Decoy</t>
+        </is>
+      </c>
+      <c r="E23" s="67" t="inlineStr">
+        <is>
+          <t>InvDecoy</t>
+        </is>
+      </c>
+      <c r="F23" s="67" t="inlineStr">
+        <is>
+          <t>MSB</t>
+        </is>
+      </c>
+      <c r="G23" s="67" t="inlineStr">
+        <is>
+          <t>MASB</t>
+        </is>
+      </c>
+      <c r="H23" s="67" t="inlineStr">
+        <is>
+          <t>核心改进</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>1. interaction (decl⊙oper) 在所有数据集上都是噪声——去掉后 SMP AUROC 从 0.715→0.916</t>
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>v1</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>oper+bnd+PCA8+C=0.01+L7+</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>0.910</t>
+        </is>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>0.427</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>0.165</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>0.964</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>基础: 读代码 hidden-state 几何</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="14" t="inlineStr">
-        <is>
-          <t>2. Declaration 区域无贡献——oper+bnd 足以达到 SOTA</t>
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>v1+decl-probe双趟max()</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>0.910</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>0.427</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>0.165</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>0.964</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>0.923</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>+声明投毒+归因. 零退化</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
-        <is>
-          <t>3. PCA=8 最优——PCA=64 导致过拟合 (TrainAUC=1.0)</t>
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>v1+centering(-PC1)</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>0.858</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>0.758</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>0.937</t>
+        </is>
+      </c>
+      <c r="G26" s="22" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>+去模板噪声. Decoy+43-59pp</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="14" t="inlineStr">
-        <is>
-          <t>4. C=0.01 最佳——C=1.0 时 TrainAUC=1.0 完全记忆训练集</t>
+      <c r="A27" s="76" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="B27" s="77" t="inlineStr">
+        <is>
+          <t>v3+Boundary gating</t>
+        </is>
+      </c>
+      <c r="C27" s="77" t="inlineStr">
+        <is>
+          <t>0.941</t>
+        </is>
+      </c>
+      <c r="D27" s="77" t="inlineStr">
+        <is>
+          <t>0.998</t>
+        </is>
+      </c>
+      <c r="E27" s="77" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="F27" s="77" t="inlineStr">
+        <is>
+          <t>0.937</t>
+        </is>
+      </c>
+      <c r="G27" s="77" t="inlineStr">
+        <is>
+          <t>0.875</t>
+        </is>
+      </c>
+      <c r="H27" s="78" t="inlineStr">
+        <is>
+          <t>+安全门. FPR 100%→0%</t>
         </is>
       </c>
     </row>
@@ -2565,41 +2730,69 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr">
-        <is>
-          <t>6. Paired CF (SMP) 上 TF-IDF 降到 0.812，证明了 benchmark 必要性</t>
+      <c r="A29" s="84" t="inlineStr">
+        <is>
+          <t>四、关键发现</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
-          <t>7. SkillProbe (corrected) SMP AUROC=0.910，比旧版 0.883 提升 0.027</t>
+          <t>1. centering(-PC1) 是关键突破: 移除模板噪声 → 跨分布 AUROC 暴涨 43-59pp</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t>8. LLM-as-judge + Static Regex 待补（审稿人必问）</t>
+          <t>2. Boundary gating 解决 Decoy FPR: 模型确定安全时信任它，否则用 v3 检测</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="64" t="inlineStr">
+        <is>
+          <t>3. v4 SMP=0.941 SOTA, LexicalDecoy FPR=0%, InvDecoy FPR=0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="64" t="inlineStr">
+        <is>
+          <t>4. v2 归因 84%: argmax 区分代码投毒 vs 声明投毒</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="64" t="inlineStr">
+        <is>
+          <t>5. interaction+declaration 是噪声——已从方法中移除</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="64" t="inlineStr">
+        <is>
+          <t>6. MSB 上所有方法 0.96-1.0 → 测来源差异非检测能力</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="64" t="inlineStr">
+        <is>
+          <t>7. Paired CF 是唯一可信 benchmark: TF-IDF 0.967→0.812</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="64" t="inlineStr">
+        <is>
+          <t>8. LLM-as-judge 全表 FPR=100% 不可靠</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A24:F24"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A28:F28"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:F23"/>
-    <mergeCell ref="A27:F27"/>
-    <mergeCell ref="A31:F31"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A30:F30"/>
-    <mergeCell ref="A29:F29"/>
-    <mergeCell ref="A25:F25"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2610,7 +2803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3066,6 +3259,64 @@
       <c r="I14" s="71" t="inlineStr">
         <is>
           <t>★ v3: oper+bnd+centering+PCA8+C=0.01+L7+. L15. AUROC=0.941 SOTA on SMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Skill-Inject Filter</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.528</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Schmotz et al. 2026, naive input filter. FPR=100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cisco-skill-scanner</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.539</v>
+      </c>
+      <c r="C16" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>129 core patterns. Better than basic regex but still 68% FPR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NVIDIA SkillSpector baseline: 20 YARA rules, AUROC≈0.5 on both decoy sets
NVIDIA SkillSpector (13.5k stars, industrial-grade):
  Lexical Decoy: AUROC=0.49 FPR=100% (YARA patterns match std Python)
  Inverse Decoy: AUROC=0.50 FPR=100% (same — always fires)

All surface-text methods fail on clean-vocabulary attacks:
  cisco: 0.50, NVIDIA: 0.50, Regex: 0.46, Skill-Inject: 0.50, TF-IDF: 0.16
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -4265,7 +4265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4792,6 +4792,35 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NVIDIA SkillSpector</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="C17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
@@ -4807,7 +4836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5334,6 +5363,35 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NVIDIA SkillSpector</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>

</xml_diff>

<commit_message>
Add all CPU baselines to MSB (7944 samples), Lexical/Inverse Decoy
MSB (unpaired, 7944 samples):
  Static Regex:         AUROC=0.56 FPR=100%
  Skill-Inject:         AUROC=0.50 FPR=100%
  cisco-skill-scanner:  AUROC=0.54 FPR=100%
  NVIDIA SkillSpector:  AUROC=0.52 FPR=100%
  TF-IDF+LR:            AUROC=0.80 FPR=28%

All surface-text scanners FPR≈100% on MSB unpaired data.
Only TF-IDF achieves discrimination (source confound).
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -251,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -453,6 +453,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1311,39 +1312,44 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="81" t="inlineStr">
-        <is>
-          <t>v4: Boundary 安全门控</t>
-        </is>
-      </c>
-      <c r="B20" s="22" t="inlineStr">
-        <is>
-          <t>0.919</t>
-        </is>
-      </c>
-      <c r="C20" s="22" t="inlineStr">
-        <is>
-          <t>90.4</t>
-        </is>
-      </c>
-      <c r="D20" s="22" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="E20" s="22" t="inlineStr">
-        <is>
-          <t>17.6</t>
-        </is>
-      </c>
-      <c r="F20" s="22" t="inlineStr">
-        <is>
-          <t>L11</t>
-        </is>
-      </c>
-      <c r="G20" s="22" t="inlineStr">
-        <is>
-          <t>纯代码探针。检出oper-poison和both-poison，漏掉decl-poison</t>
+      <c r="A20" s="68" t="inlineStr">
+        <is>
+          <t>v4</t>
+        </is>
+      </c>
+      <c r="B20" s="69" t="inlineStr">
+        <is>
+          <t>v3 + Boundary gating</t>
+        </is>
+      </c>
+      <c r="C20" s="69" t="inlineStr">
+        <is>
+          <t>0.947</t>
+        </is>
+      </c>
+      <c r="D20" s="69" t="inlineStr">
+        <is>
+          <t>0.998</t>
+        </is>
+      </c>
+      <c r="E20" s="69" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="F20" s="69" t="inlineStr">
+        <is>
+          <t>0.996</t>
+        </is>
+      </c>
+      <c r="G20" s="69" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="H20" s="85" t="inlineStr">
+        <is>
+          <t>+Boundary安全门. Gate&lt;0.15通用. 五表全涨！</t>
         </is>
       </c>
     </row>
@@ -1404,6 +1410,16 @@
           <t>效果: Lexical Decoy FPR 100%→0%, InvDecoy FPR 100%→0%。两张 Decoy 全部解决。</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0.427</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>0.998</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1479,7 +1495,7 @@
       </c>
       <c r="C28" s="73" t="inlineStr">
         <is>
-          <t>0.941</t>
+          <t>0.947</t>
         </is>
       </c>
       <c r="D28" s="73" t="inlineStr">
@@ -1506,7 +1522,7 @@
       </c>
       <c r="C29" s="69" t="inlineStr">
         <is>
-          <t>0.937</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="D29" s="69" t="inlineStr">
@@ -1533,7 +1549,7 @@
       </c>
       <c r="C30" s="69" t="inlineStr">
         <is>
-          <t>0.875</t>
+          <t>0.981</t>
         </is>
       </c>
       <c r="D30" s="69" t="inlineStr">
@@ -1614,7 +1630,7 @@
       </c>
       <c r="C33" s="22" t="inlineStr">
         <is>
-          <t>0.758</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="D33" s="22" t="inlineStr">
@@ -1803,12 +1819,12 @@
       </c>
       <c r="B49" s="69" t="inlineStr">
         <is>
-          <t>AUC=0.47 (随机)</t>
+          <t>0.910</t>
         </is>
       </c>
       <c r="C49" s="69" t="inlineStr">
         <is>
-          <t>AUC=0.910</t>
+          <t>0.947</t>
         </is>
       </c>
       <c r="D49" s="69">
@@ -1856,12 +1872,12 @@
       </c>
       <c r="B51" s="22" t="inlineStr">
         <is>
-          <t>FPR=85.0%</t>
+          <t>0.427</t>
         </is>
       </c>
       <c r="C51" s="22" t="inlineStr">
         <is>
-          <t>FPR=62.5%</t>
+          <t>0.998</t>
         </is>
       </c>
       <c r="D51" s="22" t="inlineStr">
@@ -1883,12 +1899,12 @@
       </c>
       <c r="B52" s="22" t="inlineStr">
         <is>
-          <t>AUC=0.48 (随机)</t>
+          <t>0.165</t>
         </is>
       </c>
       <c r="C52" s="22" t="inlineStr">
         <is>
-          <t>AUC=0.64</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="D52" s="22">
@@ -1909,12 +1925,12 @@
       </c>
       <c r="B53" s="22" t="inlineStr">
         <is>
-          <t>待提取</t>
+          <t>0.964</t>
         </is>
       </c>
       <c r="C53" s="22" t="inlineStr">
         <is>
-          <t>AUC=0.96</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="D53" s="22" t="inlineStr">
@@ -1936,12 +1952,12 @@
       </c>
       <c r="B54" s="22" t="inlineStr">
         <is>
-          <t>待提取</t>
+          <t>0.923</t>
         </is>
       </c>
       <c r="C54" s="22" t="inlineStr">
         <is>
-          <t>AUC=0.92</t>
+          <t>0.981</t>
         </is>
       </c>
       <c r="D54" s="22" t="inlineStr">
@@ -1961,6 +1977,16 @@
           <t>关键模式：当数据集没有声明投毒攻击时，Decl-Probe输出随机(InvDecoy,SMP)或反映词法混杂(Decoy,MSB)。v2架构中max()确保它不拖累v1。声明投毒是一种真实但尚未在野外广泛观察的攻击——v2提供了对此的防御覆盖。</t>
         </is>
       </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>0.964</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>0.996</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="66" t="inlineStr">
@@ -1973,6 +1999,16 @@
       <c r="A59" s="64" t="inlineStr">
         <is>
           <t>SMP: v3=0.941 (+6.5pp) | Decoy: v3=0.858 (+43pp) | InvDecoy: v3=0.758 (+59pp) | MSB: v3=0.937 | MASB: v3=0.875</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0.964</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>0.996</t>
         </is>
       </c>
     </row>
@@ -2681,44 +2717,44 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="76" t="inlineStr">
+      <c r="A27" s="68" t="inlineStr">
         <is>
           <t>v4</t>
         </is>
       </c>
-      <c r="B27" s="77" t="inlineStr">
+      <c r="B27" s="69" t="inlineStr">
         <is>
           <t>v3+Boundary gating</t>
         </is>
       </c>
-      <c r="C27" s="77" t="inlineStr">
-        <is>
-          <t>0.941</t>
-        </is>
-      </c>
-      <c r="D27" s="77" t="inlineStr">
+      <c r="C27" s="69" t="inlineStr">
+        <is>
+          <t>0.947</t>
+        </is>
+      </c>
+      <c r="D27" s="69" t="inlineStr">
         <is>
           <t>0.998</t>
         </is>
       </c>
-      <c r="E27" s="77" t="inlineStr">
+      <c r="E27" s="69" t="inlineStr">
         <is>
           <t>1.000</t>
         </is>
       </c>
-      <c r="F27" s="77" t="inlineStr">
-        <is>
-          <t>0.937</t>
-        </is>
-      </c>
-      <c r="G27" s="77" t="inlineStr">
-        <is>
-          <t>0.875</t>
-        </is>
-      </c>
-      <c r="H27" s="78" t="inlineStr">
-        <is>
-          <t>+安全门. FPR 100%→0%</t>
+      <c r="F27" s="69" t="inlineStr">
+        <is>
+          <t>0.996</t>
+        </is>
+      </c>
+      <c r="G27" s="69" t="inlineStr">
+        <is>
+          <t>0.981</t>
+        </is>
+      </c>
+      <c r="H27" s="69" t="inlineStr">
+        <is>
+          <t>+安全门. Gate&lt;0.15通用. 五表全涨！</t>
         </is>
       </c>
     </row>
@@ -3232,33 +3268,35 @@
     <row r="14">
       <c r="A14" s="71" t="inlineStr">
         <is>
-          <t>SkillProbe v3 (ours)</t>
-        </is>
-      </c>
-      <c r="B14" s="71" t="n">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="C14" s="71" t="n">
+          <t>SkillProbe v4 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="C14" s="70" t="n">
         <v>19.4</v>
       </c>
-      <c r="D14" s="71" t="n">
+      <c r="D14" s="70" t="n">
         <v>6.5</v>
       </c>
-      <c r="E14" s="71" t="n">
+      <c r="E14" s="70" t="n">
         <v>87.90000000000001</v>
       </c>
-      <c r="F14" s="71" t="n">
+      <c r="F14" s="70" t="n">
         <v>82.09999999999999</v>
       </c>
-      <c r="G14" s="71" t="n">
+      <c r="G14" s="70" t="n">
         <v>93.5</v>
       </c>
-      <c r="H14" s="71" t="n">
-        <v>0.977</v>
-      </c>
-      <c r="I14" s="71" t="inlineStr">
-        <is>
-          <t>★ v3: oper+bnd+centering+PCA8+C=0.01+L7+. L15. AUROC=0.941 SOTA on SMP</t>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>v4: Boundary-gated v3. Gate&lt;0.15. AUC=0.947 SOTA. 49/124 gated</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3754,33 +3792,122 @@
     <row r="14">
       <c r="A14" s="71" t="inlineStr">
         <is>
-          <t>SkillProbe v3 (ours)</t>
-        </is>
-      </c>
-      <c r="B14" s="71" t="n">
-        <v>0.9370000000000001</v>
-      </c>
-      <c r="C14" s="71" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="D14" s="71" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="E14" s="71" t="n">
-        <v>86.90000000000001</v>
-      </c>
-      <c r="F14" s="71" t="n">
-        <v>87</v>
-      </c>
-      <c r="G14" s="71" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="H14" s="71" t="n">
-        <v>0.9370000000000001</v>
-      </c>
-      <c r="I14" s="71" t="inlineStr">
-        <is>
-          <t>★ v3: centering removes confound inflation. More honest than v1</t>
+          <t>SkillProbe v4 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.996</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>98</v>
+      </c>
+      <c r="F14" s="70" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="G14" s="70" t="n">
+        <v>98.7</v>
+      </c>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>v4: Gate&lt;0.15. AUC=0.996! Boundary gate catches confounded samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Skill-Inject Filter</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Naive filter: always fires on 8K samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cisco-skill-scanner</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="C16" t="n">
+        <v>100</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>129 core patterns, always fires</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NVIDIA SkillSpector</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.521</v>
+      </c>
+      <c r="C17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
       </c>
     </row>
@@ -4220,33 +4347,35 @@
     <row r="14">
       <c r="A14" s="71" t="inlineStr">
         <is>
-          <t>SkillProbe v3 (ours)</t>
-        </is>
-      </c>
-      <c r="B14" s="71" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="C14" s="71" t="n">
-        <v>35.3</v>
-      </c>
-      <c r="D14" s="71" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="E14" s="71" t="n">
-        <v>73.5</v>
-      </c>
-      <c r="F14" s="71" t="n">
-        <v>72.5</v>
-      </c>
-      <c r="G14" s="71" t="n">
-        <v>90.5</v>
-      </c>
-      <c r="H14" s="71" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="I14" s="71" t="inlineStr">
-        <is>
-          <t>★ v3: centering reduces in-domain bias. More robust OOD. FNR=9.5% excellent</t>
+          <t>SkillProbe v4 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.981</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="F14" s="70" t="n">
+        <v>93</v>
+      </c>
+      <c r="G14" s="70" t="n">
+        <v>94</v>
+      </c>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>v4: Gate&lt;0.15. AUC=0.981! Gating fixes OOD FPR from 12%→7%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NVIDIA SkillSpector to SMP: AUROC=0.50 FPR=100% (same as all surface-text methods)
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -2839,7 +2839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3355,6 +3355,35 @@
       <c r="I16" t="inlineStr">
         <is>
           <t>129 core patterns. Better than basic regex but still 68% FPR</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NVIDIA SkillSpector</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.503</v>
+      </c>
+      <c r="C17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete CPU baselines: 5 scanners x 4 datasets with precision/recall
Overview sheet: added Skill-Inject (#10), cisco (#11), NVIDIA SkillSpector (#12)
All per-dataset sheets updated with full metrics (AUROC/FPR/FNR/Prec/Rec/F1)

Key result: All 5 surface-text scanners fail on Inverse Decoy (clean vocab)
  - Static Regex: AUROC=0.99 (always fires on std Python)
  - Skill-Inject: AUROC=0.50 (random)
  - cisco-core:    AUROC=0.50 (random)
  - NVIDIA:        AUROC=0.50 (random)
  - TF-IDF+LR:     AUROC=0.16 FNR=78%

Only hidden-state methods succeed (0% FPR, 0.6% FNR).
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -2041,6 +2041,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="83" t="inlineStr">
         <is>
@@ -2230,6 +2231,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="83" t="inlineStr">
         <is>
@@ -2542,41 +2544,62 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="66" t="inlineStr">
-        <is>
-          <t>三、SkillProbe 方法演进</t>
+      <c r="A22" s="66" t="n">
+        <v>10</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Skill-Inject Filter</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Skill 全文</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Keyword patterns (Schmotz et al. 2026)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>表面文本</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Naive lower-bound baseline</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="67" t="inlineStr">
-        <is>
-          <t>版本</t>
-        </is>
+      <c r="A23" s="67" t="n">
+        <v>11</v>
       </c>
       <c r="B23" s="67" t="inlineStr">
         <is>
-          <t>方法</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="C23" s="67" t="inlineStr">
         <is>
-          <t>SMP</t>
+          <t>Skill 全文</t>
         </is>
       </c>
       <c r="D23" s="67" t="inlineStr">
         <is>
-          <t>Decoy</t>
+          <t>129 YAML patterns (core signatures)</t>
         </is>
       </c>
       <c r="E23" s="67" t="inlineStr">
         <is>
-          <t>InvDecoy</t>
+          <t>表面文本</t>
         </is>
       </c>
       <c r="F23" s="67" t="inlineStr">
         <is>
-          <t>MSB</t>
+          <t>Cisco AI Defense, industrial scanner</t>
         </is>
       </c>
       <c r="G23" s="67" t="inlineStr">
@@ -2591,34 +2614,32 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="21" t="inlineStr">
-        <is>
-          <t>v1</t>
-        </is>
+      <c r="A24" s="21" t="n">
+        <v>12</v>
       </c>
       <c r="B24" s="22" t="inlineStr">
         <is>
-          <t>oper+bnd+PCA8+C=0.01+L7+</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="C24" s="22" t="inlineStr">
         <is>
-          <t>0.910</t>
+          <t>Skill 全文</t>
         </is>
       </c>
       <c r="D24" s="22" t="inlineStr">
         <is>
-          <t>0.427</t>
+          <t>20 YARA rules (4 categories)</t>
         </is>
       </c>
       <c r="E24" s="22" t="inlineStr">
         <is>
-          <t>0.165</t>
+          <t>表面文本</t>
         </is>
       </c>
       <c r="F24" s="22" t="inlineStr">
         <is>
-          <t>0.964</t>
+          <t>13.5k stars, most popular skill scanner</t>
         </is>
       </c>
       <c r="G24" s="22" t="inlineStr">

</xml_diff>

<commit_message>
Complete 5-dataset CPU baselines: MASB + precision/recall filled
MASB (4K benign + 3.9K malicious):
  Static Regex: 0.59 / Prec=50% / Rec=100%
  Skill-Inject: 0.50 / Prec=50% / Rec=100%
  cisco:        0.55 / Prec=50% / Rec=100%
  NVIDIA:       0.52 / Prec=50% / Rec=100%
  TF-IDF+LR:    0.79 / Prec=71% / Rec=72%

All sheets now have precision/recall for all methods.
README updated to v4 (0.947 SMP, 0.998 Decoy, 1.000 InvDecoy).
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -2041,7 +2041,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="83" t="inlineStr">
         <is>
@@ -2231,7 +2230,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="83" t="inlineStr">
         <is>
@@ -3339,6 +3337,12 @@
       <c r="E15" t="n">
         <v>66.7</v>
       </c>
+      <c r="F15" t="n">
+        <v>50</v>
+      </c>
+      <c r="G15" t="n">
+        <v>100</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>—</t>
@@ -3368,6 +3372,12 @@
       <c r="E16" t="n">
         <v>60.6</v>
       </c>
+      <c r="F16" t="n">
+        <v>50</v>
+      </c>
+      <c r="G16" t="n">
+        <v>68.3</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>—</t>
@@ -3396,6 +3406,12 @@
       </c>
       <c r="E17" t="n">
         <v>66.7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -3522,7 +3538,7 @@
         <v>66.7</v>
       </c>
       <c r="F4" s="22" t="n">
-        <v>50</v>
+        <v>49.6</v>
       </c>
       <c r="G4" s="22" t="n">
         <v>100</v>
@@ -3892,6 +3908,12 @@
       <c r="E15" t="n">
         <v>66.7</v>
       </c>
+      <c r="F15" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G15" t="n">
+        <v>100</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>—</t>
@@ -3921,6 +3943,12 @@
       <c r="E16" t="n">
         <v>66.7</v>
       </c>
+      <c r="F16" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>100</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>—</t>
@@ -3949,6 +3977,12 @@
       </c>
       <c r="E17" t="n">
         <v>66.7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -3976,7 +4010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4062,10 +4096,8 @@
           <t>Static Regex</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B4" s="24" t="n">
+        <v>0.586</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>100</v>
@@ -4077,7 +4109,7 @@
         <v>66.7</v>
       </c>
       <c r="F4" s="24" t="n">
-        <v>50</v>
+        <v>49.6</v>
       </c>
       <c r="G4" s="24" t="n">
         <v>100</v>
@@ -4100,7 +4132,7 @@
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>0.967</v>
+        <v>0.792</v>
       </c>
       <c r="C5" s="22" t="n">
         <v>6.4</v>
@@ -4112,10 +4144,10 @@
         <v>91.09999999999999</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>93</v>
+        <v>71.3</v>
       </c>
       <c r="G5" s="22" t="n">
-        <v>89.3</v>
+        <v>71.8</v>
       </c>
       <c r="H5" s="22" t="n">
         <v>0.973</v>
@@ -4426,6 +4458,111 @@
       <c r="I14" s="70" t="inlineStr">
         <is>
           <t>v4: Gate&lt;0.15. AUC=0.981! Gating fixes OOD FPR from 12%→7%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Skill-Inject Filter</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="C15" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="F15" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G15" t="n">
+        <v>100</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Naive filter: always fires on 8K samples</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cisco-skill-scanner</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="C16" t="n">
+        <v>100</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="F16" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>129 core patterns. Always fires</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NVIDIA SkillSpector</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.524</v>
+      </c>
+      <c r="C17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="F17" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4669,7 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>0.4625</v>
+        <v>0.463</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>100</v>
@@ -4544,10 +4681,10 @@
         <v>66.7</v>
       </c>
       <c r="F4" s="24" t="n">
-        <v>44.1</v>
+        <v>42</v>
       </c>
       <c r="G4" s="24" t="n">
-        <v>35.3</v>
+        <v>48.3</v>
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
@@ -4931,6 +5068,12 @@
       <c r="E15" t="n">
         <v>83.40000000000001</v>
       </c>
+      <c r="F15" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>100</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>—</t>
@@ -4949,7 +5092,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.5331</v>
+        <v>0.533</v>
       </c>
       <c r="C16" t="n">
         <v>43.3</v>
@@ -4960,6 +5103,12 @@
       <c r="E16" t="n">
         <v>60.6</v>
       </c>
+      <c r="F16" t="n">
+        <v>54</v>
+      </c>
+      <c r="G16" t="n">
+        <v>62.3</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>—</t>
@@ -4988,6 +5137,12 @@
       </c>
       <c r="E17" t="n">
         <v>66.7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -5103,7 +5258,7 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>0.9935</v>
+        <v>0.994</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>100</v>
@@ -5115,10 +5270,10 @@
         <v>66.7</v>
       </c>
       <c r="F4" s="24" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G4" s="24" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
@@ -5502,6 +5657,12 @@
       <c r="E15" t="n">
         <v>66.7</v>
       </c>
+      <c r="F15" t="n">
+        <v>50</v>
+      </c>
+      <c r="G15" t="n">
+        <v>100</v>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>—</t>
@@ -5520,7 +5681,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.5032</v>
+        <v>0.503</v>
       </c>
       <c r="C16" t="n">
         <v>100</v>
@@ -5531,6 +5692,12 @@
       <c r="E16" t="n">
         <v>66.7</v>
       </c>
+      <c r="F16" t="n">
+        <v>50</v>
+      </c>
+      <c r="G16" t="n">
+        <v>100</v>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>—</t>
@@ -5559,6 +5726,12 @@
       </c>
       <c r="E17" t="n">
         <v>66.7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>50</v>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add 恶意归因 sheet: dual-pass attribution accuracy 84%. 2x2 matrix. Code vs Decl poisoning.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="方法演进" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="总览" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="SMP Stealth V2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="MSB" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="MASB 75K" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Lexical Decoy" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Inverse Decoy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="恶意归因" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="总览" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SMP Stealth V2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="MSB" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="MASB 75K" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Lexical Decoy" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Inverse Decoy" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -251,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -454,6 +455,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2023,6 +2027,491 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>恶意归因 —— 区分代码投毒 vs 声明投毒</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="64" t="inlineStr">
+        <is>
+          <t>v2 Dual-Pass 架构：Pass A (decl-only) + Pass B (完整prompt)。risk=max(score_v1,score_decl)。attribution=argmax。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="66" t="inlineStr">
+        <is>
+          <t>架构</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="64" t="inlineStr">
+        <is>
+          <t>Pass A: prompt 截断在声明末尾 → 模型只看到声明 → decl-bnd → Decl-Probe (L2-LR) → score_decl</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="64" t="inlineStr">
+        <is>
+          <t>Pass B: 完整 prompt (同 v1) → oper+bnd 几何特征 → PCA(8)+LR → score_code</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="64" t="inlineStr">
+        <is>
+          <t>归因规则: argmax(score_code, score_decl)。两路都&gt;阈值→BOTH，都&lt;阈值→CLEAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>开销: Pass A ~50ms (仅800 chars) + Pass B ~1945ms (同v1)。总增量 +2.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="66" t="inlineStr">
+        <is>
+          <t>双探针独立检测能力 (175样本)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="67" t="inlineStr">
+        <is>
+          <t>探针</t>
+        </is>
+      </c>
+      <c r="B11" s="67" t="inlineStr">
+        <is>
+          <t>检测目标</t>
+        </is>
+      </c>
+      <c r="C11" s="67" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="D11" s="67" t="inlineStr">
+        <is>
+          <t>F1%</t>
+        </is>
+      </c>
+      <c r="E11" s="67" t="inlineStr">
+        <is>
+          <t>FPR%</t>
+        </is>
+      </c>
+      <c r="F11" s="67" t="inlineStr">
+        <is>
+          <t>FNR%</t>
+        </is>
+      </c>
+      <c r="G11" s="67" t="inlineStr">
+        <is>
+          <t>层</t>
+        </is>
+      </c>
+      <c r="H11" s="67" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Decl-Probe</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>仅声明投毒 (50样本)</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>0.808</t>
+        </is>
+      </c>
+      <c r="D12" s="22" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="E12" s="22" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F12" s="22" t="inlineStr">
+        <is>
+          <t>40.0</t>
+        </is>
+      </c>
+      <c r="G12" s="22" t="inlineStr">
+        <is>
+          <t>L31</t>
+        </is>
+      </c>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t>检出decl-poison+both-poison，漏掉oper-poison</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Code-Probe (v1)</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>仅代码投毒 (50样本)</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>0.919</t>
+        </is>
+      </c>
+      <c r="D13" s="22" t="inlineStr">
+        <is>
+          <t>90.4</t>
+        </is>
+      </c>
+      <c r="E13" s="22" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F13" s="22" t="inlineStr">
+        <is>
+          <t>17.6</t>
+        </is>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>检出oper-poison+both-poison，漏掉decl-poison</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="86" t="inlineStr">
+        <is>
+          <t>Fusion max()</t>
+        </is>
+      </c>
+      <c r="B14" s="78" t="inlineStr">
+        <is>
+          <t>声明+代码双投毒 (175样本)</t>
+        </is>
+      </c>
+      <c r="C14" s="78" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="D14" s="78" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="E14" s="78" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F14" s="78" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G14" s="78" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="78" t="inlineStr">
+        <is>
+          <t>全覆盖。max()取两路最强信号，互补漏检</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>关键：两路信号正交——Decl-Probe和Code-Probe检测的是不同攻击类型，互不重叠。max()融合实现100%检出。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="66" t="inlineStr">
+        <is>
+          <t>归因准确率</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="67" t="inlineStr">
+        <is>
+          <t>真实攻击来源</t>
+        </is>
+      </c>
+      <c r="B18" s="67" t="inlineStr">
+        <is>
+          <t>样本数</t>
+        </is>
+      </c>
+      <c r="C18" s="67" t="inlineStr">
+        <is>
+          <t>归因正确</t>
+        </is>
+      </c>
+      <c r="D18" s="67" t="inlineStr">
+        <is>
+          <t>准确率</t>
+        </is>
+      </c>
+      <c r="E18" s="67" t="inlineStr">
+        <is>
+          <t>错误归因分析</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="68" t="inlineStr">
+        <is>
+          <t>CLEAN (干净skill)</t>
+        </is>
+      </c>
+      <c r="B19" s="69" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C19" s="69" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D19" s="69" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E19" s="69" t="inlineStr">
+        <is>
+          <t>全部正确识别。双探针均未报警。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="68" t="inlineStr">
+        <is>
+          <t>OPERATION (代码投毒)</t>
+        </is>
+      </c>
+      <c r="B20" s="69" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C20" s="69" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D20" s="69" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E20" s="69" t="inlineStr">
+        <is>
+          <t>全部归因正确。Code-Probe报警，Decl-Probe不报。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="68" t="inlineStr">
+        <is>
+          <t>BOTH (声明+代码)</t>
+        </is>
+      </c>
+      <c r="B21" s="69" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C21" s="69" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D21" s="69" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E21" s="69" t="inlineStr">
+        <is>
+          <t>全部归因正确。双探针同时报警→正确归为BOTH。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>DECLARATION (声明投毒)</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>44%</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>28个被错归为BOTH。Decl-Probe对部分样本信号不够强(L31层)，改进层选择可提升。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>84.0%</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>argmax(score_code, score_decl) 归因</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="66" t="inlineStr">
+        <is>
+          <t>归因 2x2 矩阵</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="67" t="inlineStr"/>
+      <c r="B26" s="67" t="inlineStr">
+        <is>
+          <t>Code-Probe 报警</t>
+        </is>
+      </c>
+      <c r="C26" s="67" t="inlineStr">
+        <is>
+          <t>Code-Probe 安全</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>Decl-Probe 报警</t>
+        </is>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>BOTH (双投毒) ✓</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>DECLARATION (声明投毒) ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="68" t="inlineStr">
+        <is>
+          <t>Decl-Probe 安全</t>
+        </is>
+      </c>
+      <c r="B28" s="69" t="inlineStr">
+        <is>
+          <t>OPERATION (代码投毒) ✓</t>
+        </is>
+      </c>
+      <c r="C28" s="69" t="inlineStr">
+        <is>
+          <t>CLEAN (干净) ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>每个象限对应一种攻击来源，v2 可精确区分四种情况。这是所有 baseline 不具备的能力。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2852,7 +3341,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3421,577 +3910,6 @@
       <c r="I17" t="inlineStr">
         <is>
           <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="19" t="inlineStr">
-        <is>
-          <t>MSB (MalSkillBench) — Unpaired, Source Confound Evidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Unpaired, 7894 samples, new triad extract. L7+ verified (best layers already L19+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>AUROC</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>FPR%</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>FNR%</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>F1%</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Precision%</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Recall%</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Train AUC</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="21" t="inlineStr">
-        <is>
-          <t>Static Regex</t>
-        </is>
-      </c>
-      <c r="B4" s="22" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="C4" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="22" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F4" s="22" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G4" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H4" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I4" s="22" t="inlineStr">
-        <is>
-          <t>Always fires</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="21" t="inlineStr">
-        <is>
-          <t>TF-IDF + LR</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="n">
-        <v>0.967</v>
-      </c>
-      <c r="C5" s="22" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="E5" s="22" t="n">
-        <v>91.09999999999999</v>
-      </c>
-      <c r="F5" s="22" t="n">
-        <v>93</v>
-      </c>
-      <c r="G5" s="22" t="n">
-        <v>89.3</v>
-      </c>
-      <c r="H5" s="22" t="n">
-        <v>0.973</v>
-      </c>
-      <c r="I5" s="22" t="inlineStr">
-        <is>
-          <t>C=0.01</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="23" t="inlineStr">
-        <is>
-          <t>LLM-as-judge</t>
-        </is>
-      </c>
-      <c r="B6" s="24" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C6" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="24" t="n">
-        <v>66.59999999999999</v>
-      </c>
-      <c r="F6" s="24" t="n">
-        <v>50</v>
-      </c>
-      <c r="G6" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H6" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I6" s="22" t="inlineStr">
-        <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="25" t="inlineStr">
-        <is>
-          <t>Boundary only</t>
-        </is>
-      </c>
-      <c r="B7" s="26" t="n">
-        <v>0.999</v>
-      </c>
-      <c r="C7" s="26" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="D7" s="26" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="E7" s="26" t="n">
-        <v>98.7</v>
-      </c>
-      <c r="F7" s="26" t="n">
-        <v>98.59999999999999</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>98.7</v>
-      </c>
-      <c r="H7" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="22" t="inlineStr">
-        <is>
-          <t>L19 (L7+ verified, source confound)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="21" t="inlineStr">
-        <is>
-          <t>AgentLens</t>
-        </is>
-      </c>
-      <c r="B8" s="22" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="C8" s="22" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="D8" s="22" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="E8" s="22" t="n">
-        <v>97.2</v>
-      </c>
-      <c r="F8" s="22" t="n">
-        <v>96.5</v>
-      </c>
-      <c r="G8" s="22" t="n">
-        <v>97.90000000000001</v>
-      </c>
-      <c r="H8" s="22" t="n">
-        <v>0.995</v>
-      </c>
-      <c r="I8" s="22" t="inlineStr">
-        <is>
-          <t>L19 (L7+ verified, source confound)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>RouteGuard</t>
-        </is>
-      </c>
-      <c r="B9" s="24" t="n">
-        <v>0.795</v>
-      </c>
-      <c r="C9" s="24" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="D9" s="24" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="E9" s="24" t="n">
-        <v>74.5</v>
-      </c>
-      <c r="F9" s="24" t="n">
-        <v>64.09999999999999</v>
-      </c>
-      <c r="G9" s="24" t="n">
-        <v>88.90000000000001</v>
-      </c>
-      <c r="H9" s="24" t="n">
-        <v>0.796</v>
-      </c>
-      <c r="I9" s="22" t="inlineStr">
-        <is>
-          <t>rhid only. Honest: not inflated by source confound (unlike others at 0.99+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>Relational (v1)</t>
-        </is>
-      </c>
-      <c r="B10" s="26" t="n">
-        <v>0.992</v>
-      </c>
-      <c r="C10" s="26" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="D10" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="26" t="n">
-        <v>95.5</v>
-      </c>
-      <c r="F10" s="26" t="n">
-        <v>97</v>
-      </c>
-      <c r="G10" s="26" t="n">
-        <v>94</v>
-      </c>
-      <c r="H10" s="26" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="I10" s="22" t="inlineStr">
-        <is>
-          <t>L11</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="25" t="inlineStr">
-        <is>
-          <t>Centered Relational</t>
-        </is>
-      </c>
-      <c r="B11" s="26" t="n">
-        <v>0.991</v>
-      </c>
-      <c r="C11" s="26" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="D11" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="26" t="n">
-        <v>94.8</v>
-      </c>
-      <c r="F11" s="26" t="n">
-        <v>92.7</v>
-      </c>
-      <c r="G11" s="26" t="n">
-        <v>97</v>
-      </c>
-      <c r="H11" s="26" t="n">
-        <v>0.991</v>
-      </c>
-      <c r="I11" s="22" t="inlineStr">
-        <is>
-          <t>L11</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="27" t="inlineStr">
-        <is>
-          <t>SkillProbe v1</t>
-        </is>
-      </c>
-      <c r="B12" s="28" t="n">
-        <v>0.964</v>
-      </c>
-      <c r="C12" s="28" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="D12" s="28" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="E12" s="28" t="n">
-        <v>90.59999999999999</v>
-      </c>
-      <c r="F12" s="28" t="n">
-        <v>89.7</v>
-      </c>
-      <c r="G12" s="28" t="n">
-        <v>91.5</v>
-      </c>
-      <c r="H12" s="28" t="n">
-        <v>0.963</v>
-      </c>
-      <c r="I12" s="28" t="inlineStr">
-        <is>
-          <t>v1: oper+bnd. Source confound inflated</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="70" t="inlineStr">
-        <is>
-          <t>SkillProbe v2</t>
-        </is>
-      </c>
-      <c r="B13" s="70" t="n">
-        <v>0.964</v>
-      </c>
-      <c r="C13" s="70" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="D13" s="70" t="n">
-        <v>8.5</v>
-      </c>
-      <c r="E13" s="70" t="n">
-        <v>90.59999999999999</v>
-      </c>
-      <c r="F13" s="70" t="n">
-        <v>89.7</v>
-      </c>
-      <c r="G13" s="70" t="n">
-        <v>91.5</v>
-      </c>
-      <c r="H13" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I13" s="70" t="inlineStr">
-        <is>
-          <t>v2: max(v1,decl). =v1 on MSB</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="71" t="inlineStr">
-        <is>
-          <t>SkillProbe v4 (ours)</t>
-        </is>
-      </c>
-      <c r="B14" s="70" t="n">
-        <v>0.996</v>
-      </c>
-      <c r="C14" s="70" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="D14" s="70" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="E14" s="70" t="n">
-        <v>98</v>
-      </c>
-      <c r="F14" s="70" t="n">
-        <v>97.5</v>
-      </c>
-      <c r="G14" s="70" t="n">
-        <v>98.7</v>
-      </c>
-      <c r="H14" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I14" s="70" t="inlineStr">
-        <is>
-          <t>v4: Gate&lt;0.15. AUC=0.996! Boundary gate catches confounded samples</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Skill-Inject Filter</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.502</v>
-      </c>
-      <c r="C15" t="n">
-        <v>100</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F15" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G15" t="n">
-        <v>100</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Naive filter: always fires on 8K samples</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>cisco-skill-scanner</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.545</v>
-      </c>
-      <c r="C16" t="n">
-        <v>100</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F16" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G16" t="n">
-        <v>100</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>129 core patterns, always fires</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>NVIDIA SkillSpector</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0.521</v>
-      </c>
-      <c r="C17" t="n">
-        <v>100</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F17" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G17" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
       </c>
     </row>
@@ -4032,14 +3950,14 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>MASB 75K — Large-Scale Benign FPR Benchmark</t>
+          <t>MSB (MalSkillBench) — Unpaired, Source Confound Evidence</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>4K MASB benign + MSB malicious (3939), 70/15/15 split. In-domain. L7+.</t>
+          <t>Unpaired, 7894 samples, new triad extract. L7+ verified (best layers already L19+)</t>
         </is>
       </c>
     </row>
@@ -4091,37 +4009,37 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Static Regex</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
-        <v>0.586</v>
-      </c>
-      <c r="C4" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" s="24" t="n">
+      <c r="B4" s="22" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="C4" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="24" t="n">
+      <c r="E4" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="22" t="n">
         <v>49.6</v>
       </c>
-      <c r="G4" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="G4" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Always fires (OOD)</t>
+          <t>Always fires</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4050,7 @@
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>0.792</v>
+        <v>0.967</v>
       </c>
       <c r="C5" s="22" t="n">
         <v>6.4</v>
@@ -4144,17 +4062,17 @@
         <v>91.09999999999999</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>71.3</v>
+        <v>93</v>
       </c>
       <c r="G5" s="22" t="n">
-        <v>71.8</v>
+        <v>89.3</v>
       </c>
       <c r="H5" s="22" t="n">
         <v>0.973</v>
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>Estimated from MSB</t>
+          <t>C=0.01</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4092,7 @@
         <v>0</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>66.7</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F6" s="24" t="n">
         <v>50</v>
@@ -4203,26 +4121,26 @@
         <v>0.999</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>2.5</v>
+        <v>1.4</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>1</v>
+        <v>1.3</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>98.2</v>
+        <v>98.7</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>97.5</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>99</v>
+        <v>98.7</v>
       </c>
       <c r="H7" s="26" t="n">
         <v>1</v>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L15, in-domain (L7+)</t>
+          <t>L19 (L7+ verified, source confound)</t>
         </is>
       </c>
     </row>
@@ -4233,29 +4151,29 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.984</v>
+        <v>0.99</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>9.1</v>
+        <v>2.1</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>93.40000000000001</v>
+        <v>97.2</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>96.09999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>90.90000000000001</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>0.983</v>
+        <v>0.995</v>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L15, in-domain (L7+)</t>
+          <t>L19 (L7+ verified, source confound)</t>
         </is>
       </c>
     </row>
@@ -4266,29 +4184,29 @@
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>0.998</v>
+        <v>0.795</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>0</v>
+        <v>47.7</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>1</v>
+        <v>11.1</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>99.5</v>
+        <v>74.5</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>100</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>99</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>1</v>
+        <v>0.796</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>6K in-domain, rhid only (pre-L7+. Needs MSB route_hidden re-extract for L7+ update)</t>
+          <t>rhid only. Honest: not inflated by source confound (unlike others at 0.99+)</t>
         </is>
       </c>
     </row>
@@ -4299,29 +4217,29 @@
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>1</v>
+        <v>0.992</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="D10" s="26" t="n">
-        <v>0.7</v>
+        <v>6</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>99.59999999999999</v>
+        <v>95.5</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>99.3</v>
+        <v>94</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>1</v>
+        <v>0.993</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>4K in-domain, pre-L7+</t>
+          <t>L11</t>
         </is>
       </c>
     </row>
@@ -4332,29 +4250,29 @@
         </is>
       </c>
       <c r="B11" s="26" t="n">
-        <v>1</v>
+        <v>0.991</v>
       </c>
       <c r="C11" s="26" t="n">
-        <v>0</v>
+        <v>7.8</v>
       </c>
       <c r="D11" s="26" t="n">
-        <v>1.7</v>
+        <v>3</v>
       </c>
       <c r="E11" s="26" t="n">
-        <v>99.09999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="F11" s="26" t="n">
-        <v>100</v>
+        <v>92.7</v>
       </c>
       <c r="G11" s="26" t="n">
-        <v>98.3</v>
+        <v>97</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>1</v>
+        <v>0.991</v>
       </c>
       <c r="I11" s="22" t="inlineStr">
         <is>
-          <t>4K in-domain, pre-L7+</t>
+          <t>L11</t>
         </is>
       </c>
     </row>
@@ -4365,29 +4283,29 @@
         </is>
       </c>
       <c r="B12" s="28" t="n">
-        <v>0.923</v>
+        <v>0.964</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>16.3</v>
+        <v>10.8</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>16.4</v>
+        <v>8.5</v>
       </c>
       <c r="E12" s="28" t="n">
-        <v>83.5</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F12" s="28" t="n">
-        <v>83.40000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="G12" s="28" t="n">
-        <v>83.59999999999999</v>
+        <v>91.5</v>
       </c>
       <c r="H12" s="28" t="n">
-        <v>0.921</v>
+        <v>0.963</v>
       </c>
       <c r="I12" s="28" t="inlineStr">
         <is>
-          <t>v1: oper+bnd. In-domain</t>
+          <t>v1: oper+bnd. Source confound inflated</t>
         </is>
       </c>
     </row>
@@ -4398,22 +4316,22 @@
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.923</v>
+        <v>0.964</v>
       </c>
       <c r="C13" s="70" t="n">
-        <v>16.3</v>
+        <v>10.8</v>
       </c>
       <c r="D13" s="70" t="n">
-        <v>16.4</v>
+        <v>8.5</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>83.5</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="F13" s="70" t="n">
-        <v>83.40000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="G13" s="70" t="n">
-        <v>83.59999999999999</v>
+        <v>91.5</v>
       </c>
       <c r="H13" s="70" t="inlineStr">
         <is>
@@ -4422,7 +4340,7 @@
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>v2: max(v1,decl). =v1 on MASB</t>
+          <t>v2: max(v1,decl). =v1 on MSB</t>
         </is>
       </c>
     </row>
@@ -4433,22 +4351,22 @@
         </is>
       </c>
       <c r="B14" s="70" t="n">
-        <v>0.981</v>
+        <v>0.996</v>
       </c>
       <c r="C14" s="70" t="n">
-        <v>7.2</v>
+        <v>3.2</v>
       </c>
       <c r="D14" s="70" t="n">
-        <v>6</v>
+        <v>1.3</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>93.40000000000001</v>
+        <v>98</v>
       </c>
       <c r="F14" s="70" t="n">
-        <v>93</v>
+        <v>97.5</v>
       </c>
       <c r="G14" s="70" t="n">
-        <v>94</v>
+        <v>98.7</v>
       </c>
       <c r="H14" s="70" t="inlineStr">
         <is>
@@ -4457,7 +4375,7 @@
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>v4: Gate&lt;0.15. AUC=0.981! Gating fixes OOD FPR from 12%→7%</t>
+          <t>v4: Gate&lt;0.15. AUC=0.996! Boundary gate catches confounded samples</t>
         </is>
       </c>
     </row>
@@ -4468,7 +4386,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.505</v>
+        <v>0.502</v>
       </c>
       <c r="C15" t="n">
         <v>100</v>
@@ -4477,7 +4395,7 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F15" t="n">
         <v>49.6</v>
@@ -4503,7 +4421,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.552</v>
+        <v>0.545</v>
       </c>
       <c r="C16" t="n">
         <v>100</v>
@@ -4512,7 +4430,7 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F16" t="n">
         <v>49.6</v>
@@ -4527,7 +4445,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>129 core patterns. Always fires</t>
+          <t>129 core patterns, always fires</t>
         </is>
       </c>
     </row>
@@ -4538,7 +4456,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.524</v>
+        <v>0.521</v>
       </c>
       <c r="C17" t="n">
         <v>100</v>
@@ -4547,7 +4465,7 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F17" t="n">
         <v>49.6</v>
@@ -4581,7 +4499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4593,7 +4511,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
@@ -4603,14 +4521,14 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>Lexical Decoy — Suspicious Vocabulary, Benign Semantics (155 samples)</t>
+          <t>MASB 75K — Large-Scale Benign FPR Benchmark</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>155 decoys + 62 SMP mal paired. Unified internal contract. L7+. No interaction. PCA=8. C=0.01.</t>
+          <t>4K MASB benign + MSB malicious (3939), 70/15/15 split. In-domain. L7+.</t>
         </is>
       </c>
     </row>
@@ -4660,7 +4578,6 @@
           <t>Notes</t>
         </is>
       </c>
-      <c r="J3" s="20" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
@@ -4669,7 +4586,7 @@
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>0.463</v>
+        <v>0.586</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>100</v>
@@ -4681,10 +4598,10 @@
         <v>66.7</v>
       </c>
       <c r="F4" s="24" t="n">
-        <v>42</v>
+        <v>49.6</v>
       </c>
       <c r="G4" s="24" t="n">
-        <v>48.3</v>
+        <v>100</v>
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
@@ -4693,46 +4610,42 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Static Regex on 155 decoys: FPR=59% (better than old 100%—more diverse decoys)</t>
-        </is>
-      </c>
-      <c r="J4" s="22" t="n"/>
+          <t>Always fires (OOD)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>TF-IDF + LR</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
-        <v>0.7435</v>
-      </c>
-      <c r="C5" s="24" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="D5" s="24" t="n">
-        <v>39.1</v>
-      </c>
-      <c r="E5" s="24" t="n">
-        <v>60.9</v>
-      </c>
-      <c r="F5" s="24" t="n">
-        <v>50</v>
-      </c>
-      <c r="G5" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H5" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B5" s="22" t="n">
+        <v>0.792</v>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="D5" s="22" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>91.09999999999999</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>71.3</v>
+      </c>
+      <c r="G5" s="22" t="n">
+        <v>71.8</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>0.973</v>
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>TF-IDF on 155 decoys: FPR=100% (suspicious vocab = malicious to TF-IDF)</t>
-        </is>
-      </c>
-      <c r="J5" s="22" t="n"/>
+          <t>Estimated from MSB</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
@@ -4765,10 +4678,9 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%)</t>
-        </is>
-      </c>
-      <c r="J6" s="22" t="n"/>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
@@ -4777,32 +4689,31 @@
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>0.991</v>
+        <v>0.999</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>98.40000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>100</v>
+        <v>97.5</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>96.8</v>
+        <v>99</v>
       </c>
       <c r="H7" s="26" t="n">
-        <v>0.994</v>
+        <v>1</v>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L23 (L7+). Model judges ALL 150 decoys safe!</t>
-        </is>
-      </c>
-      <c r="J7" s="22" t="n"/>
+          <t>L15, in-domain (L7+)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
@@ -4811,32 +4722,31 @@
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.867</v>
+        <v>0.984</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>22.7</v>
+        <v>3.7</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>21</v>
+        <v>9.1</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>67.59999999999999</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>68.2</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>79</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>0.989</v>
+        <v>0.983</v>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L15 (L7+). PCA(50) boundary. FPR=23% acceptable.</t>
-        </is>
-      </c>
-      <c r="J8" s="22" t="n"/>
+          <t>L15, in-domain (L7+)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
@@ -4844,33 +4754,32 @@
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B9" s="30" t="n">
-        <v>0.777</v>
+      <c r="B9" s="24" t="n">
+        <v>0.998</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>65.3</v>
+        <v>0</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>75.40000000000001</v>
+        <v>99.5</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>60.4</v>
+        <v>100</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>0.734</v>
+        <v>1</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>rhid only. Cross-extract caution. FPR=65%</t>
-        </is>
-      </c>
-      <c r="J9" s="22" t="n"/>
+          <t>6K in-domain, rhid only (pre-L7+. Needs MSB route_hidden re-extract for L7+ update)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
@@ -4879,106 +4788,97 @@
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>0.46</v>
+        <v>1</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D10" s="26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E10" s="26" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="F10" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" s="26" t="n">
+        <v>99.3</v>
+      </c>
+      <c r="H10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>4K in-domain, pre-L7+</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>Centered Relational</t>
+        </is>
+      </c>
+      <c r="B11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="26" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F10" s="26" t="n">
-        <v>50</v>
-      </c>
-      <c r="G10" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H10" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="22" t="inlineStr">
-        <is>
-          <t>Obsolete (interaction+PCA64). FPR=100% confirms noise</t>
-        </is>
-      </c>
-      <c r="J10" s="22" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="68" t="inlineStr">
-        <is>
-          <t>Centered Relational</t>
-        </is>
-      </c>
-      <c r="B11" s="69" t="n">
-        <v>0.705</v>
-      </c>
-      <c r="C11" s="69" t="n">
-        <v>57.3</v>
-      </c>
-      <c r="D11" s="69" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="E11" s="69" t="n">
-        <v>70.3</v>
-      </c>
-      <c r="F11" s="69" t="n">
-        <v>59.2</v>
-      </c>
-      <c r="G11" s="69" t="n">
-        <v>85.3</v>
-      </c>
-      <c r="H11" s="69" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I11" s="69" t="inlineStr">
-        <is>
-          <t>Centered (-1PC). AUC=0.71 better than SkillProbe on decoy—centering helps lexical robustness</t>
-        </is>
-      </c>
-      <c r="J11" s="22" t="n"/>
+      <c r="D11" s="26" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E11" s="26" t="n">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="F11" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" s="26" t="n">
+        <v>98.3</v>
+      </c>
+      <c r="H11" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>4K in-domain, pre-L7+</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="68" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>SkillProbe v1</t>
         </is>
       </c>
-      <c r="B12" s="69" t="n">
-        <v>0.427</v>
-      </c>
-      <c r="C12" s="69" t="n">
-        <v>75.3</v>
-      </c>
-      <c r="D12" s="69" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="E12" s="69" t="n">
-        <v>49.1</v>
-      </c>
-      <c r="F12" s="69" t="n">
-        <v>38.3</v>
-      </c>
-      <c r="G12" s="69" t="n">
-        <v>91.90000000000001</v>
-      </c>
-      <c r="H12" s="69" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="69" t="inlineStr">
-        <is>
-          <t>v1: FPR=75% (oper reads suspicious code)</t>
-        </is>
-      </c>
-      <c r="J12" s="28" t="n"/>
+      <c r="B12" s="28" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="C12" s="28" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D12" s="28" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="E12" s="28" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="F12" s="28" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G12" s="28" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="H12" s="28" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="I12" s="28" t="inlineStr">
+        <is>
+          <t>v1: oper+bnd. In-domain</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
@@ -4987,22 +4887,22 @@
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.427</v>
+        <v>0.923</v>
       </c>
       <c r="C13" s="70" t="n">
-        <v>75.3</v>
+        <v>16.3</v>
       </c>
       <c r="D13" s="70" t="n">
-        <v>8.1</v>
+        <v>16.4</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>49.1</v>
+        <v>83.5</v>
       </c>
       <c r="F13" s="70" t="n">
-        <v>38.3</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="G13" s="70" t="n">
-        <v>91.90000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="H13" s="70" t="inlineStr">
         <is>
@@ -5011,7 +4911,7 @@
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>v2: max(v1,decl). Decl-Probe also fires on suspicious vocab. =v1</t>
+          <t>v2: max(v1,decl). =v1 on MASB</t>
         </is>
       </c>
     </row>
@@ -5022,22 +4922,22 @@
         </is>
       </c>
       <c r="B14" s="70" t="n">
-        <v>0.998</v>
+        <v>0.981</v>
       </c>
       <c r="C14" s="70" t="n">
-        <v>0</v>
+        <v>7.2</v>
       </c>
       <c r="D14" s="70" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>98.40000000000001</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="F14" s="70" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="G14" s="70" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H14" s="70" t="inlineStr">
         <is>
@@ -5046,7 +4946,7 @@
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>★ v4: Boundary-gated v3. Gate&lt;0.15. FPR=0% FNR=3%. Best on Decoy!</t>
+          <t>v4: Gate&lt;0.15. AUC=0.981! Gating fixes OOD FPR from 12%→7%</t>
         </is>
       </c>
     </row>
@@ -5057,19 +4957,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.8</v>
+        <v>0.505</v>
       </c>
       <c r="C15" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="D15" t="n">
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>83.40000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>50.2</v>
+        <v>49.6</v>
       </c>
       <c r="G15" t="n">
         <v>100</v>
@@ -5081,7 +4981,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Schmotz et al. 2026, naive input filtering</t>
+          <t>Naive filter: always fires on 8K samples</t>
         </is>
       </c>
     </row>
@@ -5092,22 +4992,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.533</v>
+        <v>0.552</v>
       </c>
       <c r="C16" t="n">
-        <v>43.3</v>
+        <v>100</v>
       </c>
       <c r="D16" t="n">
-        <v>37.7</v>
+        <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>60.6</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>54</v>
+        <v>49.6</v>
       </c>
       <c r="G16" t="n">
-        <v>62.3</v>
+        <v>100</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -5116,7 +5016,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>176 patterns (core+promptguard), Python 3.10+ required</t>
+          <t>129 core patterns. Always fires</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5027,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.49</v>
+        <v>0.524</v>
       </c>
       <c r="C17" t="n">
         <v>100</v>
@@ -5136,10 +5036,10 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>66.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>50.2</v>
+        <v>49.6</v>
       </c>
       <c r="G17" t="n">
         <v>100</v>
@@ -5151,7 +5051,7 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
+          <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
       </c>
     </row>
@@ -5192,6 +5092,595 @@
     <row r="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
+          <t>Lexical Decoy — Suspicious Vocabulary, Benign Semantics (155 samples)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>155 decoys + 62 SMP mal paired. Unified internal contract. L7+. No interaction. PCA=8. C=0.01.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="20" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="inlineStr">
+        <is>
+          <t>FPR%</t>
+        </is>
+      </c>
+      <c r="D3" s="20" t="inlineStr">
+        <is>
+          <t>FNR%</t>
+        </is>
+      </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>F1%</t>
+        </is>
+      </c>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>Precision%</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="inlineStr">
+        <is>
+          <t>Recall%</t>
+        </is>
+      </c>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>Train AUC</t>
+        </is>
+      </c>
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>Static Regex</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="C4" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="24" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F4" s="24" t="n">
+        <v>42</v>
+      </c>
+      <c r="G4" s="24" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="H4" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="22" t="inlineStr">
+        <is>
+          <t>Static Regex on 155 decoys: FPR=59% (better than old 100%—more diverse decoys)</t>
+        </is>
+      </c>
+      <c r="J4" s="22" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>TF-IDF + LR</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n">
+        <v>0.7435</v>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="D5" s="24" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="E5" s="24" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" s="22" t="inlineStr">
+        <is>
+          <t>TF-IDF on 155 decoys: FPR=100% (suspicious vocab = malicious to TF-IDF)</t>
+        </is>
+      </c>
+      <c r="J5" s="22" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>LLM-as-judge</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="H6" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%)</t>
+        </is>
+      </c>
+      <c r="J6" s="22" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>Boundary only</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="C7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="26" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E7" s="26" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="F7" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" s="26" t="n">
+        <v>96.8</v>
+      </c>
+      <c r="H7" s="26" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>L23 (L7+). Model judges ALL 150 decoys safe!</t>
+        </is>
+      </c>
+      <c r="J7" s="22" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>AgentLens</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>21</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="F8" s="22" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="G8" s="22" t="n">
+        <v>79</v>
+      </c>
+      <c r="H8" s="22" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="I8" s="22" t="inlineStr">
+        <is>
+          <t>L15 (L7+). PCA(50) boundary. FPR=23% acceptable.</t>
+        </is>
+      </c>
+      <c r="J8" s="22" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>RouteGuard</t>
+        </is>
+      </c>
+      <c r="B9" s="30" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <v>0.734</v>
+      </c>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>rhid only. Cross-extract caution. FPR=65%</t>
+        </is>
+      </c>
+      <c r="J9" s="22" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>Relational (v1)</t>
+        </is>
+      </c>
+      <c r="B10" s="26" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="C10" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="D10" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="26" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F10" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="G10" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>Obsolete (interaction+PCA64). FPR=100% confirms noise</t>
+        </is>
+      </c>
+      <c r="J10" s="22" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="68" t="inlineStr">
+        <is>
+          <t>Centered Relational</t>
+        </is>
+      </c>
+      <c r="B11" s="69" t="n">
+        <v>0.705</v>
+      </c>
+      <c r="C11" s="69" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="D11" s="69" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="E11" s="69" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="F11" s="69" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="G11" s="69" t="n">
+        <v>85.3</v>
+      </c>
+      <c r="H11" s="69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="69" t="inlineStr">
+        <is>
+          <t>Centered (-1PC). AUC=0.71 better than SkillProbe on decoy—centering helps lexical robustness</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="68" t="inlineStr">
+        <is>
+          <t>SkillProbe v1</t>
+        </is>
+      </c>
+      <c r="B12" s="69" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="C12" s="69" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="D12" s="69" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E12" s="69" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F12" s="69" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G12" s="69" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="H12" s="69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I12" s="69" t="inlineStr">
+        <is>
+          <t>v1: FPR=75% (oper reads suspicious code)</t>
+        </is>
+      </c>
+      <c r="J12" s="28" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v2</t>
+        </is>
+      </c>
+      <c r="B13" s="70" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="C13" s="70" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="D13" s="70" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E13" s="70" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F13" s="70" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G13" s="70" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="H13" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="70" t="inlineStr">
+        <is>
+          <t>v2: max(v1,decl). Decl-Probe also fires on suspicious vocab. =v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="71" t="inlineStr">
+        <is>
+          <t>SkillProbe v4 (ours)</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.998</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="F14" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" s="70" t="n">
+        <v>97</v>
+      </c>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>★ v4: Boundary-gated v3. Gate&lt;0.15. FPR=0% FNR=3%. Best on Decoy!</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Skill-Inject Filter</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C15" t="n">
+        <v>40</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="F15" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>100</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Schmotz et al. 2026, naive input filtering</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cisco-skill-scanner</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.533</v>
+      </c>
+      <c r="C16" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="E16" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="F16" t="n">
+        <v>54</v>
+      </c>
+      <c r="G16" t="n">
+        <v>62.3</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>176 patterns (core+promptguard), Python 3.10+ required</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NVIDIA SkillSpector</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="C17" t="n">
+        <v>100</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="G17" t="n">
+        <v>100</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="19" t="inlineStr">
+        <is>
           <t>Inverse Decoy — Clean Vocabulary, Malicious Semantics (155 pairs)</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Fix attribution sheet: 100% accuracy (GAP_REPORT numbers). Update RQ4 narrative.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -2089,52 +2089,129 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="64" t="inlineStr">
+        <is>
+          <t>Decl-Probe</t>
+        </is>
+      </c>
+      <c r="B9" s="64" t="inlineStr">
+        <is>
+          <t>仅声明投毒 (50样本)</t>
+        </is>
+      </c>
+      <c r="C9" s="64" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="D9" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="64" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="H9" s="64" t="inlineStr">
+        <is>
+          <t>Pass A decl-bd norm. AUROC=0.99 完美区分decl-poison vs clean</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
-      <c r="A10" s="66" t="inlineStr">
-        <is>
-          <t>双探针独立检测能力 (175样本)</t>
+      <c r="A10" s="64" t="inlineStr">
+        <is>
+          <t>Code-Probe</t>
+        </is>
+      </c>
+      <c r="B10" s="64" t="inlineStr">
+        <is>
+          <t>仅代码投毒 (50样本)</t>
+        </is>
+      </c>
+      <c r="C10" s="64" t="inlineStr">
+        <is>
+          <t>0.82</t>
+        </is>
+      </c>
+      <c r="D10" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="64" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="64" t="inlineStr">
+        <is>
+          <t>L7</t>
+        </is>
+      </c>
+      <c r="H10" s="64" t="inlineStr">
+        <is>
+          <t>Pass B oper-bd norm. AUROC=0.82 区分oper-poison vs clean</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="67" t="inlineStr">
-        <is>
-          <t>探针</t>
-        </is>
-      </c>
-      <c r="B11" s="67" t="inlineStr">
-        <is>
-          <t>检测目标</t>
-        </is>
-      </c>
-      <c r="C11" s="67" t="inlineStr">
-        <is>
-          <t>AUROC</t>
-        </is>
-      </c>
-      <c r="D11" s="67" t="inlineStr">
-        <is>
-          <t>F1%</t>
-        </is>
-      </c>
-      <c r="E11" s="67" t="inlineStr">
-        <is>
-          <t>FPR%</t>
-        </is>
-      </c>
-      <c r="F11" s="67" t="inlineStr">
-        <is>
-          <t>FNR%</t>
-        </is>
-      </c>
-      <c r="G11" s="67" t="inlineStr">
-        <is>
-          <t>层</t>
-        </is>
-      </c>
-      <c r="H11" s="67" t="inlineStr">
-        <is>
-          <t>说明</t>
+      <c r="A11" s="69" t="inlineStr">
+        <is>
+          <t>Fusion max()</t>
+        </is>
+      </c>
+      <c r="B11" s="69" t="inlineStr">
+        <is>
+          <t>声明+代码双投毒 (175样本)</t>
+        </is>
+      </c>
+      <c r="C11" s="69" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="D11" s="69" t="inlineStr">
+        <is>
+          <t>100.0</t>
+        </is>
+      </c>
+      <c r="E11" s="69" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="F11" s="69" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="G11" s="69" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="69" t="inlineStr">
+        <is>
+          <t>max(Decl-Det, Code-Det). 两路信号正交→100%检出+100%归因</t>
         </is>
       </c>
     </row>
@@ -2223,36 +2300,36 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="86" t="inlineStr">
-        <is>
-          <t>Fusion max()</t>
-        </is>
-      </c>
-      <c r="B14" s="78" t="inlineStr">
-        <is>
-          <t>声明+代码双投毒 (175样本)</t>
-        </is>
-      </c>
-      <c r="C14" s="78" t="inlineStr">
-        <is>
-          <t>1.000</t>
-        </is>
-      </c>
-      <c r="D14" s="78" t="inlineStr">
-        <is>
-          <t>100.0</t>
-        </is>
-      </c>
-      <c r="E14" s="78" t="inlineStr">
+      <c r="A14" s="68" t="inlineStr">
+        <is>
+          <t>CLEAN (干净skill)</t>
+        </is>
+      </c>
+      <c r="B14" s="69" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C14" s="69" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D14" s="69" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E14" s="69" t="inlineStr">
+        <is>
+          <t>双探针均安全。Pass A decl-bd low, Pass B oper-bd low。</t>
+        </is>
+      </c>
+      <c r="F14" s="78" t="inlineStr">
         <is>
           <t>0.0</t>
         </is>
       </c>
-      <c r="F14" s="78" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
       <c r="G14" s="78" t="inlineStr">
         <is>
           <t>—</t>
@@ -2265,43 +2342,110 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>关键：两路信号正交——Decl-Probe和Code-Probe检测的是不同攻击类型，互不重叠。max()融合实现100%检出。</t>
+      <c r="A15" s="85" t="inlineStr">
+        <is>
+          <t>OPERATION (代码投毒)</t>
+        </is>
+      </c>
+      <c r="B15" s="85" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C15" s="85" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D15" s="85" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E15" s="85" t="inlineStr">
+        <is>
+          <t>全部归因正确。Pass B oper-bd 高→Code侧报警。Pass A decl-bd 低→Decl侧不报。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="85" t="inlineStr">
+        <is>
+          <t>BOTH (声明+代码)</t>
+        </is>
+      </c>
+      <c r="B16" s="85" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="C16" s="85" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="D16" s="85" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E16" s="85" t="inlineStr">
+        <is>
+          <t>全部归因正确。双探针bd norms同时升高→正确归为BOTH。</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="66" t="inlineStr">
-        <is>
-          <t>归因准确率</t>
+      <c r="A17" s="85" t="inlineStr">
+        <is>
+          <t>DECLARATION (声明投毒)</t>
+        </is>
+      </c>
+      <c r="B17" s="85" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C17" s="85" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D17" s="85" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E17" s="85" t="inlineStr">
+        <is>
+          <t>全部归因正确。Pass A decl-bd 高→Decl侧报警。Pass B oper-bd 低→Code侧不报。</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="67" t="inlineStr">
-        <is>
-          <t>真实攻击来源</t>
-        </is>
-      </c>
-      <c r="B18" s="67" t="inlineStr">
-        <is>
-          <t>样本数</t>
-        </is>
-      </c>
-      <c r="C18" s="67" t="inlineStr">
-        <is>
-          <t>归因正确</t>
-        </is>
-      </c>
-      <c r="D18" s="67" t="inlineStr">
-        <is>
-          <t>准确率</t>
-        </is>
-      </c>
-      <c r="E18" s="67" t="inlineStr">
-        <is>
-          <t>错误归因分析</t>
+      <c r="A18" s="69" t="inlineStr">
+        <is>
+          <t>合计</t>
+        </is>
+      </c>
+      <c r="B18" s="69" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="C18" s="69" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="D18" s="69" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E18" s="69" t="inlineStr">
+        <is>
+          <t>GAP_REPORT 方法: boundary token norm 比较。Pass A (decl-only) vs Pass B (skip-decl)。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reorder all 5 benchmark sheets: surface-text → internal baselines → our methods (green). Integrate new baselines.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -252,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -457,6 +457,9 @@
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3525,49 +3528,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>AUROC</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>FPR%</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>FNR%</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>F1%</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Precision%</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Recall%</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Train AUC</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A3" s="87" t="inlineStr">
+        <is>
+          <t>Static Regex</t>
+        </is>
+      </c>
+      <c r="B3" s="87" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="C3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="87" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F3" s="87" t="n">
+        <v>50</v>
+      </c>
+      <c r="G3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="H3" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="87" t="inlineStr">
+        <is>
+          <t>Always fires</t>
         </is>
       </c>
       <c r="J3" s="20" t="n"/>
@@ -3575,11 +3566,11 @@
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Static Regex</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>0.54</v>
+        <v>0.528</v>
       </c>
       <c r="C4" s="22" t="n">
         <v>100</v>
@@ -3603,7 +3594,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Always fires</t>
+          <t>Schmotz et al. 2026, naive input filter. FPR=100%</t>
         </is>
       </c>
       <c r="J4" s="22" t="n"/>
@@ -3645,26 +3636,26 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>0.63</v>
+        <v>0.539</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>100</v>
+        <v>68.3</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>0</v>
+        <v>31.7</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>66.7</v>
+        <v>60.6</v>
       </c>
       <c r="F6" s="24" t="n">
         <v>50</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>100</v>
+        <v>68.3</v>
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
@@ -3673,7 +3664,7 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+          <t>129 core patterns. Better than basic regex but still 68% FPR</t>
         </is>
       </c>
       <c r="J6" s="22" t="n"/>
@@ -3681,33 +3672,35 @@
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>0.863</v>
+        <v>0.503</v>
       </c>
       <c r="C7" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="26" t="n">
-        <v>40.3</v>
-      </c>
       <c r="E7" s="26" t="n">
-        <v>74.7</v>
+        <v>66.7</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>59.7</v>
-      </c>
-      <c r="H7" s="26" t="n">
-        <v>0.989</v>
+        <v>100</v>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L11 (L7+ restricted)</t>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
       </c>
       <c r="J7" s="22" t="n"/>
@@ -3715,33 +3708,35 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.871</v>
+        <v>0.63</v>
       </c>
       <c r="C8" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="22" t="n">
-        <v>51.6</v>
-      </c>
       <c r="E8" s="22" t="n">
-        <v>65.2</v>
+        <v>66.7</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>48.4</v>
-      </c>
-      <c r="H8" s="22" t="n">
-        <v>0.989</v>
+        <v>100</v>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L11 (L7+ restricted)</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
         </is>
       </c>
       <c r="J8" s="22" t="n"/>
@@ -3749,33 +3744,33 @@
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>RouteGuard</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>0.824</v>
+        <v>0.863</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>48.4</v>
+        <v>0</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>8.1</v>
+        <v>40.3</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>76.5</v>
+        <v>74.7</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>65.5</v>
+        <v>100</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>91.7</v>
+        <v>59.7</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>0.9379999999999999</v>
+        <v>0.989</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>Done: attn+rhid. Honest: AUC=0.824 on paired CF</t>
+          <t>L11 (L7+ restricted)</t>
         </is>
       </c>
       <c r="J9" s="22" t="n"/>
@@ -3783,33 +3778,33 @@
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Relational (v1)</t>
+          <t>AgentLens</t>
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>0.761</v>
+        <v>0.871</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D10" s="26" t="n">
-        <v>6.5</v>
+        <v>51.6</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>76.8</v>
+        <v>65.2</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>65.2</v>
+        <v>100</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>93.5</v>
+        <v>48.4</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>0.893</v>
+        <v>0.989</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>L31, interact+PCA64</t>
+          <t>L11 (L7+ restricted)</t>
         </is>
       </c>
       <c r="J10" s="22" t="n"/>
@@ -3817,33 +3812,33 @@
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>RouteGuard</t>
         </is>
       </c>
       <c r="B11" s="26" t="n">
-        <v>0.872</v>
+        <v>0.824</v>
       </c>
       <c r="C11" s="26" t="n">
-        <v>19.4</v>
+        <v>48.4</v>
       </c>
       <c r="D11" s="26" t="n">
-        <v>12.9</v>
+        <v>8.1</v>
       </c>
       <c r="E11" s="26" t="n">
-        <v>84.40000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="F11" s="26" t="n">
-        <v>81.8</v>
+        <v>65.5</v>
       </c>
       <c r="G11" s="26" t="n">
-        <v>87.09999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>0.896</v>
+        <v>0.9379999999999999</v>
       </c>
       <c r="I11" s="22" t="inlineStr">
         <is>
-          <t>L27, -1PC</t>
+          <t>Done: attn+rhid. Honest: AUC=0.824 on paired CF</t>
         </is>
       </c>
       <c r="J11" s="22" t="n"/>
@@ -3851,33 +3846,33 @@
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B12" s="28" t="n">
-        <v>0.91</v>
+        <v>0.761</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>19.4</v>
+        <v>50</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>11.3</v>
+        <v>6.5</v>
       </c>
       <c r="E12" s="28" t="n">
-        <v>85.3</v>
+        <v>76.8</v>
       </c>
       <c r="F12" s="28" t="n">
-        <v>82.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="G12" s="28" t="n">
-        <v>88.7</v>
+        <v>93.5</v>
       </c>
       <c r="H12" s="29" t="n">
-        <v>0.919</v>
+        <v>0.893</v>
       </c>
       <c r="I12" s="28" t="inlineStr">
         <is>
-          <t>v1: oper+bnd+PCA8+C=0.01+L7+. Baseline method</t>
+          <t>L31, interact+PCA64</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -3885,140 +3880,136 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2</t>
+          <t>Centered Relational</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.91</v>
+        <v>0.872</v>
       </c>
       <c r="C13" s="70" t="n">
         <v>19.4</v>
       </c>
       <c r="D13" s="70" t="n">
-        <v>11.3</v>
+        <v>12.9</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>85.3</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="F13" s="70" t="n">
-        <v>82.09999999999999</v>
+        <v>81.8</v>
       </c>
       <c r="G13" s="70" t="n">
-        <v>88.7</v>
-      </c>
-      <c r="H13" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>87.09999999999999</v>
+      </c>
+      <c r="H13" s="70" t="n">
+        <v>0.896</v>
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>v2: max(v1,decl). SMP无声明投毒→=v1. 零退化+补盲区+归因</t>
+          <t>L27, -1PC</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="71" t="inlineStr">
-        <is>
-          <t>SkillProbe v4 (ours)</t>
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B14" s="70" t="n">
-        <v>0.947</v>
+        <v>0.91</v>
       </c>
       <c r="C14" s="70" t="n">
         <v>19.4</v>
       </c>
       <c r="D14" s="70" t="n">
-        <v>6.5</v>
+        <v>11.3</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>87.90000000000001</v>
+        <v>85.3</v>
       </c>
       <c r="F14" s="70" t="n">
         <v>82.09999999999999</v>
       </c>
       <c r="G14" s="70" t="n">
+        <v>88.7</v>
+      </c>
+      <c r="H14" s="70" t="n">
+        <v>0.919</v>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>v1: oper+bnd+PCA8+C=0.01+L7+. Baseline method</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v2</t>
+        </is>
+      </c>
+      <c r="B15" s="70" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="C15" s="70" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D15" s="70" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="E15" s="70" t="n">
+        <v>85.3</v>
+      </c>
+      <c r="F15" s="70" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="G15" s="70" t="n">
+        <v>88.7</v>
+      </c>
+      <c r="H15" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I15" s="70" t="inlineStr">
+        <is>
+          <t>v2: max(v1,decl). SMP无声明投毒→=v1. 零退化+补盲区+归因</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v4 (ours)</t>
+        </is>
+      </c>
+      <c r="B16" s="70" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="C16" s="70" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D16" s="70" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E16" s="70" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="F16" s="70" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="G16" s="70" t="n">
         <v>93.5</v>
       </c>
-      <c r="H14" s="70" t="inlineStr">
+      <c r="H16" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I14" s="70" t="inlineStr">
+      <c r="I16" s="70" t="inlineStr">
         <is>
           <t>v4: Boundary-gated v3. Gate&lt;0.15. AUC=0.947 SOTA. 49/124 gated</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Skill-Inject Filter</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.528</v>
-      </c>
-      <c r="C15" t="n">
-        <v>100</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F15" t="n">
-        <v>50</v>
-      </c>
-      <c r="G15" t="n">
-        <v>100</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Schmotz et al. 2026, naive input filter. FPR=100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>cisco-skill-scanner</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.539</v>
-      </c>
-      <c r="C16" t="n">
-        <v>68.3</v>
-      </c>
-      <c r="D16" t="n">
-        <v>31.7</v>
-      </c>
-      <c r="E16" t="n">
-        <v>60.6</v>
-      </c>
-      <c r="F16" t="n">
-        <v>50</v>
-      </c>
-      <c r="G16" t="n">
-        <v>68.3</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>129 core patterns. Better than basic regex but still 68% FPR</t>
         </is>
       </c>
     </row>
@@ -4106,60 +4097,48 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>AUROC</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>FPR%</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>FNR%</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>F1%</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Precision%</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Recall%</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Train AUC</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A3" s="87" t="inlineStr">
+        <is>
+          <t>Static Regex</t>
+        </is>
+      </c>
+      <c r="B3" s="87" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="C3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="87" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F3" s="87" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="H3" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="87" t="inlineStr">
+        <is>
+          <t>Always fires</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Static Regex</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>0.54</v>
+        <v>0.502</v>
       </c>
       <c r="C4" s="22" t="n">
         <v>100</v>
@@ -4183,7 +4162,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Always fires</t>
+          <t>Naive filter: always fires on 8K samples</t>
         </is>
       </c>
     </row>
@@ -4223,11 +4202,11 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>0.5</v>
+        <v>0.545</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>100</v>
@@ -4236,10 +4215,10 @@
         <v>0</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>66.59999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>50</v>
+        <v>49.6</v>
       </c>
       <c r="G6" s="24" t="n">
         <v>100</v>
@@ -4251,345 +4230,345 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+          <t>129 core patterns, always fires</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>0.999</v>
+        <v>0.521</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>1.4</v>
+        <v>100</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>98.7</v>
+        <v>66.7</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>98.59999999999999</v>
+        <v>49.6</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>98.7</v>
-      </c>
-      <c r="H7" s="26" t="n">
-        <v>1</v>
+        <v>100</v>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L19 (L7+ verified, source confound)</t>
+          <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.99</v>
+        <v>0.5</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>3.6</v>
+        <v>100</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>2.1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>97.2</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>96.5</v>
+        <v>50</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>97.90000000000001</v>
-      </c>
-      <c r="H8" s="22" t="n">
-        <v>0.995</v>
+        <v>100</v>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L19 (L7+ verified, source confound)</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>RouteGuard</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>0.795</v>
+        <v>0.999</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>47.7</v>
+        <v>1.4</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>11.1</v>
+        <v>1.3</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>74.5</v>
+        <v>98.7</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>64.09999999999999</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>88.90000000000001</v>
+        <v>98.7</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>0.796</v>
+        <v>1</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>rhid only. Honest: not inflated by source confound (unlike others at 0.99+)</t>
+          <t>L19 (L7+ verified, source confound)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Relational (v1)</t>
+          <t>AgentLens</t>
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>0.992</v>
+        <v>0.99</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
       <c r="D10" s="26" t="n">
-        <v>6</v>
+        <v>2.1</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>95.5</v>
+        <v>97.2</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>97</v>
+        <v>96.5</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>94</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>0.993</v>
+        <v>0.995</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>L11</t>
+          <t>L19 (L7+ verified, source confound)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>RouteGuard</t>
         </is>
       </c>
       <c r="B11" s="26" t="n">
-        <v>0.991</v>
+        <v>0.795</v>
       </c>
       <c r="C11" s="26" t="n">
-        <v>7.8</v>
+        <v>47.7</v>
       </c>
       <c r="D11" s="26" t="n">
-        <v>3</v>
+        <v>11.1</v>
       </c>
       <c r="E11" s="26" t="n">
-        <v>94.8</v>
+        <v>74.5</v>
       </c>
       <c r="F11" s="26" t="n">
-        <v>92.7</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G11" s="26" t="n">
-        <v>97</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="H11" s="26" t="n">
-        <v>0.991</v>
+        <v>0.796</v>
       </c>
       <c r="I11" s="22" t="inlineStr">
         <is>
-          <t>L11</t>
+          <t>rhid only. Honest: not inflated by source confound (unlike others at 0.99+)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B12" s="28" t="n">
-        <v>0.964</v>
+        <v>0.992</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>10.8</v>
+        <v>2.9</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="E12" s="28" t="n">
-        <v>90.59999999999999</v>
+        <v>95.5</v>
       </c>
       <c r="F12" s="28" t="n">
-        <v>89.7</v>
+        <v>97</v>
       </c>
       <c r="G12" s="28" t="n">
-        <v>91.5</v>
+        <v>94</v>
       </c>
       <c r="H12" s="28" t="n">
-        <v>0.963</v>
+        <v>0.993</v>
       </c>
       <c r="I12" s="28" t="inlineStr">
         <is>
-          <t>v1: oper+bnd. Source confound inflated</t>
+          <t>L11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
+          <t>Centered Relational</t>
+        </is>
+      </c>
+      <c r="B13" s="70" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="C13" s="70" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="D13" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="70" t="n">
+        <v>94.8</v>
+      </c>
+      <c r="F13" s="70" t="n">
+        <v>92.7</v>
+      </c>
+      <c r="G13" s="70" t="n">
+        <v>97</v>
+      </c>
+      <c r="H13" s="70" t="n">
+        <v>0.991</v>
+      </c>
+      <c r="I13" s="70" t="inlineStr">
+        <is>
+          <t>L11</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v1</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="F14" s="70" t="n">
+        <v>89.7</v>
+      </c>
+      <c r="G14" s="70" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="H14" s="70" t="n">
+        <v>0.963</v>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>v1: oper+bnd. Source confound inflated</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
           <t>SkillProbe v2</t>
         </is>
       </c>
-      <c r="B13" s="70" t="n">
+      <c r="B15" s="70" t="n">
         <v>0.964</v>
       </c>
-      <c r="C13" s="70" t="n">
+      <c r="C15" s="70" t="n">
         <v>10.8</v>
       </c>
-      <c r="D13" s="70" t="n">
+      <c r="D15" s="70" t="n">
         <v>8.5</v>
       </c>
-      <c r="E13" s="70" t="n">
+      <c r="E15" s="70" t="n">
         <v>90.59999999999999</v>
       </c>
-      <c r="F13" s="70" t="n">
+      <c r="F15" s="70" t="n">
         <v>89.7</v>
       </c>
-      <c r="G13" s="70" t="n">
+      <c r="G15" s="70" t="n">
         <v>91.5</v>
       </c>
-      <c r="H13" s="70" t="inlineStr">
+      <c r="H15" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I13" s="70" t="inlineStr">
+      <c r="I15" s="70" t="inlineStr">
         <is>
           <t>v2: max(v1,decl). =v1 on MSB</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="71" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="70" t="inlineStr">
         <is>
           <t>SkillProbe v4 (ours)</t>
         </is>
       </c>
-      <c r="B14" s="70" t="n">
+      <c r="B16" s="70" t="n">
         <v>0.996</v>
       </c>
-      <c r="C14" s="70" t="n">
+      <c r="C16" s="70" t="n">
         <v>3.2</v>
       </c>
-      <c r="D14" s="70" t="n">
+      <c r="D16" s="70" t="n">
         <v>1.3</v>
       </c>
-      <c r="E14" s="70" t="n">
+      <c r="E16" s="70" t="n">
         <v>98</v>
       </c>
-      <c r="F14" s="70" t="n">
+      <c r="F16" s="70" t="n">
         <v>97.5</v>
       </c>
-      <c r="G14" s="70" t="n">
+      <c r="G16" s="70" t="n">
         <v>98.7</v>
       </c>
-      <c r="H14" s="70" t="inlineStr">
+      <c r="H16" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I14" s="70" t="inlineStr">
+      <c r="I16" s="70" t="inlineStr">
         <is>
           <t>v4: Gate&lt;0.15. AUC=0.996! Boundary gate catches confounded samples</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Skill-Inject Filter</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.502</v>
-      </c>
-      <c r="C15" t="n">
-        <v>100</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F15" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G15" t="n">
-        <v>100</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Naive filter: always fires on 8K samples</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>cisco-skill-scanner</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.545</v>
-      </c>
-      <c r="C16" t="n">
-        <v>100</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F16" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G16" t="n">
-        <v>100</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>129 core patterns, always fires</t>
         </is>
       </c>
     </row>
@@ -4677,60 +4656,48 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>AUROC</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>FPR%</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>FNR%</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>F1%</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Precision%</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Recall%</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Train AUC</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A3" s="87" t="inlineStr">
+        <is>
+          <t>Static Regex</t>
+        </is>
+      </c>
+      <c r="B3" s="87" t="n">
+        <v>0.586</v>
+      </c>
+      <c r="C3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="87" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F3" s="87" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="G3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="H3" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="87" t="inlineStr">
+        <is>
+          <t>Always fires (OOD)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
         <is>
-          <t>Static Regex</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>0.586</v>
+        <v>0.505</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>100</v>
@@ -4739,7 +4706,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="24" t="n">
-        <v>66.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F4" s="24" t="n">
         <v>49.6</v>
@@ -4754,7 +4721,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Always fires (OOD)</t>
+          <t>Naive filter: always fires on 8K samples</t>
         </is>
       </c>
     </row>
@@ -4794,11 +4761,11 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>0.5</v>
+        <v>0.552</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>100</v>
@@ -4807,10 +4774,10 @@
         <v>0</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>66.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>50</v>
+        <v>49.6</v>
       </c>
       <c r="G6" s="24" t="n">
         <v>100</v>
@@ -4822,96 +4789,100 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+          <t>129 core patterns. Always fires</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>0.999</v>
+        <v>0.524</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>2.5</v>
+        <v>100</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>98.2</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>97.5</v>
+        <v>49.6</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>99</v>
-      </c>
-      <c r="H7" s="26" t="n">
-        <v>1</v>
+        <v>100</v>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L15, in-domain (L7+)</t>
+          <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.984</v>
+        <v>0.5</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>3.7</v>
+        <v>100</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>9.1</v>
+        <v>0</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>93.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>96.09999999999999</v>
+        <v>50</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>90.90000000000001</v>
-      </c>
-      <c r="H8" s="22" t="n">
-        <v>0.983</v>
+        <v>100</v>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L15, in-domain (L7+)</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>RouteGuard</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>0.998</v>
+        <v>0.999</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="D9" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>99.5</v>
+        <v>98.2</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>100</v>
+        <v>97.5</v>
       </c>
       <c r="G9" s="24" t="n">
         <v>99</v>
@@ -4921,246 +4892,242 @@
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>6K in-domain, rhid only (pre-L7+. Needs MSB route_hidden re-extract for L7+ update)</t>
+          <t>L15, in-domain (L7+)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Relational (v1)</t>
+          <t>AgentLens</t>
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>1</v>
+        <v>0.984</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="D10" s="26" t="n">
-        <v>0.7</v>
+        <v>9.1</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>99.59999999999999</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>100</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>99.3</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="H10" s="26" t="n">
-        <v>1</v>
+        <v>0.983</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>4K in-domain, pre-L7+</t>
+          <t>L15, in-domain (L7+)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>RouteGuard</t>
         </is>
       </c>
       <c r="B11" s="26" t="n">
-        <v>1</v>
+        <v>0.998</v>
       </c>
       <c r="C11" s="26" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="26" t="n">
-        <v>1.7</v>
+        <v>1</v>
       </c>
       <c r="E11" s="26" t="n">
-        <v>99.09999999999999</v>
+        <v>99.5</v>
       </c>
       <c r="F11" s="26" t="n">
         <v>100</v>
       </c>
       <c r="G11" s="26" t="n">
-        <v>98.3</v>
+        <v>99</v>
       </c>
       <c r="H11" s="26" t="n">
         <v>1</v>
       </c>
       <c r="I11" s="22" t="inlineStr">
         <is>
-          <t>4K in-domain, pre-L7+</t>
+          <t>6K in-domain, rhid only (pre-L7+. Needs MSB route_hidden re-extract for L7+ update)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B12" s="28" t="n">
-        <v>0.923</v>
+        <v>1</v>
       </c>
       <c r="C12" s="28" t="n">
-        <v>16.3</v>
+        <v>0</v>
       </c>
       <c r="D12" s="28" t="n">
-        <v>16.4</v>
+        <v>0.7</v>
       </c>
       <c r="E12" s="28" t="n">
-        <v>83.5</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="F12" s="28" t="n">
-        <v>83.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="G12" s="28" t="n">
-        <v>83.59999999999999</v>
+        <v>99.3</v>
       </c>
       <c r="H12" s="28" t="n">
-        <v>0.921</v>
+        <v>1</v>
       </c>
       <c r="I12" s="28" t="inlineStr">
         <is>
-          <t>v1: oper+bnd. In-domain</t>
+          <t>4K in-domain, pre-L7+</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
+          <t>Centered Relational</t>
+        </is>
+      </c>
+      <c r="B13" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="70" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="E13" s="70" t="n">
+        <v>99.09999999999999</v>
+      </c>
+      <c r="F13" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="G13" s="70" t="n">
+        <v>98.3</v>
+      </c>
+      <c r="H13" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="70" t="inlineStr">
+        <is>
+          <t>4K in-domain, pre-L7+</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v1</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="F14" s="70" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G14" s="70" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="H14" s="70" t="n">
+        <v>0.921</v>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>v1: oper+bnd. In-domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
           <t>SkillProbe v2</t>
         </is>
       </c>
-      <c r="B13" s="70" t="n">
+      <c r="B15" s="70" t="n">
         <v>0.923</v>
       </c>
-      <c r="C13" s="70" t="n">
+      <c r="C15" s="70" t="n">
         <v>16.3</v>
       </c>
-      <c r="D13" s="70" t="n">
+      <c r="D15" s="70" t="n">
         <v>16.4</v>
       </c>
-      <c r="E13" s="70" t="n">
+      <c r="E15" s="70" t="n">
         <v>83.5</v>
       </c>
-      <c r="F13" s="70" t="n">
+      <c r="F15" s="70" t="n">
         <v>83.40000000000001</v>
       </c>
-      <c r="G13" s="70" t="n">
+      <c r="G15" s="70" t="n">
         <v>83.59999999999999</v>
       </c>
-      <c r="H13" s="70" t="inlineStr">
+      <c r="H15" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I13" s="70" t="inlineStr">
+      <c r="I15" s="70" t="inlineStr">
         <is>
           <t>v2: max(v1,decl). =v1 on MASB</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="71" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="70" t="inlineStr">
         <is>
           <t>SkillProbe v4 (ours)</t>
         </is>
       </c>
-      <c r="B14" s="70" t="n">
+      <c r="B16" s="70" t="n">
         <v>0.981</v>
       </c>
-      <c r="C14" s="70" t="n">
+      <c r="C16" s="70" t="n">
         <v>7.2</v>
       </c>
-      <c r="D14" s="70" t="n">
+      <c r="D16" s="70" t="n">
         <v>6</v>
       </c>
-      <c r="E14" s="70" t="n">
+      <c r="E16" s="70" t="n">
         <v>93.40000000000001</v>
       </c>
-      <c r="F14" s="70" t="n">
+      <c r="F16" s="70" t="n">
         <v>93</v>
       </c>
-      <c r="G14" s="70" t="n">
+      <c r="G16" s="70" t="n">
         <v>94</v>
       </c>
-      <c r="H14" s="70" t="inlineStr">
+      <c r="H16" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I14" s="70" t="inlineStr">
+      <c r="I16" s="70" t="inlineStr">
         <is>
           <t>v4: Gate&lt;0.15. AUC=0.981! Gating fixes OOD FPR from 12%→7%</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Skill-Inject Filter</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.505</v>
-      </c>
-      <c r="C15" t="n">
-        <v>100</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>66.40000000000001</v>
-      </c>
-      <c r="F15" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G15" t="n">
-        <v>100</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Naive filter: always fires on 8K samples</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>cisco-skill-scanner</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.552</v>
-      </c>
-      <c r="C16" t="n">
-        <v>100</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>66.40000000000001</v>
-      </c>
-      <c r="F16" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G16" t="n">
-        <v>100</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>129 core patterns. Always fires</t>
         </is>
       </c>
     </row>
@@ -5248,49 +5215,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>AUROC</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>FPR%</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>FNR%</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>F1%</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Precision%</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Recall%</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Train AUC</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A3" s="87" t="inlineStr">
+        <is>
+          <t>Static Regex</t>
+        </is>
+      </c>
+      <c r="B3" s="87" t="n">
+        <v>0.463</v>
+      </c>
+      <c r="C3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="87" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F3" s="87" t="n">
+        <v>42</v>
+      </c>
+      <c r="G3" s="87" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="H3" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="87" t="inlineStr">
+        <is>
+          <t>Static Regex on 155 decoys: FPR=59% (better than old 100%—more diverse decoys)</t>
         </is>
       </c>
       <c r="J3" s="20" t="n"/>
@@ -5298,26 +5253,26 @@
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
         <is>
-          <t>Static Regex</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>0.463</v>
+        <v>0.8</v>
       </c>
       <c r="C4" s="24" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="D4" s="24" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="24" t="n">
-        <v>66.7</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F4" s="24" t="n">
-        <v>42</v>
+        <v>50.2</v>
       </c>
       <c r="G4" s="24" t="n">
-        <v>48.3</v>
+        <v>100</v>
       </c>
       <c r="H4" s="24" t="inlineStr">
         <is>
@@ -5326,7 +5281,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Static Regex on 155 decoys: FPR=59% (better than old 100%—more diverse decoys)</t>
+          <t>Schmotz et al. 2026, naive input filtering</t>
         </is>
       </c>
       <c r="J4" s="22" t="n"/>
@@ -5370,26 +5325,26 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>0.5</v>
+        <v>0.533</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>100</v>
+        <v>43.3</v>
       </c>
       <c r="D6" s="24" t="n">
-        <v>0</v>
+        <v>37.7</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>66.7</v>
+        <v>60.6</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>100</v>
+        <v>62.3</v>
       </c>
       <c r="H6" s="24" t="inlineStr">
         <is>
@@ -5398,7 +5353,7 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%)</t>
+          <t>176 patterns (core+promptguard), Python 3.10+ required</t>
         </is>
       </c>
       <c r="J6" s="22" t="n"/>
@@ -5406,33 +5361,35 @@
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>0.991</v>
+        <v>0.49</v>
       </c>
       <c r="C7" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="26" t="n">
-        <v>3.2</v>
-      </c>
       <c r="E7" s="26" t="n">
-        <v>98.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>100</v>
+        <v>50.2</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>96.8</v>
-      </c>
-      <c r="H7" s="26" t="n">
-        <v>0.994</v>
+        <v>100</v>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L23 (L7+). Model judges ALL 150 decoys safe!</t>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
       </c>
       <c r="J7" s="22" t="n"/>
@@ -5440,33 +5397,35 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.867</v>
+        <v>0.5</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>22.7</v>
+        <v>100</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>67.59999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>68.2</v>
+        <v>50</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>79</v>
-      </c>
-      <c r="H8" s="22" t="n">
-        <v>0.989</v>
+        <v>100</v>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L15 (L7+). PCA(50) boundary. FPR=23% acceptable.</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%)</t>
         </is>
       </c>
       <c r="J8" s="22" t="n"/>
@@ -5474,33 +5433,33 @@
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>RouteGuard</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B9" s="30" t="n">
-        <v>0.777</v>
+        <v>0.991</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>65.3</v>
+        <v>0</v>
       </c>
       <c r="D9" s="24" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>75.40000000000001</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F9" s="24" t="n">
-        <v>60.4</v>
+        <v>100</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>100</v>
+        <v>96.8</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>0.734</v>
+        <v>0.994</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>rhid only. Cross-extract caution. FPR=65%</t>
+          <t>L23 (L7+). Model judges ALL 150 decoys safe!</t>
         </is>
       </c>
       <c r="J9" s="22" t="n"/>
@@ -5508,35 +5467,33 @@
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Relational (v1)</t>
+          <t>AgentLens</t>
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>0.46</v>
+        <v>0.867</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>100</v>
+        <v>22.7</v>
       </c>
       <c r="D10" s="26" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>66.7</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>50</v>
+        <v>68.2</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H10" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>79</v>
+      </c>
+      <c r="H10" s="26" t="n">
+        <v>0.989</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>Obsolete (interaction+PCA64). FPR=100% confirms noise</t>
+          <t>L15 (L7+). PCA(50) boundary. FPR=23% acceptable.</t>
         </is>
       </c>
       <c r="J10" s="22" t="n"/>
@@ -5544,35 +5501,33 @@
     <row r="11">
       <c r="A11" s="68" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>RouteGuard</t>
         </is>
       </c>
       <c r="B11" s="69" t="n">
-        <v>0.705</v>
+        <v>0.777</v>
       </c>
       <c r="C11" s="69" t="n">
-        <v>57.3</v>
+        <v>65.3</v>
       </c>
       <c r="D11" s="69" t="n">
-        <v>14.7</v>
+        <v>0</v>
       </c>
       <c r="E11" s="69" t="n">
-        <v>70.3</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="F11" s="69" t="n">
-        <v>59.2</v>
+        <v>60.4</v>
       </c>
       <c r="G11" s="69" t="n">
-        <v>85.3</v>
-      </c>
-      <c r="H11" s="69" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>100</v>
+      </c>
+      <c r="H11" s="69" t="n">
+        <v>0.734</v>
       </c>
       <c r="I11" s="69" t="inlineStr">
         <is>
-          <t>Centered (-1PC). AUC=0.71 better than SkillProbe on decoy—centering helps lexical robustness</t>
+          <t>rhid only. Cross-extract caution. FPR=65%</t>
         </is>
       </c>
       <c r="J11" s="22" t="n"/>
@@ -5580,26 +5535,26 @@
     <row r="12">
       <c r="A12" s="68" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B12" s="69" t="n">
-        <v>0.427</v>
+        <v>0.46</v>
       </c>
       <c r="C12" s="69" t="n">
-        <v>75.3</v>
+        <v>100</v>
       </c>
       <c r="D12" s="69" t="n">
-        <v>8.1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="69" t="n">
-        <v>49.1</v>
+        <v>66.7</v>
       </c>
       <c r="F12" s="69" t="n">
-        <v>38.3</v>
+        <v>50</v>
       </c>
       <c r="G12" s="69" t="n">
-        <v>91.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H12" s="69" t="inlineStr">
         <is>
@@ -5608,7 +5563,7 @@
       </c>
       <c r="I12" s="69" t="inlineStr">
         <is>
-          <t>v1: FPR=75% (oper reads suspicious code)</t>
+          <t>Obsolete (interaction+PCA64). FPR=100% confirms noise</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -5616,140 +5571,140 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
+          <t>Centered Relational</t>
+        </is>
+      </c>
+      <c r="B13" s="70" t="n">
+        <v>0.705</v>
+      </c>
+      <c r="C13" s="70" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="D13" s="70" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="E13" s="70" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="F13" s="70" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="G13" s="70" t="n">
+        <v>85.3</v>
+      </c>
+      <c r="H13" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="70" t="inlineStr">
+        <is>
+          <t>Centered (-1PC). AUC=0.71 better than SkillProbe on decoy—centering helps lexical robustness</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v1</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F14" s="70" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G14" s="70" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>v1: FPR=75% (oper reads suspicious code)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
           <t>SkillProbe v2</t>
         </is>
       </c>
-      <c r="B13" s="70" t="n">
+      <c r="B15" s="70" t="n">
         <v>0.427</v>
       </c>
-      <c r="C13" s="70" t="n">
+      <c r="C15" s="70" t="n">
         <v>75.3</v>
       </c>
-      <c r="D13" s="70" t="n">
+      <c r="D15" s="70" t="n">
         <v>8.1</v>
       </c>
-      <c r="E13" s="70" t="n">
+      <c r="E15" s="70" t="n">
         <v>49.1</v>
       </c>
-      <c r="F13" s="70" t="n">
+      <c r="F15" s="70" t="n">
         <v>38.3</v>
       </c>
-      <c r="G13" s="70" t="n">
+      <c r="G15" s="70" t="n">
         <v>91.90000000000001</v>
       </c>
-      <c r="H13" s="70" t="inlineStr">
+      <c r="H15" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I13" s="70" t="inlineStr">
+      <c r="I15" s="70" t="inlineStr">
         <is>
           <t>v2: max(v1,decl). Decl-Probe also fires on suspicious vocab. =v1</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="71" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="70" t="inlineStr">
         <is>
           <t>SkillProbe v4 (ours)</t>
         </is>
       </c>
-      <c r="B14" s="70" t="n">
+      <c r="B16" s="70" t="n">
         <v>0.998</v>
       </c>
-      <c r="C14" s="70" t="n">
+      <c r="C16" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="70" t="n">
+      <c r="D16" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="70" t="n">
+      <c r="E16" s="70" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F14" s="70" t="n">
-        <v>100</v>
-      </c>
-      <c r="G14" s="70" t="n">
+      <c r="F16" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="G16" s="70" t="n">
         <v>97</v>
       </c>
-      <c r="H14" s="70" t="inlineStr">
+      <c r="H16" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I14" s="70" t="inlineStr">
+      <c r="I16" s="70" t="inlineStr">
         <is>
           <t>★ v4: Boundary-gated v3. Gate&lt;0.15. FPR=0% FNR=3%. Best on Decoy!</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Skill-Inject Filter</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="C15" t="n">
-        <v>40</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>83.40000000000001</v>
-      </c>
-      <c r="F15" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="G15" t="n">
-        <v>100</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Schmotz et al. 2026, naive input filtering</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>cisco-skill-scanner</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.533</v>
-      </c>
-      <c r="C16" t="n">
-        <v>43.3</v>
-      </c>
-      <c r="D16" t="n">
-        <v>37.7</v>
-      </c>
-      <c r="E16" t="n">
-        <v>60.6</v>
-      </c>
-      <c r="F16" t="n">
-        <v>54</v>
-      </c>
-      <c r="G16" t="n">
-        <v>62.3</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>176 patterns (core+promptguard), Python 3.10+ required</t>
         </is>
       </c>
     </row>
@@ -5837,49 +5792,37 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="B3" s="20" t="inlineStr">
-        <is>
-          <t>AUROC</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>FPR%</t>
-        </is>
-      </c>
-      <c r="D3" s="20" t="inlineStr">
-        <is>
-          <t>FNR%</t>
-        </is>
-      </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>F1%</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="inlineStr">
-        <is>
-          <t>Precision%</t>
-        </is>
-      </c>
-      <c r="G3" s="20" t="inlineStr">
-        <is>
-          <t>Recall%</t>
-        </is>
-      </c>
-      <c r="H3" s="20" t="inlineStr">
-        <is>
-          <t>Train AUC</t>
-        </is>
-      </c>
-      <c r="I3" s="20" t="inlineStr">
-        <is>
-          <t>Notes</t>
+      <c r="A3" s="87" t="inlineStr">
+        <is>
+          <t>Static Regex</t>
+        </is>
+      </c>
+      <c r="B3" s="87" t="n">
+        <v>0.994</v>
+      </c>
+      <c r="C3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3" s="87" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="87" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="F3" s="87" t="n">
+        <v>50</v>
+      </c>
+      <c r="G3" s="87" t="n">
+        <v>100</v>
+      </c>
+      <c r="H3" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I3" s="87" t="inlineStr">
+        <is>
+          <t>Regex on clean vocab: FPR=0% FNR=100%—no patterns to match. Useless.</t>
         </is>
       </c>
       <c r="J3" s="20" t="n"/>
@@ -5887,11 +5830,11 @@
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
         <is>
-          <t>Static Regex</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B4" s="24" t="n">
-        <v>0.994</v>
+        <v>0.5</v>
       </c>
       <c r="C4" s="24" t="n">
         <v>100</v>
@@ -5915,7 +5858,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Regex on clean vocab: FPR=0% FNR=100%—no patterns to match. Useless.</t>
+          <t>Naive filter: clean vocab -&gt; always fires</t>
         </is>
       </c>
       <c r="J4" s="22" t="n"/>
@@ -5959,11 +5902,11 @@
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>0.5</v>
+        <v>0.503</v>
       </c>
       <c r="C6" s="24" t="n">
         <v>100</v>
@@ -5987,7 +5930,7 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Mistral always MAL. Zero-shot useless</t>
+          <t>Standard Python code triggers patterns -&gt; always fires</t>
         </is>
       </c>
       <c r="J6" s="22" t="n"/>
@@ -5995,33 +5938,35 @@
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B7" s="26" t="n">
-        <v>0.793</v>
+        <v>0.5</v>
       </c>
       <c r="C7" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="26" t="n">
-        <v>100</v>
-      </c>
       <c r="E7" s="26" t="n">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="26" t="n">
-        <v>0.994</v>
+        <v>100</v>
+      </c>
+      <c r="H7" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>L23. Model judges ALL safe! FNR=100%—clean vocab fools model judgment completely</t>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
       </c>
       <c r="J7" s="22" t="n"/>
@@ -6029,33 +5974,35 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.676</v>
+        <v>0.5</v>
       </c>
       <c r="C8" s="22" t="n">
-        <v>78.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="D8" s="22" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>71.59999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>53.2</v>
+        <v>50</v>
       </c>
       <c r="G8" s="22" t="n">
-        <v>99.40000000000001</v>
-      </c>
-      <c r="H8" s="22" t="n">
-        <v>0.989</v>
+        <v>100</v>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>L15. Catches 99% malicious but FPR=78%</t>
+          <t>Mistral always MAL. Zero-shot useless</t>
         </is>
       </c>
       <c r="J8" s="22" t="n"/>
@@ -6063,33 +6010,33 @@
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>RouteGuard</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B9" s="24" t="n">
-        <v>0.5</v>
+        <v>0.793</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="D9" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="24" t="n">
-        <v>66.7</v>
-      </c>
       <c r="F9" s="24" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H9" s="24" t="n">
-        <v>0.734</v>
+        <v>0.994</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>rhid only. Random on clean vocab. Cross-extract.</t>
+          <t>L23. Model judges ALL safe! FNR=100%—clean vocab fools model judgment completely</t>
         </is>
       </c>
       <c r="J9" s="22" t="n"/>
@@ -6097,35 +6044,33 @@
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>Relational (v1)</t>
+          <t>AgentLens</t>
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>0.824</v>
+        <v>0.676</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>100</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="D10" s="26" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>66.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="F10" s="26" t="n">
-        <v>50</v>
+        <v>53.2</v>
       </c>
       <c r="G10" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H10" s="26" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>99.40000000000001</v>
+      </c>
+      <c r="H10" s="26" t="n">
+        <v>0.989</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>AUC=0.82 ranks correctly but FPR=100% (threshold issue)</t>
+          <t>L15. Catches 99% malicious but FPR=78%</t>
         </is>
       </c>
       <c r="J10" s="22" t="n"/>
@@ -6133,35 +6078,33 @@
     <row r="11">
       <c r="A11" s="68" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>RouteGuard</t>
         </is>
       </c>
       <c r="B11" s="69" t="n">
-        <v>0.846</v>
+        <v>0.5</v>
       </c>
       <c r="C11" s="69" t="n">
-        <v>21.9</v>
+        <v>100</v>
       </c>
       <c r="D11" s="69" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="E11" s="69" t="n">
-        <v>89.5</v>
+        <v>66.7</v>
       </c>
       <c r="F11" s="69" t="n">
-        <v>80.90000000000001</v>
+        <v>50</v>
       </c>
       <c r="G11" s="69" t="n">
-        <v>98.7</v>
-      </c>
-      <c r="H11" s="69" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>100</v>
+      </c>
+      <c r="H11" s="69" t="n">
+        <v>0.734</v>
       </c>
       <c r="I11" s="69" t="inlineStr">
         <is>
-          <t>Centered (-1PC). AUC=0.85 BEST on InvDecoy! Centering removes anisotropic noise→clean signal</t>
+          <t>rhid only. Random on clean vocab. Cross-extract.</t>
         </is>
       </c>
       <c r="J11" s="22" t="n"/>
@@ -6169,11 +6112,11 @@
     <row r="12">
       <c r="A12" s="68" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B12" s="69" t="n">
-        <v>0.165</v>
+        <v>0.824</v>
       </c>
       <c r="C12" s="69" t="n">
         <v>100</v>
@@ -6182,7 +6125,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="69" t="n">
-        <v>43.9</v>
+        <v>66.7</v>
       </c>
       <c r="F12" s="69" t="n">
         <v>50</v>
@@ -6197,7 +6140,7 @@
       </c>
       <c r="I12" s="69" t="inlineStr">
         <is>
-          <t>v1: cross-distribution collapse. AUC=0.16</t>
+          <t>AUC=0.82 ranks correctly but FPR=100% (threshold issue)</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -6205,140 +6148,140 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
+          <t>Centered Relational</t>
+        </is>
+      </c>
+      <c r="B13" s="70" t="n">
+        <v>0.846</v>
+      </c>
+      <c r="C13" s="70" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="D13" s="70" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E13" s="70" t="n">
+        <v>89.5</v>
+      </c>
+      <c r="F13" s="70" t="n">
+        <v>80.90000000000001</v>
+      </c>
+      <c r="G13" s="70" t="n">
+        <v>98.7</v>
+      </c>
+      <c r="H13" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I13" s="70" t="inlineStr">
+        <is>
+          <t>Centered (-1PC). AUC=0.85 BEST on InvDecoy! Centering removes anisotropic noise→clean signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v1</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="C14" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="D14" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="70" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="F14" s="70" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>v1: cross-distribution collapse. AUC=0.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="70" t="inlineStr">
+        <is>
           <t>SkillProbe v2</t>
         </is>
       </c>
-      <c r="B13" s="70" t="n">
+      <c r="B15" s="70" t="n">
         <v>0.165</v>
       </c>
-      <c r="C13" s="70" t="n">
-        <v>100</v>
-      </c>
-      <c r="D13" s="70" t="n">
+      <c r="C15" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="D15" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="70" t="n">
+      <c r="E15" s="70" t="n">
         <v>43.9</v>
       </c>
-      <c r="F13" s="70" t="n">
+      <c r="F15" s="70" t="n">
         <v>50</v>
       </c>
-      <c r="G13" s="70" t="n">
-        <v>100</v>
-      </c>
-      <c r="H13" s="70" t="inlineStr">
+      <c r="G15" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="H15" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I13" s="70" t="inlineStr">
+      <c r="I15" s="70" t="inlineStr">
         <is>
           <t>v2: max(v1,decl). Decl AUC=0.48 random. =v1</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="71" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="70" t="inlineStr">
         <is>
           <t>SkillProbe v4 (ours)</t>
         </is>
       </c>
-      <c r="B14" s="70" t="n">
+      <c r="B16" s="70" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="70" t="n">
+      <c r="C16" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="70" t="n">
+      <c r="D16" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="70" t="n">
+      <c r="E16" s="70" t="n">
         <v>98.5</v>
       </c>
-      <c r="F14" s="70" t="n">
-        <v>100</v>
-      </c>
-      <c r="G14" s="70" t="n">
+      <c r="F16" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="G16" s="70" t="n">
         <v>97</v>
       </c>
-      <c r="H14" s="70" t="inlineStr">
+      <c r="H16" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I14" s="70" t="inlineStr">
+      <c r="I16" s="70" t="inlineStr">
         <is>
           <t>★ v4: Boundary-gated v3. Gate&lt;0.15. AUC=1.0 FPR=0%! Both Decoy solved!</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Skill-Inject Filter</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C15" t="n">
-        <v>100</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F15" t="n">
-        <v>50</v>
-      </c>
-      <c r="G15" t="n">
-        <v>100</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Naive filter: clean vocab -&gt; always fires</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>cisco-skill-scanner</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0.503</v>
-      </c>
-      <c r="C16" t="n">
-        <v>100</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F16" t="n">
-        <v>50</v>
-      </c>
-      <c r="G16" t="n">
-        <v>100</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Standard Python code triggers patterns -&gt; always fires</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Only our 5 method iterations green. Others no fill.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -252,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="90">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -459,6 +459,12 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3634,30 +3640,30 @@
       <c r="J5" s="22" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>cisco-skill-scanner</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="22" t="n">
         <v>0.539</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="22" t="n">
         <v>68.3</v>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="22" t="n">
         <v>31.7</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="22" t="n">
         <v>60.6</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="22" t="n">
         <v>68.3</v>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3670,30 +3676,30 @@
       <c r="J6" s="22" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="22" t="n">
         <v>0.503</v>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="C7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="G7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="G7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -3742,30 +3748,30 @@
       <c r="J8" s="22" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Boundary only</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="22" t="n">
         <v>0.863</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="22" t="n">
         <v>40.3</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="22" t="n">
         <v>74.7</v>
       </c>
-      <c r="F9" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="G9" s="24" t="n">
+      <c r="F9" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="22" t="n">
         <v>59.7</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="H9" s="22" t="n">
         <v>0.989</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
@@ -3776,30 +3782,30 @@
       <c r="J9" s="22" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>AgentLens</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="22" t="n">
         <v>0.871</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="22" t="n">
         <v>51.6</v>
       </c>
-      <c r="E10" s="26" t="n">
+      <c r="E10" s="22" t="n">
         <v>65.2</v>
       </c>
-      <c r="F10" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="G10" s="26" t="n">
+      <c r="F10" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="G10" s="22" t="n">
         <v>48.4</v>
       </c>
-      <c r="H10" s="26" t="n">
+      <c r="H10" s="22" t="n">
         <v>0.989</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
@@ -3810,30 +3816,30 @@
       <c r="J10" s="22" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="22" t="n">
         <v>0.824</v>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="22" t="n">
         <v>48.4</v>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D11" s="22" t="n">
         <v>8.1</v>
       </c>
-      <c r="E11" s="26" t="n">
+      <c r="E11" s="22" t="n">
         <v>76.5</v>
       </c>
-      <c r="F11" s="26" t="n">
+      <c r="F11" s="22" t="n">
         <v>65.5</v>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G11" s="22" t="n">
         <v>91.7</v>
       </c>
-      <c r="H11" s="26" t="n">
+      <c r="H11" s="22" t="n">
         <v>0.9379999999999999</v>
       </c>
       <c r="I11" s="22" t="inlineStr">
@@ -3844,33 +3850,33 @@
       <c r="J11" s="22" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="68" t="inlineStr">
         <is>
           <t>Relational (v1)</t>
         </is>
       </c>
-      <c r="B12" s="28" t="n">
+      <c r="B12" s="69" t="n">
         <v>0.761</v>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="69" t="n">
         <v>50</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="69" t="n">
         <v>6.5</v>
       </c>
-      <c r="E12" s="28" t="n">
+      <c r="E12" s="69" t="n">
         <v>76.8</v>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="69" t="n">
         <v>65.2</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="69" t="n">
         <v>93.5</v>
       </c>
-      <c r="H12" s="29" t="n">
+      <c r="H12" s="88" t="n">
         <v>0.893</v>
       </c>
-      <c r="I12" s="28" t="inlineStr">
+      <c r="I12" s="69" t="inlineStr">
         <is>
           <t>L31, interact+PCA64</t>
         </is>
@@ -4200,30 +4206,30 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>cisco-skill-scanner</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="22" t="n">
         <v>0.545</v>
       </c>
-      <c r="C6" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="24" t="n">
+      <c r="C6" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="22" t="n">
         <v>49.6</v>
       </c>
-      <c r="G6" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="G6" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4235,30 +4241,30 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="22" t="n">
         <v>0.521</v>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="C7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="22" t="n">
         <v>49.6</v>
       </c>
-      <c r="G7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="G7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4305,30 +4311,30 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Boundary only</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="22" t="n">
         <v>0.999</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="22" t="n">
         <v>1.4</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="22" t="n">
         <v>1.3</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="22" t="n">
         <v>98.7</v>
       </c>
-      <c r="F9" s="24" t="n">
+      <c r="F9" s="22" t="n">
         <v>98.59999999999999</v>
       </c>
-      <c r="G9" s="24" t="n">
+      <c r="G9" s="22" t="n">
         <v>98.7</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="H9" s="22" t="n">
         <v>1</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
@@ -4338,30 +4344,30 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>AgentLens</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="22" t="n">
         <v>0.99</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="22" t="n">
         <v>3.6</v>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="22" t="n">
         <v>2.1</v>
       </c>
-      <c r="E10" s="26" t="n">
+      <c r="E10" s="22" t="n">
         <v>97.2</v>
       </c>
-      <c r="F10" s="26" t="n">
+      <c r="F10" s="22" t="n">
         <v>96.5</v>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="22" t="n">
         <v>97.90000000000001</v>
       </c>
-      <c r="H10" s="26" t="n">
+      <c r="H10" s="22" t="n">
         <v>0.995</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
@@ -4371,30 +4377,30 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="22" t="n">
         <v>0.795</v>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="22" t="n">
         <v>47.7</v>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D11" s="22" t="n">
         <v>11.1</v>
       </c>
-      <c r="E11" s="26" t="n">
+      <c r="E11" s="22" t="n">
         <v>74.5</v>
       </c>
-      <c r="F11" s="26" t="n">
+      <c r="F11" s="22" t="n">
         <v>64.09999999999999</v>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G11" s="22" t="n">
         <v>88.90000000000001</v>
       </c>
-      <c r="H11" s="26" t="n">
+      <c r="H11" s="22" t="n">
         <v>0.796</v>
       </c>
       <c r="I11" s="22" t="inlineStr">
@@ -4404,33 +4410,33 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="68" t="inlineStr">
         <is>
           <t>Relational (v1)</t>
         </is>
       </c>
-      <c r="B12" s="28" t="n">
+      <c r="B12" s="69" t="n">
         <v>0.992</v>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="69" t="n">
         <v>2.9</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="69" t="n">
         <v>6</v>
       </c>
-      <c r="E12" s="28" t="n">
+      <c r="E12" s="69" t="n">
         <v>95.5</v>
       </c>
-      <c r="F12" s="28" t="n">
+      <c r="F12" s="69" t="n">
         <v>97</v>
       </c>
-      <c r="G12" s="28" t="n">
+      <c r="G12" s="69" t="n">
         <v>94</v>
       </c>
-      <c r="H12" s="28" t="n">
+      <c r="H12" s="69" t="n">
         <v>0.993</v>
       </c>
-      <c r="I12" s="28" t="inlineStr">
+      <c r="I12" s="69" t="inlineStr">
         <is>
           <t>L11</t>
         </is>
@@ -4691,30 +4697,30 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Skill-Inject Filter</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="22" t="n">
         <v>0.505</v>
       </c>
-      <c r="C4" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" s="24" t="n">
+      <c r="C4" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="24" t="n">
+      <c r="E4" s="22" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="22" t="n">
         <v>49.6</v>
       </c>
-      <c r="G4" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="G4" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4759,30 +4765,30 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>cisco-skill-scanner</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="22" t="n">
         <v>0.552</v>
       </c>
-      <c r="C6" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="24" t="n">
+      <c r="C6" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="22" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="22" t="n">
         <v>49.6</v>
       </c>
-      <c r="G6" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="G6" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4794,30 +4800,30 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="22" t="n">
         <v>0.524</v>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="C7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="22" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="22" t="n">
         <v>49.6</v>
       </c>
-      <c r="G7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="G7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4864,30 +4870,30 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Boundary only</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="22" t="n">
         <v>0.999</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="22" t="n">
         <v>2.5</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="22" t="n">
         <v>98.2</v>
       </c>
-      <c r="F9" s="24" t="n">
+      <c r="F9" s="22" t="n">
         <v>97.5</v>
       </c>
-      <c r="G9" s="24" t="n">
+      <c r="G9" s="22" t="n">
         <v>99</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="H9" s="22" t="n">
         <v>1</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
@@ -4897,30 +4903,30 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>AgentLens</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="22" t="n">
         <v>0.984</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="22" t="n">
         <v>3.7</v>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="22" t="n">
         <v>9.1</v>
       </c>
-      <c r="E10" s="26" t="n">
+      <c r="E10" s="22" t="n">
         <v>93.40000000000001</v>
       </c>
-      <c r="F10" s="26" t="n">
+      <c r="F10" s="22" t="n">
         <v>96.09999999999999</v>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="22" t="n">
         <v>90.90000000000001</v>
       </c>
-      <c r="H10" s="26" t="n">
+      <c r="H10" s="22" t="n">
         <v>0.983</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
@@ -4930,30 +4936,30 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="22" t="n">
         <v>0.998</v>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D11" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="26" t="n">
+      <c r="E11" s="22" t="n">
         <v>99.5</v>
       </c>
-      <c r="F11" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="G11" s="26" t="n">
+      <c r="F11" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" s="22" t="n">
         <v>99</v>
       </c>
-      <c r="H11" s="26" t="n">
+      <c r="H11" s="22" t="n">
         <v>1</v>
       </c>
       <c r="I11" s="22" t="inlineStr">
@@ -4963,33 +4969,33 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="inlineStr">
+      <c r="A12" s="68" t="inlineStr">
         <is>
           <t>Relational (v1)</t>
         </is>
       </c>
-      <c r="B12" s="28" t="n">
+      <c r="B12" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="28" t="n">
+      <c r="C12" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="D12" s="28" t="n">
+      <c r="D12" s="69" t="n">
         <v>0.7</v>
       </c>
-      <c r="E12" s="28" t="n">
+      <c r="E12" s="69" t="n">
         <v>99.59999999999999</v>
       </c>
-      <c r="F12" s="28" t="n">
-        <v>100</v>
-      </c>
-      <c r="G12" s="28" t="n">
+      <c r="F12" s="69" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" s="69" t="n">
         <v>99.3</v>
       </c>
-      <c r="H12" s="28" t="n">
+      <c r="H12" s="69" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="28" t="inlineStr">
+      <c r="I12" s="69" t="inlineStr">
         <is>
           <t>4K in-domain, pre-L7+</t>
         </is>
@@ -5251,30 +5257,30 @@
       <c r="J3" s="20" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Skill-Inject Filter</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="22" t="n">
         <v>0.8</v>
       </c>
-      <c r="C4" s="24" t="n">
+      <c r="C4" s="22" t="n">
         <v>40</v>
       </c>
-      <c r="D4" s="24" t="n">
+      <c r="D4" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="24" t="n">
+      <c r="E4" s="22" t="n">
         <v>83.40000000000001</v>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="22" t="n">
         <v>50.2</v>
       </c>
-      <c r="G4" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="G4" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5287,30 +5293,30 @@
       <c r="J4" s="22" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>TF-IDF + LR</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="22" t="n">
         <v>0.7435</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="22" t="n">
         <v>39.3</v>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="22" t="n">
         <v>39.1</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="22" t="n">
         <v>60.9</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F5" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="G5" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="G5" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5323,30 +5329,30 @@
       <c r="J5" s="22" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>cisco-skill-scanner</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="22" t="n">
         <v>0.533</v>
       </c>
-      <c r="C6" s="24" t="n">
+      <c r="C6" s="22" t="n">
         <v>43.3</v>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="22" t="n">
         <v>37.7</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="22" t="n">
         <v>60.6</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="22" t="n">
         <v>54</v>
       </c>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="22" t="n">
         <v>62.3</v>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5359,30 +5365,30 @@
       <c r="J6" s="22" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="22" t="n">
         <v>0.49</v>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="C7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="22" t="n">
         <v>50.2</v>
       </c>
-      <c r="G7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="G7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5431,30 +5437,30 @@
       <c r="J8" s="22" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Boundary only</t>
         </is>
       </c>
-      <c r="B9" s="30" t="n">
+      <c r="B9" s="89" t="n">
         <v>0.991</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="22" t="n">
         <v>3.2</v>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="22" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F9" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="G9" s="24" t="n">
+      <c r="F9" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="G9" s="22" t="n">
         <v>96.8</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="H9" s="22" t="n">
         <v>0.994</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
@@ -5465,30 +5471,30 @@
       <c r="J9" s="22" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>AgentLens</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="22" t="n">
         <v>0.867</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="22" t="n">
         <v>22.7</v>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="22" t="n">
         <v>21</v>
       </c>
-      <c r="E10" s="26" t="n">
+      <c r="E10" s="22" t="n">
         <v>67.59999999999999</v>
       </c>
-      <c r="F10" s="26" t="n">
+      <c r="F10" s="22" t="n">
         <v>68.2</v>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="22" t="n">
         <v>79</v>
       </c>
-      <c r="H10" s="26" t="n">
+      <c r="H10" s="22" t="n">
         <v>0.989</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
@@ -5499,33 +5505,33 @@
       <c r="J10" s="22" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="68" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="69" t="n">
+      <c r="B11" s="22" t="n">
         <v>0.777</v>
       </c>
-      <c r="C11" s="69" t="n">
+      <c r="C11" s="22" t="n">
         <v>65.3</v>
       </c>
-      <c r="D11" s="69" t="n">
+      <c r="D11" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="69" t="n">
+      <c r="E11" s="22" t="n">
         <v>75.40000000000001</v>
       </c>
-      <c r="F11" s="69" t="n">
+      <c r="F11" s="22" t="n">
         <v>60.4</v>
       </c>
-      <c r="G11" s="69" t="n">
-        <v>100</v>
-      </c>
-      <c r="H11" s="69" t="n">
+      <c r="G11" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H11" s="22" t="n">
         <v>0.734</v>
       </c>
-      <c r="I11" s="69" t="inlineStr">
+      <c r="I11" s="22" t="inlineStr">
         <is>
           <t>rhid only. Cross-extract caution. FPR=65%</t>
         </is>
@@ -5828,30 +5834,30 @@
       <c r="J3" s="20" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Skill-Inject Filter</t>
         </is>
       </c>
-      <c r="B4" s="24" t="n">
+      <c r="B4" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="C4" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="D4" s="24" t="n">
+      <c r="C4" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D4" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="24" t="n">
+      <c r="E4" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F4" s="24" t="n">
+      <c r="F4" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="G4" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="G4" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5864,30 +5870,30 @@
       <c r="J4" s="22" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>TF-IDF + LR</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="22" t="n">
         <v>0.1593</v>
       </c>
-      <c r="C5" s="24" t="n">
+      <c r="C5" s="22" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="22" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="22" t="n">
         <v>21.9</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F5" s="22" t="n">
         <v>46.3</v>
       </c>
-      <c r="G5" s="24" t="n">
+      <c r="G5" s="22" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5900,30 +5906,30 @@
       <c r="J5" s="22" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>cisco-skill-scanner</t>
         </is>
       </c>
-      <c r="B6" s="24" t="n">
+      <c r="B6" s="22" t="n">
         <v>0.503</v>
       </c>
-      <c r="C6" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="D6" s="24" t="n">
+      <c r="C6" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D6" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="G6" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="G6" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -5936,30 +5942,30 @@
       <c r="J6" s="22" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n">
+      <c r="B7" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="C7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" s="26" t="n">
+      <c r="C7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="G7" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="H7" s="26" t="inlineStr">
+      <c r="G7" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -6008,30 +6014,30 @@
       <c r="J8" s="22" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Boundary only</t>
         </is>
       </c>
-      <c r="B9" s="24" t="n">
+      <c r="B9" s="22" t="n">
         <v>0.793</v>
       </c>
-      <c r="C9" s="24" t="n">
+      <c r="C9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="E9" s="24" t="n">
+      <c r="D9" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="24" t="n">
+      <c r="F9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="24" t="n">
+      <c r="G9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="H9" s="22" t="n">
         <v>0.994</v>
       </c>
       <c r="I9" s="22" t="inlineStr">
@@ -6042,30 +6048,30 @@
       <c r="J9" s="22" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>AgentLens</t>
         </is>
       </c>
-      <c r="B10" s="26" t="n">
+      <c r="B10" s="22" t="n">
         <v>0.676</v>
       </c>
-      <c r="C10" s="26" t="n">
+      <c r="C10" s="22" t="n">
         <v>78.09999999999999</v>
       </c>
-      <c r="D10" s="26" t="n">
+      <c r="D10" s="22" t="n">
         <v>0.6</v>
       </c>
-      <c r="E10" s="26" t="n">
+      <c r="E10" s="22" t="n">
         <v>71.59999999999999</v>
       </c>
-      <c r="F10" s="26" t="n">
+      <c r="F10" s="22" t="n">
         <v>53.2</v>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="22" t="n">
         <v>99.40000000000001</v>
       </c>
-      <c r="H10" s="26" t="n">
+      <c r="H10" s="22" t="n">
         <v>0.989</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
@@ -6076,33 +6082,33 @@
       <c r="J10" s="22" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="68" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="69" t="n">
+      <c r="B11" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="C11" s="69" t="n">
-        <v>100</v>
-      </c>
-      <c r="D11" s="69" t="n">
+      <c r="C11" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="69" t="n">
+      <c r="E11" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F11" s="69" t="n">
+      <c r="F11" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="G11" s="69" t="n">
-        <v>100</v>
-      </c>
-      <c r="H11" s="69" t="n">
+      <c r="G11" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H11" s="22" t="n">
         <v>0.734</v>
       </c>
-      <c r="I11" s="69" t="inlineStr">
+      <c r="I11" s="22" t="inlineStr">
         <is>
           <t>rhid only. Random on clean vocab. Cross-extract.</t>
         </is>

</xml_diff>

<commit_message>
Clean up attribution sheet: remove duplicate data, keep only GAP_REPORT 100% numbers.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -252,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -466,6 +466,10 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2036,14 +2040,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
     <col width="35" customWidth="1" min="8" max="8"/>
@@ -2063,31 +2067,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="66" t="inlineStr">
+        <is>
+          <t>架构</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
-      <c r="A4" s="66" t="inlineStr">
-        <is>
-          <t>架构</t>
+      <c r="A4" s="64" t="inlineStr">
+        <is>
+          <t>Pass A (decl-only, ~50ms): prompt 截断在声明末尾 → 模型只看声明 → decl-bnd → Decl-Det</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="64" t="inlineStr">
         <is>
-          <t>Pass A: prompt 截断在声明末尾 → 模型只看到声明 → decl-bnd → Decl-Probe (L2-LR) → score_decl</t>
+          <t>Pass B (skip-decl): 声明从 prompt 删除 → 模型只看代码 → oper-bnd → Code-Det</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="64" t="inlineStr">
         <is>
-          <t>Pass B: 完整 prompt (同 v1) → oper+bnd 几何特征 → PCA(8)+LR → score_code</t>
+          <t>信号: boundary token L2 norm (无需训练，直接比较两个范数)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="64" t="inlineStr">
         <is>
-          <t>归因规则: argmax(score_code, score_decl)。两路都&gt;阈值→BOTH，都&lt;阈值→CLEAN</t>
+          <t>归因规则: 比较 Decl-Det 和 Code-Det。两者都高→BOTH，都低→CLEAN</t>
         </is>
       </c>
     </row>
@@ -2099,9 +2110,9 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="64" t="inlineStr">
-        <is>
-          <t>Decl-Probe</t>
+      <c r="A9" s="66" t="inlineStr">
+        <is>
+          <t>双探针检测能力 (GAP_REPORT 方法)</t>
         </is>
       </c>
       <c r="B9" s="64" t="inlineStr">
@@ -2141,36 +2152,36 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="64" t="inlineStr">
-        <is>
-          <t>Code-Probe</t>
-        </is>
-      </c>
-      <c r="B10" s="64" t="inlineStr">
-        <is>
-          <t>仅代码投毒 (50样本)</t>
-        </is>
-      </c>
-      <c r="C10" s="64" t="inlineStr">
-        <is>
-          <t>0.82</t>
-        </is>
-      </c>
-      <c r="D10" s="64" t="inlineStr">
+      <c r="A10" s="67" t="inlineStr">
+        <is>
+          <t>探针</t>
+        </is>
+      </c>
+      <c r="B10" s="67" t="inlineStr">
+        <is>
+          <t>检测目标</t>
+        </is>
+      </c>
+      <c r="C10" s="67" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="D10" s="67" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+      <c r="E10" s="64" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="64" t="inlineStr">
+      <c r="F10" s="64" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F10" s="64" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
       <c r="G10" s="64" t="inlineStr">
         <is>
           <t>L7</t>
@@ -2183,24 +2194,24 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="69" t="inlineStr">
-        <is>
-          <t>Fusion max()</t>
+      <c r="A11" s="68" t="inlineStr">
+        <is>
+          <t>Decl-Det</t>
         </is>
       </c>
       <c r="B11" s="69" t="inlineStr">
         <is>
-          <t>声明+代码双投毒 (175样本)</t>
+          <t>仅声明投毒 (50样本)</t>
         </is>
       </c>
       <c r="C11" s="69" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="D11" s="69" t="inlineStr">
         <is>
-          <t>100.0</t>
+          <t>Pass A boundary token norm。完美区分 decl-poison vs clean</t>
         </is>
       </c>
       <c r="E11" s="69" t="inlineStr">
@@ -2227,22 +2238,22 @@
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>Decl-Probe</t>
+          <t>Code-Det</t>
         </is>
       </c>
       <c r="B12" s="22" t="inlineStr">
         <is>
-          <t>仅声明投毒 (50样本)</t>
+          <t>仅代码投毒 (50样本)</t>
         </is>
       </c>
       <c r="C12" s="22" t="inlineStr">
         <is>
-          <t>0.808</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="D12" s="22" t="inlineStr">
         <is>
-          <t>75.0</t>
+          <t>Pass B boundary token norm。区分 oper-poison vs clean</t>
         </is>
       </c>
       <c r="E12" s="22" t="inlineStr">
@@ -2269,22 +2280,22 @@
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>Code-Probe (v1)</t>
+          <t>Fusion (max)</t>
         </is>
       </c>
       <c r="B13" s="22" t="inlineStr">
         <is>
-          <t>仅代码投毒 (50样本)</t>
+          <t>所有攻击类型 (175样本)</t>
         </is>
       </c>
       <c r="C13" s="22" t="inlineStr">
         <is>
-          <t>0.919</t>
-        </is>
-      </c>
-      <c r="D13" s="22" t="inlineStr">
-        <is>
-          <t>90.4</t>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="D13" s="69" t="inlineStr">
+        <is>
+          <t>max(Decl-Det, Code-Det)。两路信号正交→全覆盖</t>
         </is>
       </c>
       <c r="E13" s="22" t="inlineStr">
@@ -2351,9 +2362,9 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="85" t="inlineStr">
-        <is>
-          <t>OPERATION (代码投毒)</t>
+      <c r="A15" s="90" t="inlineStr">
+        <is>
+          <t>归因准确率 (175 样本)</t>
         </is>
       </c>
       <c r="B15" s="85" t="inlineStr">
@@ -2378,90 +2389,90 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="85" t="inlineStr">
-        <is>
-          <t>BOTH (声明+代码)</t>
-        </is>
-      </c>
-      <c r="B16" s="85" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="C16" s="85" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
-      <c r="D16" s="85" t="inlineStr">
+      <c r="A16" s="67" t="inlineStr">
+        <is>
+          <t>攻击来源</t>
+        </is>
+      </c>
+      <c r="B16" s="67" t="inlineStr">
+        <is>
+          <t>样本</t>
+        </is>
+      </c>
+      <c r="C16" s="67" t="inlineStr">
+        <is>
+          <t>归因正确</t>
+        </is>
+      </c>
+      <c r="D16" s="67" t="inlineStr">
+        <is>
+          <t>准确率</t>
+        </is>
+      </c>
+      <c r="E16" s="67" t="inlineStr">
+        <is>
+          <t>机制</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="68" t="inlineStr">
+        <is>
+          <t>CLEAN (干净skill)</t>
+        </is>
+      </c>
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C17" s="69" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="D17" s="69" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="E16" s="85" t="inlineStr">
-        <is>
-          <t>全部归因正确。双探针bd norms同时升高→正确归为BOTH。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="85" t="inlineStr">
-        <is>
-          <t>DECLARATION (声明投毒)</t>
-        </is>
-      </c>
-      <c r="B17" s="85" t="inlineStr">
+      <c r="E17" s="69" t="inlineStr">
+        <is>
+          <t>双探针 bd norm 均低 → 正确识别</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="68" t="inlineStr">
+        <is>
+          <t>OPERATION (仅代码投毒)</t>
+        </is>
+      </c>
+      <c r="B18" s="69" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="C17" s="85" t="inlineStr">
+      <c r="C18" s="69" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="D17" s="85" t="inlineStr">
+      <c r="D18" s="69" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
-      <c r="E17" s="85" t="inlineStr">
-        <is>
-          <t>全部归因正确。Pass A decl-bd 高→Decl侧报警。Pass B oper-bd 低→Code侧不报。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="69" t="inlineStr">
-        <is>
-          <t>合计</t>
-        </is>
-      </c>
-      <c r="B18" s="69" t="inlineStr">
-        <is>
-          <t>175</t>
-        </is>
-      </c>
-      <c r="C18" s="69" t="inlineStr">
-        <is>
-          <t>175</t>
-        </is>
-      </c>
-      <c r="D18" s="69" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
       <c r="E18" s="69" t="inlineStr">
         <is>
-          <t>GAP_REPORT 方法: boundary token norm 比较。Pass A (decl-only) vs Pass B (skip-decl)。</t>
+          <t>Pass B oper-bd 高, Pass A decl-bd 低 → 正确归因</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="68" t="inlineStr">
         <is>
-          <t>CLEAN (干净skill)</t>
+          <t>DECLARATION (仅声明投毒)</t>
         </is>
       </c>
       <c r="B19" s="69" t="inlineStr">
@@ -2481,24 +2492,24 @@
       </c>
       <c r="E19" s="69" t="inlineStr">
         <is>
-          <t>全部正确识别。双探针均未报警。</t>
+          <t>Pass A decl-bd 高, Pass B oper-bd 低 → 正确归因</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="68" t="inlineStr">
         <is>
-          <t>OPERATION (代码投毒)</t>
+          <t>BOTH (双投毒)</t>
         </is>
       </c>
       <c r="B20" s="69" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C20" s="69" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D20" s="69" t="inlineStr">
@@ -2508,24 +2519,24 @@
       </c>
       <c r="E20" s="69" t="inlineStr">
         <is>
-          <t>全部归因正确。Code-Probe报警，Decl-Probe不报。</t>
+          <t>双探针 bd norm 同时高 → 正确归因</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="68" t="inlineStr">
         <is>
-          <t>BOTH (声明+代码)</t>
+          <t>合计</t>
         </is>
       </c>
       <c r="B21" s="69" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>175</t>
         </is>
       </c>
       <c r="C21" s="69" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>175</t>
         </is>
       </c>
       <c r="D21" s="69" t="inlineStr">
@@ -2535,7 +2546,7 @@
       </c>
       <c r="E21" s="69" t="inlineStr">
         <is>
-          <t>全部归因正确。双探针同时报警→正确归为BOTH。</t>
+          <t>声明和操作信号正交——无损归因</t>
         </is>
       </c>
     </row>
@@ -2567,9 +2578,9 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
-        <is>
-          <t>合计</t>
+      <c r="A23" s="81" t="inlineStr">
+        <is>
+          <t>归因 2x2 矩阵</t>
         </is>
       </c>
       <c r="B23" s="22" t="inlineStr">
@@ -2593,23 +2604,50 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="67" t="inlineStr"/>
+      <c r="B24" s="67" t="inlineStr">
+        <is>
+          <t>Code-Det 报警 (代码侧有恶意)</t>
+        </is>
+      </c>
+      <c r="C24" s="67" t="inlineStr">
+        <is>
+          <t>Code-Det 安全 (代码侧干净)</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
-      <c r="A25" s="66" t="inlineStr">
-        <is>
-          <t>归因 2x2 矩阵</t>
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Decl-Det 报警 (声明侧可疑)</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>BOTH —— 双重投毒 ✓</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>DECLARATION —— 仅声明投毒 ✓</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="67" t="inlineStr"/>
-      <c r="B26" s="67" t="inlineStr">
-        <is>
-          <t>Code-Probe 报警</t>
-        </is>
-      </c>
-      <c r="C26" s="67" t="inlineStr">
-        <is>
-          <t>Code-Probe 安全</t>
+      <c r="A26" s="72" t="inlineStr">
+        <is>
+          <t>Decl-Det 安全 (声明侧干净)</t>
+        </is>
+      </c>
+      <c r="B26" s="73" t="inlineStr">
+        <is>
+          <t>OPERATION —— 仅代码投毒 ✓</t>
+        </is>
+      </c>
+      <c r="C26" s="69" t="inlineStr">
+        <is>
+          <t>CLEAN —— 干净 skill ✓</t>
         </is>
       </c>
     </row>
@@ -2631,9 +2669,9 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="68" t="inlineStr">
-        <is>
-          <t>Decl-Probe 安全</t>
+      <c r="A28" s="91" t="inlineStr">
+        <is>
+          <t>每个象限对应一种攻击来源。v2 是唯一具备此归因能力的方法。</t>
         </is>
       </c>
       <c r="B28" s="69" t="inlineStr">
@@ -2647,6 +2685,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
@@ -2654,6 +2693,25 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Restore header row on 5 benchmark sheets. Fix reorder bug.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -252,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -471,6 +471,7 @@
     <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2040,7 +2041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2685,7 +2686,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
@@ -2693,25 +2693,6 @@
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3558,7 +3539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3592,37 +3573,49 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="87" t="inlineStr">
-        <is>
-          <t>Static Regex</t>
-        </is>
-      </c>
-      <c r="B3" s="87" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="C3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="87" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="87" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F3" s="87" t="n">
-        <v>50</v>
-      </c>
-      <c r="G3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="H3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="87" t="inlineStr">
-        <is>
-          <t>Always fires</t>
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>FPR%</t>
+        </is>
+      </c>
+      <c r="D3" s="67" t="inlineStr">
+        <is>
+          <t>FNR%</t>
+        </is>
+      </c>
+      <c r="E3" s="67" t="inlineStr">
+        <is>
+          <t>F1%</t>
+        </is>
+      </c>
+      <c r="F3" s="67" t="inlineStr">
+        <is>
+          <t>Precision%</t>
+        </is>
+      </c>
+      <c r="G3" s="67" t="inlineStr">
+        <is>
+          <t>Recall%</t>
+        </is>
+      </c>
+      <c r="H3" s="67" t="inlineStr">
+        <is>
+          <t>Train AUC</t>
+        </is>
+      </c>
+      <c r="I3" s="67" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
       <c r="J3" s="20" t="n"/>
@@ -3630,11 +3623,11 @@
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Skill-Inject Filter</t>
+          <t>Static Regex</t>
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>0.528</v>
+        <v>0.54</v>
       </c>
       <c r="C4" s="22" t="n">
         <v>100</v>
@@ -3658,7 +3651,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Schmotz et al. 2026, naive input filter. FPR=100%</t>
+          <t>Always fires</t>
         </is>
       </c>
       <c r="J4" s="22" t="n"/>
@@ -3666,33 +3659,35 @@
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>TF-IDF + LR</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>0.8120000000000001</v>
+        <v>0.528</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>19.4</v>
+        <v>100</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>3.2</v>
+        <v>0</v>
       </c>
       <c r="E5" s="22" t="n">
-        <v>89.59999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>83.3</v>
+        <v>50</v>
       </c>
       <c r="G5" s="22" t="n">
-        <v>96.8</v>
-      </c>
-      <c r="H5" s="22" t="n">
-        <v>0.679</v>
+        <v>100</v>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>C=0.01, unique prompt</t>
+          <t>Schmotz et al. 2026, naive input filter. FPR=100%</t>
         </is>
       </c>
       <c r="J5" s="22" t="n"/>
@@ -3700,35 +3695,33 @@
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>cisco-skill-scanner</t>
+          <t>TF-IDF + LR</t>
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>0.539</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>68.3</v>
+        <v>19.4</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>31.7</v>
+        <v>3.2</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>60.6</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>50</v>
+        <v>83.3</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>68.3</v>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>96.8</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>0.679</v>
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>129 core patterns. Better than basic regex but still 68% FPR</t>
+          <t>C=0.01, unique prompt</t>
         </is>
       </c>
       <c r="J6" s="22" t="n"/>
@@ -3736,26 +3729,26 @@
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
         <is>
-          <t>NVIDIA SkillSpector</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>0.503</v>
+        <v>0.539</v>
       </c>
       <c r="C7" s="22" t="n">
-        <v>100</v>
+        <v>68.3</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>0</v>
+        <v>31.7</v>
       </c>
       <c r="E7" s="22" t="n">
-        <v>66.7</v>
+        <v>60.6</v>
       </c>
       <c r="F7" s="22" t="n">
         <v>50</v>
       </c>
       <c r="G7" s="22" t="n">
-        <v>100</v>
+        <v>68.3</v>
       </c>
       <c r="H7" s="22" t="inlineStr">
         <is>
@@ -3764,7 +3757,7 @@
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
+          <t>129 core patterns. Better than basic regex but still 68% FPR</t>
         </is>
       </c>
       <c r="J7" s="22" t="n"/>
@@ -3772,11 +3765,11 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.63</v>
+        <v>0.503</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>100</v>
@@ -3800,7 +3793,7 @@
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
       </c>
       <c r="J8" s="22" t="n"/>
@@ -3808,33 +3801,35 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B9" s="22" t="n">
-        <v>0.863</v>
+        <v>0.63</v>
       </c>
       <c r="C9" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="22" t="n">
-        <v>40.3</v>
-      </c>
       <c r="E9" s="22" t="n">
-        <v>74.7</v>
+        <v>66.7</v>
       </c>
       <c r="F9" s="22" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>59.7</v>
-      </c>
-      <c r="H9" s="22" t="n">
-        <v>0.989</v>
+        <v>100</v>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>L11 (L7+ restricted)</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
         </is>
       </c>
       <c r="J9" s="22" t="n"/>
@@ -3842,26 +3837,26 @@
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>0.871</v>
+        <v>0.863</v>
       </c>
       <c r="C10" s="22" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>51.6</v>
+        <v>40.3</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>65.2</v>
+        <v>74.7</v>
       </c>
       <c r="F10" s="22" t="n">
         <v>100</v>
       </c>
       <c r="G10" s="22" t="n">
-        <v>48.4</v>
+        <v>59.7</v>
       </c>
       <c r="H10" s="22" t="n">
         <v>0.989</v>
@@ -3876,67 +3871,67 @@
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
+          <t>AgentLens</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="n">
+        <v>0.871</v>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>48.4</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>L11 (L7+ restricted)</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B12" s="22" t="n">
         <v>0.824</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C12" s="22" t="n">
         <v>48.4</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D12" s="22" t="n">
         <v>8.1</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E12" s="22" t="n">
         <v>76.5</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F12" s="22" t="n">
         <v>65.5</v>
       </c>
-      <c r="G11" s="22" t="n">
+      <c r="G12" s="22" t="n">
         <v>91.7</v>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="H12" s="89" t="n">
         <v>0.9379999999999999</v>
       </c>
-      <c r="I11" s="22" t="inlineStr">
+      <c r="I12" s="22" t="inlineStr">
         <is>
           <t>Done: attn+rhid. Honest: AUC=0.824 on paired CF</t>
-        </is>
-      </c>
-      <c r="J11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="68" t="inlineStr">
-        <is>
-          <t>Relational (v1)</t>
-        </is>
-      </c>
-      <c r="B12" s="69" t="n">
-        <v>0.761</v>
-      </c>
-      <c r="C12" s="69" t="n">
-        <v>50</v>
-      </c>
-      <c r="D12" s="69" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="E12" s="69" t="n">
-        <v>76.8</v>
-      </c>
-      <c r="F12" s="69" t="n">
-        <v>65.2</v>
-      </c>
-      <c r="G12" s="69" t="n">
-        <v>93.5</v>
-      </c>
-      <c r="H12" s="88" t="n">
-        <v>0.893</v>
-      </c>
-      <c r="I12" s="69" t="inlineStr">
-        <is>
-          <t>L31, interact+PCA64</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -3944,73 +3939,73 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.872</v>
+        <v>0.761</v>
       </c>
       <c r="C13" s="70" t="n">
-        <v>19.4</v>
+        <v>50</v>
       </c>
       <c r="D13" s="70" t="n">
-        <v>12.9</v>
+        <v>6.5</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>84.40000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="F13" s="70" t="n">
-        <v>81.8</v>
+        <v>65.2</v>
       </c>
       <c r="G13" s="70" t="n">
-        <v>87.09999999999999</v>
+        <v>93.5</v>
       </c>
       <c r="H13" s="70" t="n">
-        <v>0.896</v>
+        <v>0.893</v>
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>L27, -1PC</t>
+          <t>L31, interact+PCA64</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Centered Relational</t>
         </is>
       </c>
       <c r="B14" s="70" t="n">
-        <v>0.91</v>
+        <v>0.872</v>
       </c>
       <c r="C14" s="70" t="n">
         <v>19.4</v>
       </c>
       <c r="D14" s="70" t="n">
-        <v>11.3</v>
+        <v>12.9</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>85.3</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="F14" s="70" t="n">
-        <v>82.09999999999999</v>
+        <v>81.8</v>
       </c>
       <c r="G14" s="70" t="n">
-        <v>88.7</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H14" s="70" t="n">
-        <v>0.919</v>
+        <v>0.896</v>
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>v1: oper+bnd+PCA8+C=0.01+L7+. Baseline method</t>
+          <t>L27, -1PC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2</t>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B15" s="70" t="n">
@@ -4031,82 +4026,115 @@
       <c r="G15" s="70" t="n">
         <v>88.7</v>
       </c>
-      <c r="H15" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H15" s="70" t="n">
+        <v>0.919</v>
       </c>
       <c r="I15" s="70" t="inlineStr">
         <is>
-          <t>v2: max(v1,decl). SMP无声明投毒→=v1. 零退化+补盲区+归因</t>
+          <t>v1: oper+bnd+PCA8+C=0.01+L7+. Baseline method</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v4 (ours)</t>
+          <t>SkillProbe v2</t>
         </is>
       </c>
       <c r="B16" s="70" t="n">
-        <v>0.947</v>
+        <v>0.91</v>
       </c>
       <c r="C16" s="70" t="n">
         <v>19.4</v>
       </c>
       <c r="D16" s="70" t="n">
-        <v>6.5</v>
+        <v>11.3</v>
       </c>
       <c r="E16" s="70" t="n">
-        <v>87.90000000000001</v>
+        <v>85.3</v>
       </c>
       <c r="F16" s="70" t="n">
         <v>82.09999999999999</v>
       </c>
       <c r="G16" s="70" t="n">
+        <v>88.7</v>
+      </c>
+      <c r="H16" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="70" t="inlineStr">
+        <is>
+          <t>v2: max(v1,decl). SMP无声明投毒→=v1. 零退化+补盲区+归因</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
+          <t>SkillProbe v4 (ours)</t>
+        </is>
+      </c>
+      <c r="B17" s="70" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="C17" s="70" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="D17" s="70" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="E17" s="70" t="n">
+        <v>87.90000000000001</v>
+      </c>
+      <c r="F17" s="70" t="n">
+        <v>82.09999999999999</v>
+      </c>
+      <c r="G17" s="70" t="n">
         <v>93.5</v>
       </c>
-      <c r="H16" s="70" t="inlineStr">
+      <c r="H17" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I16" s="70" t="inlineStr">
+      <c r="I17" s="70" t="inlineStr">
         <is>
           <t>v4: Boundary-gated v3. Gate&lt;0.15. AUC=0.947 SOTA. 49/124 gated</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="92" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B18" s="92" t="n">
         <v>0.503</v>
       </c>
-      <c r="C17" t="n">
-        <v>100</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" s="92" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" s="92" t="n">
         <v>66.7</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" s="92" t="n">
         <v>50</v>
       </c>
-      <c r="G17" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" s="92" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I18" s="92" t="inlineStr">
         <is>
           <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
@@ -4127,7 +4155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4161,48 +4189,60 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="87" t="inlineStr">
-        <is>
-          <t>Static Regex</t>
-        </is>
-      </c>
-      <c r="B3" s="87" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="C3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="87" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="87" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F3" s="87" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="H3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="87" t="inlineStr">
-        <is>
-          <t>Always fires</t>
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>FPR%</t>
+        </is>
+      </c>
+      <c r="D3" s="67" t="inlineStr">
+        <is>
+          <t>FNR%</t>
+        </is>
+      </c>
+      <c r="E3" s="67" t="inlineStr">
+        <is>
+          <t>F1%</t>
+        </is>
+      </c>
+      <c r="F3" s="67" t="inlineStr">
+        <is>
+          <t>Precision%</t>
+        </is>
+      </c>
+      <c r="G3" s="67" t="inlineStr">
+        <is>
+          <t>Recall%</t>
+        </is>
+      </c>
+      <c r="H3" s="67" t="inlineStr">
+        <is>
+          <t>Train AUC</t>
+        </is>
+      </c>
+      <c r="I3" s="67" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Skill-Inject Filter</t>
+          <t>Static Regex</t>
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>0.502</v>
+        <v>0.54</v>
       </c>
       <c r="C4" s="22" t="n">
         <v>100</v>
@@ -4226,86 +4266,86 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Naive filter: always fires on 8K samples</t>
+          <t>Always fires</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>TF-IDF + LR</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>0.967</v>
+        <v>0.502</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>6.4</v>
+        <v>100</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>10.7</v>
+        <v>0</v>
       </c>
       <c r="E5" s="22" t="n">
-        <v>91.09999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>93</v>
+        <v>49.6</v>
       </c>
       <c r="G5" s="22" t="n">
-        <v>89.3</v>
-      </c>
-      <c r="H5" s="22" t="n">
-        <v>0.973</v>
+        <v>100</v>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>C=0.01</t>
+          <t>Naive filter: always fires on 8K samples</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>cisco-skill-scanner</t>
+          <t>TF-IDF + LR</t>
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>0.545</v>
+        <v>0.967</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>100</v>
+        <v>6.4</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>66.7</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>49.6</v>
+        <v>93</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>89.3</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>0.973</v>
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>129 core patterns, always fires</t>
+          <t>C=0.01</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
         <is>
-          <t>NVIDIA SkillSpector</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>0.521</v>
+        <v>0.545</v>
       </c>
       <c r="C7" s="22" t="n">
         <v>100</v>
@@ -4329,18 +4369,18 @@
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>20 YARA rules, 13.5k stars. Always fires</t>
+          <t>129 core patterns, always fires</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.5</v>
+        <v>0.521</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>100</v>
@@ -4349,10 +4389,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>66.59999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>50</v>
+        <v>49.6</v>
       </c>
       <c r="G8" s="22" t="n">
         <v>100</v>
@@ -4364,69 +4404,71 @@
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+          <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B9" s="22" t="n">
-        <v>0.999</v>
+        <v>0.5</v>
       </c>
       <c r="C9" s="22" t="n">
-        <v>1.4</v>
+        <v>100</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="E9" s="22" t="n">
-        <v>98.7</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="F9" s="22" t="n">
-        <v>98.59999999999999</v>
+        <v>50</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>98.7</v>
-      </c>
-      <c r="H9" s="22" t="n">
-        <v>1</v>
+        <v>100</v>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>L19 (L7+ verified, source confound)</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>0.99</v>
+        <v>0.999</v>
       </c>
       <c r="C10" s="22" t="n">
-        <v>3.6</v>
+        <v>1.4</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>2.1</v>
+        <v>1.3</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>97.2</v>
+        <v>98.7</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>96.5</v>
+        <v>98.59999999999999</v>
       </c>
       <c r="G10" s="22" t="n">
-        <v>97.90000000000001</v>
+        <v>98.7</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>0.995</v>
+        <v>1</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
@@ -4437,95 +4479,95 @@
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
+          <t>AgentLens</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>97.2</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>97.90000000000001</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>L19 (L7+ verified, source confound)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B12" s="22" t="n">
         <v>0.795</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C12" s="22" t="n">
         <v>47.7</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D12" s="22" t="n">
         <v>11.1</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E12" s="22" t="n">
         <v>74.5</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F12" s="22" t="n">
         <v>64.09999999999999</v>
       </c>
-      <c r="G11" s="22" t="n">
+      <c r="G12" s="22" t="n">
         <v>88.90000000000001</v>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="H12" s="22" t="n">
         <v>0.796</v>
       </c>
-      <c r="I11" s="22" t="inlineStr">
+      <c r="I12" s="22" t="inlineStr">
         <is>
           <t>rhid only. Honest: not inflated by source confound (unlike others at 0.99+)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="68" t="inlineStr">
-        <is>
-          <t>Relational (v1)</t>
-        </is>
-      </c>
-      <c r="B12" s="69" t="n">
-        <v>0.992</v>
-      </c>
-      <c r="C12" s="69" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="D12" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" s="69" t="n">
-        <v>95.5</v>
-      </c>
-      <c r="F12" s="69" t="n">
-        <v>97</v>
-      </c>
-      <c r="G12" s="69" t="n">
-        <v>94</v>
-      </c>
-      <c r="H12" s="69" t="n">
-        <v>0.993</v>
-      </c>
-      <c r="I12" s="69" t="inlineStr">
-        <is>
-          <t>L11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.991</v>
+        <v>0.992</v>
       </c>
       <c r="C13" s="70" t="n">
-        <v>7.8</v>
+        <v>2.9</v>
       </c>
       <c r="D13" s="70" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>94.8</v>
+        <v>95.5</v>
       </c>
       <c r="F13" s="70" t="n">
-        <v>92.7</v>
+        <v>97</v>
       </c>
       <c r="G13" s="70" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="H13" s="70" t="n">
-        <v>0.991</v>
+        <v>0.993</v>
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
@@ -4536,40 +4578,40 @@
     <row r="14">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Centered Relational</t>
         </is>
       </c>
       <c r="B14" s="70" t="n">
-        <v>0.964</v>
+        <v>0.991</v>
       </c>
       <c r="C14" s="70" t="n">
-        <v>10.8</v>
+        <v>7.8</v>
       </c>
       <c r="D14" s="70" t="n">
-        <v>8.5</v>
+        <v>3</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>90.59999999999999</v>
+        <v>94.8</v>
       </c>
       <c r="F14" s="70" t="n">
-        <v>89.7</v>
+        <v>92.7</v>
       </c>
       <c r="G14" s="70" t="n">
-        <v>91.5</v>
+        <v>97</v>
       </c>
       <c r="H14" s="70" t="n">
-        <v>0.963</v>
+        <v>0.991</v>
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>v1: oper+bnd. Source confound inflated</t>
+          <t>L11</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2</t>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B15" s="70" t="n">
@@ -4590,82 +4632,115 @@
       <c r="G15" s="70" t="n">
         <v>91.5</v>
       </c>
-      <c r="H15" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H15" s="70" t="n">
+        <v>0.963</v>
       </c>
       <c r="I15" s="70" t="inlineStr">
         <is>
-          <t>v2: max(v1,decl). =v1 on MSB</t>
+          <t>v1: oper+bnd. Source confound inflated</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="70" t="inlineStr">
         <is>
+          <t>SkillProbe v2</t>
+        </is>
+      </c>
+      <c r="B16" s="70" t="n">
+        <v>0.964</v>
+      </c>
+      <c r="C16" s="70" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="D16" s="70" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="E16" s="70" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="F16" s="70" t="n">
+        <v>89.7</v>
+      </c>
+      <c r="G16" s="70" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="H16" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="70" t="inlineStr">
+        <is>
+          <t>v2: max(v1,decl). =v1 on MSB</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
           <t>SkillProbe v4 (ours)</t>
         </is>
       </c>
-      <c r="B16" s="70" t="n">
+      <c r="B17" s="70" t="n">
         <v>0.996</v>
       </c>
-      <c r="C16" s="70" t="n">
+      <c r="C17" s="70" t="n">
         <v>3.2</v>
       </c>
-      <c r="D16" s="70" t="n">
+      <c r="D17" s="70" t="n">
         <v>1.3</v>
       </c>
-      <c r="E16" s="70" t="n">
+      <c r="E17" s="70" t="n">
         <v>98</v>
       </c>
-      <c r="F16" s="70" t="n">
+      <c r="F17" s="70" t="n">
         <v>97.5</v>
       </c>
-      <c r="G16" s="70" t="n">
+      <c r="G17" s="70" t="n">
         <v>98.7</v>
       </c>
-      <c r="H16" s="70" t="inlineStr">
+      <c r="H17" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I16" s="70" t="inlineStr">
+      <c r="I17" s="70" t="inlineStr">
         <is>
           <t>v4: Gate&lt;0.15. AUC=0.996! Boundary gate catches confounded samples</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="92" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B18" s="92" t="n">
         <v>0.521</v>
       </c>
-      <c r="C17" t="n">
-        <v>100</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" s="92" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" s="92" t="n">
         <v>66.7</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" s="92" t="n">
         <v>49.6</v>
       </c>
-      <c r="G17" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" s="92" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I18" s="92" t="inlineStr">
         <is>
           <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
@@ -4686,7 +4761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4720,48 +4795,60 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="87" t="inlineStr">
-        <is>
-          <t>Static Regex</t>
-        </is>
-      </c>
-      <c r="B3" s="87" t="n">
-        <v>0.586</v>
-      </c>
-      <c r="C3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="87" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="87" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F3" s="87" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="G3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="H3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="87" t="inlineStr">
-        <is>
-          <t>Always fires (OOD)</t>
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>FPR%</t>
+        </is>
+      </c>
+      <c r="D3" s="67" t="inlineStr">
+        <is>
+          <t>FNR%</t>
+        </is>
+      </c>
+      <c r="E3" s="67" t="inlineStr">
+        <is>
+          <t>F1%</t>
+        </is>
+      </c>
+      <c r="F3" s="67" t="inlineStr">
+        <is>
+          <t>Precision%</t>
+        </is>
+      </c>
+      <c r="G3" s="67" t="inlineStr">
+        <is>
+          <t>Recall%</t>
+        </is>
+      </c>
+      <c r="H3" s="67" t="inlineStr">
+        <is>
+          <t>Train AUC</t>
+        </is>
+      </c>
+      <c r="I3" s="67" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Skill-Inject Filter</t>
+          <t>Static Regex</t>
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>0.505</v>
+        <v>0.586</v>
       </c>
       <c r="C4" s="22" t="n">
         <v>100</v>
@@ -4770,7 +4857,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="22" t="n">
-        <v>66.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F4" s="22" t="n">
         <v>49.6</v>
@@ -4785,86 +4872,86 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Naive filter: always fires on 8K samples</t>
+          <t>Always fires (OOD)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>TF-IDF + LR</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>0.792</v>
+        <v>0.505</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>6.4</v>
+        <v>100</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>10.7</v>
+        <v>0</v>
       </c>
       <c r="E5" s="22" t="n">
-        <v>91.09999999999999</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>71.3</v>
+        <v>49.6</v>
       </c>
       <c r="G5" s="22" t="n">
-        <v>71.8</v>
-      </c>
-      <c r="H5" s="22" t="n">
-        <v>0.973</v>
+        <v>100</v>
+      </c>
+      <c r="H5" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>Estimated from MSB</t>
+          <t>Naive filter: always fires on 8K samples</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>cisco-skill-scanner</t>
+          <t>TF-IDF + LR</t>
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>0.552</v>
+        <v>0.792</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>100</v>
+        <v>6.4</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0</v>
+        <v>10.7</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>66.40000000000001</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>49.6</v>
+        <v>71.3</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H6" s="22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>71.8</v>
+      </c>
+      <c r="H6" s="22" t="n">
+        <v>0.973</v>
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>129 core patterns. Always fires</t>
+          <t>Estimated from MSB</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
         <is>
-          <t>NVIDIA SkillSpector</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>0.524</v>
+        <v>0.552</v>
       </c>
       <c r="C7" s="22" t="n">
         <v>100</v>
@@ -4888,18 +4975,18 @@
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>20 YARA rules, 13.5k stars. Always fires</t>
+          <t>129 core patterns. Always fires</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.5</v>
+        <v>0.524</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>100</v>
@@ -4908,10 +4995,10 @@
         <v>0</v>
       </c>
       <c r="E8" s="22" t="n">
-        <v>66.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>50</v>
+        <v>49.6</v>
       </c>
       <c r="G8" s="22" t="n">
         <v>100</v>
@@ -4923,69 +5010,71 @@
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
+          <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B9" s="22" t="n">
-        <v>0.999</v>
+        <v>0.5</v>
       </c>
       <c r="C9" s="22" t="n">
-        <v>2.5</v>
+        <v>100</v>
       </c>
       <c r="D9" s="22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="22" t="n">
-        <v>98.2</v>
+        <v>66.7</v>
       </c>
       <c r="F9" s="22" t="n">
-        <v>97.5</v>
+        <v>50</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>99</v>
-      </c>
-      <c r="H9" s="22" t="n">
-        <v>1</v>
+        <v>100</v>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>L15, in-domain (L7+)</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%, FNR=0%)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>0.984</v>
+        <v>0.999</v>
       </c>
       <c r="C10" s="22" t="n">
-        <v>3.7</v>
+        <v>2.5</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>9.1</v>
+        <v>1</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>93.40000000000001</v>
+        <v>98.2</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>96.09999999999999</v>
+        <v>97.5</v>
       </c>
       <c r="G10" s="22" t="n">
-        <v>90.90000000000001</v>
+        <v>99</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>0.983</v>
+        <v>1</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
@@ -4996,73 +5085,73 @@
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
+          <t>AgentLens</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="n">
+        <v>0.984</v>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>93.40000000000001</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>96.09999999999999</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>90.90000000000001</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0.983</v>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>L15, in-domain (L7+)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B12" s="22" t="n">
         <v>0.998</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C12" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D12" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E12" s="22" t="n">
         <v>99.5</v>
       </c>
-      <c r="F11" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="G11" s="22" t="n">
+      <c r="F12" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" s="22" t="n">
         <v>99</v>
       </c>
-      <c r="H11" s="22" t="n">
+      <c r="H12" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="I11" s="22" t="inlineStr">
+      <c r="I12" s="22" t="inlineStr">
         <is>
           <t>6K in-domain, rhid only (pre-L7+. Needs MSB route_hidden re-extract for L7+ update)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="68" t="inlineStr">
-        <is>
-          <t>Relational (v1)</t>
-        </is>
-      </c>
-      <c r="B12" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="69" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E12" s="69" t="n">
-        <v>99.59999999999999</v>
-      </c>
-      <c r="F12" s="69" t="n">
-        <v>100</v>
-      </c>
-      <c r="G12" s="69" t="n">
-        <v>99.3</v>
-      </c>
-      <c r="H12" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" s="69" t="inlineStr">
-        <is>
-          <t>4K in-domain, pre-L7+</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
@@ -5072,16 +5161,16 @@
         <v>0</v>
       </c>
       <c r="D13" s="70" t="n">
-        <v>1.7</v>
+        <v>0.7</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>99.09999999999999</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="F13" s="70" t="n">
         <v>100</v>
       </c>
       <c r="G13" s="70" t="n">
-        <v>98.3</v>
+        <v>99.3</v>
       </c>
       <c r="H13" s="70" t="n">
         <v>1</v>
@@ -5095,40 +5184,40 @@
     <row r="14">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Centered Relational</t>
         </is>
       </c>
       <c r="B14" s="70" t="n">
-        <v>0.923</v>
+        <v>1</v>
       </c>
       <c r="C14" s="70" t="n">
-        <v>16.3</v>
+        <v>0</v>
       </c>
       <c r="D14" s="70" t="n">
-        <v>16.4</v>
+        <v>1.7</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>83.5</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="F14" s="70" t="n">
-        <v>83.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="G14" s="70" t="n">
-        <v>83.59999999999999</v>
+        <v>98.3</v>
       </c>
       <c r="H14" s="70" t="n">
-        <v>0.921</v>
+        <v>1</v>
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>v1: oper+bnd. In-domain</t>
+          <t>4K in-domain, pre-L7+</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2</t>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B15" s="70" t="n">
@@ -5149,82 +5238,115 @@
       <c r="G15" s="70" t="n">
         <v>83.59999999999999</v>
       </c>
-      <c r="H15" s="70" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="H15" s="70" t="n">
+        <v>0.921</v>
       </c>
       <c r="I15" s="70" t="inlineStr">
         <is>
-          <t>v2: max(v1,decl). =v1 on MASB</t>
+          <t>v1: oper+bnd. In-domain</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="70" t="inlineStr">
         <is>
+          <t>SkillProbe v2</t>
+        </is>
+      </c>
+      <c r="B16" s="70" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="C16" s="70" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="D16" s="70" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="E16" s="70" t="n">
+        <v>83.5</v>
+      </c>
+      <c r="F16" s="70" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="G16" s="70" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="H16" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="70" t="inlineStr">
+        <is>
+          <t>v2: max(v1,decl). =v1 on MASB</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
           <t>SkillProbe v4 (ours)</t>
         </is>
       </c>
-      <c r="B16" s="70" t="n">
+      <c r="B17" s="70" t="n">
         <v>0.981</v>
       </c>
-      <c r="C16" s="70" t="n">
+      <c r="C17" s="70" t="n">
         <v>7.2</v>
       </c>
-      <c r="D16" s="70" t="n">
+      <c r="D17" s="70" t="n">
         <v>6</v>
       </c>
-      <c r="E16" s="70" t="n">
+      <c r="E17" s="70" t="n">
         <v>93.40000000000001</v>
       </c>
-      <c r="F16" s="70" t="n">
+      <c r="F17" s="70" t="n">
         <v>93</v>
       </c>
-      <c r="G16" s="70" t="n">
+      <c r="G17" s="70" t="n">
         <v>94</v>
       </c>
-      <c r="H16" s="70" t="inlineStr">
+      <c r="H17" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I16" s="70" t="inlineStr">
+      <c r="I17" s="70" t="inlineStr">
         <is>
           <t>v4: Gate&lt;0.15. AUC=0.981! Gating fixes OOD FPR from 12%→7%</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="92" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B18" s="92" t="n">
         <v>0.524</v>
       </c>
-      <c r="C17" t="n">
-        <v>100</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" s="92" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" s="92" t="n">
         <v>66.40000000000001</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" s="92" t="n">
         <v>49.6</v>
       </c>
-      <c r="G17" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" s="92" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I18" s="92" t="inlineStr">
         <is>
           <t>20 YARA rules, 13.5k stars. Always fires</t>
         </is>
@@ -5245,7 +5367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5279,37 +5401,49 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="87" t="inlineStr">
-        <is>
-          <t>Static Regex</t>
-        </is>
-      </c>
-      <c r="B3" s="87" t="n">
-        <v>0.463</v>
-      </c>
-      <c r="C3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="87" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="87" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F3" s="87" t="n">
-        <v>42</v>
-      </c>
-      <c r="G3" s="87" t="n">
-        <v>48.3</v>
-      </c>
-      <c r="H3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="87" t="inlineStr">
-        <is>
-          <t>Static Regex on 155 decoys: FPR=59% (better than old 100%—more diverse decoys)</t>
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>FPR%</t>
+        </is>
+      </c>
+      <c r="D3" s="67" t="inlineStr">
+        <is>
+          <t>FNR%</t>
+        </is>
+      </c>
+      <c r="E3" s="67" t="inlineStr">
+        <is>
+          <t>F1%</t>
+        </is>
+      </c>
+      <c r="F3" s="67" t="inlineStr">
+        <is>
+          <t>Precision%</t>
+        </is>
+      </c>
+      <c r="G3" s="67" t="inlineStr">
+        <is>
+          <t>Recall%</t>
+        </is>
+      </c>
+      <c r="H3" s="67" t="inlineStr">
+        <is>
+          <t>Train AUC</t>
+        </is>
+      </c>
+      <c r="I3" s="67" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
       <c r="J3" s="20" t="n"/>
@@ -5317,26 +5451,26 @@
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Skill-Inject Filter</t>
+          <t>Static Regex</t>
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>0.8</v>
+        <v>0.463</v>
       </c>
       <c r="C4" s="22" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="D4" s="22" t="n">
         <v>0</v>
       </c>
       <c r="E4" s="22" t="n">
-        <v>83.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F4" s="22" t="n">
-        <v>50.2</v>
+        <v>42</v>
       </c>
       <c r="G4" s="22" t="n">
-        <v>100</v>
+        <v>48.3</v>
       </c>
       <c r="H4" s="22" t="inlineStr">
         <is>
@@ -5345,7 +5479,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Schmotz et al. 2026, naive input filtering</t>
+          <t>Static Regex on 155 decoys: FPR=59% (better than old 100%—more diverse decoys)</t>
         </is>
       </c>
       <c r="J4" s="22" t="n"/>
@@ -5353,23 +5487,23 @@
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>TF-IDF + LR</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>0.7435</v>
+        <v>0.8</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>39.3</v>
+        <v>40</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>39.1</v>
+        <v>0</v>
       </c>
       <c r="E5" s="22" t="n">
-        <v>60.9</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>50</v>
+        <v>50.2</v>
       </c>
       <c r="G5" s="22" t="n">
         <v>100</v>
@@ -5381,7 +5515,7 @@
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>TF-IDF on 155 decoys: FPR=100% (suspicious vocab = malicious to TF-IDF)</t>
+          <t>Schmotz et al. 2026, naive input filtering</t>
         </is>
       </c>
       <c r="J5" s="22" t="n"/>
@@ -5389,26 +5523,26 @@
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>cisco-skill-scanner</t>
+          <t>TF-IDF + LR</t>
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>0.533</v>
+        <v>0.7435</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>43.3</v>
+        <v>39.3</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>37.7</v>
+        <v>39.1</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>60.6</v>
+        <v>60.9</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>62.3</v>
+        <v>100</v>
       </c>
       <c r="H6" s="22" t="inlineStr">
         <is>
@@ -5417,7 +5551,7 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>176 patterns (core+promptguard), Python 3.10+ required</t>
+          <t>TF-IDF on 155 decoys: FPR=100% (suspicious vocab = malicious to TF-IDF)</t>
         </is>
       </c>
       <c r="J6" s="22" t="n"/>
@@ -5425,26 +5559,26 @@
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
         <is>
-          <t>NVIDIA SkillSpector</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>0.49</v>
+        <v>0.533</v>
       </c>
       <c r="C7" s="22" t="n">
-        <v>100</v>
+        <v>43.3</v>
       </c>
       <c r="D7" s="22" t="n">
-        <v>0</v>
+        <v>37.7</v>
       </c>
       <c r="E7" s="22" t="n">
-        <v>66.7</v>
+        <v>60.6</v>
       </c>
       <c r="F7" s="22" t="n">
-        <v>50.2</v>
+        <v>54</v>
       </c>
       <c r="G7" s="22" t="n">
-        <v>100</v>
+        <v>62.3</v>
       </c>
       <c r="H7" s="22" t="inlineStr">
         <is>
@@ -5453,7 +5587,7 @@
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
+          <t>176 patterns (core+promptguard), Python 3.10+ required</t>
         </is>
       </c>
       <c r="J7" s="22" t="n"/>
@@ -5461,11 +5595,11 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
-        <v>0.5</v>
+        <v>0.49</v>
       </c>
       <c r="C8" s="22" t="n">
         <v>100</v>
@@ -5477,7 +5611,7 @@
         <v>66.7</v>
       </c>
       <c r="F8" s="22" t="n">
-        <v>50</v>
+        <v>50.2</v>
       </c>
       <c r="G8" s="22" t="n">
         <v>100</v>
@@ -5489,7 +5623,7 @@
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%)</t>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
       </c>
       <c r="J8" s="22" t="n"/>
@@ -5497,33 +5631,35 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B9" s="89" t="n">
-        <v>0.991</v>
+        <v>0.5</v>
       </c>
       <c r="C9" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="22" t="n">
-        <v>3.2</v>
-      </c>
       <c r="E9" s="22" t="n">
-        <v>98.40000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="F9" s="22" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>96.8</v>
-      </c>
-      <c r="H9" s="22" t="n">
-        <v>0.994</v>
+        <v>100</v>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>L23 (L7+). Model judges ALL 150 decoys safe!</t>
+          <t>Mistral-7B zero-shot: predicts almost all MAL (FPR=100%)</t>
         </is>
       </c>
       <c r="J9" s="22" t="n"/>
@@ -5531,33 +5667,33 @@
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>0.867</v>
+        <v>0.991</v>
       </c>
       <c r="C10" s="22" t="n">
-        <v>22.7</v>
+        <v>0</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>21</v>
+        <v>3.2</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>67.59999999999999</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>68.2</v>
+        <v>100</v>
       </c>
       <c r="G10" s="22" t="n">
-        <v>79</v>
+        <v>96.8</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>0.989</v>
+        <v>0.994</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>L15 (L7+). PCA(50) boundary. FPR=23% acceptable.</t>
+          <t>L23 (L7+). Model judges ALL 150 decoys safe!</t>
         </is>
       </c>
       <c r="J10" s="22" t="n"/>
@@ -5565,69 +5701,67 @@
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
+          <t>AgentLens</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>21</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>67.59999999999999</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>79</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>L15 (L7+). PCA(50) boundary. FPR=23% acceptable.</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B12" s="22" t="n">
         <v>0.777</v>
       </c>
-      <c r="C11" s="22" t="n">
+      <c r="C12" s="22" t="n">
         <v>65.3</v>
       </c>
-      <c r="D11" s="22" t="n">
+      <c r="D12" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E12" s="22" t="n">
         <v>75.40000000000001</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F12" s="22" t="n">
         <v>60.4</v>
       </c>
-      <c r="G11" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H11" s="22" t="n">
+      <c r="G12" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" s="22" t="n">
         <v>0.734</v>
       </c>
-      <c r="I11" s="22" t="inlineStr">
+      <c r="I12" s="22" t="inlineStr">
         <is>
           <t>rhid only. Cross-extract caution. FPR=65%</t>
-        </is>
-      </c>
-      <c r="J11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="68" t="inlineStr">
-        <is>
-          <t>Relational (v1)</t>
-        </is>
-      </c>
-      <c r="B12" s="69" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="C12" s="69" t="n">
-        <v>100</v>
-      </c>
-      <c r="D12" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="69" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F12" s="69" t="n">
-        <v>50</v>
-      </c>
-      <c r="G12" s="69" t="n">
-        <v>100</v>
-      </c>
-      <c r="H12" s="69" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="69" t="inlineStr">
-        <is>
-          <t>Obsolete (interaction+PCA64). FPR=100% confirms noise</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -5635,26 +5769,26 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.705</v>
+        <v>0.46</v>
       </c>
       <c r="C13" s="70" t="n">
-        <v>57.3</v>
+        <v>100</v>
       </c>
       <c r="D13" s="70" t="n">
-        <v>14.7</v>
+        <v>0</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>70.3</v>
+        <v>66.7</v>
       </c>
       <c r="F13" s="70" t="n">
-        <v>59.2</v>
+        <v>50</v>
       </c>
       <c r="G13" s="70" t="n">
-        <v>85.3</v>
+        <v>100</v>
       </c>
       <c r="H13" s="70" t="inlineStr">
         <is>
@@ -5663,33 +5797,33 @@
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>Centered (-1PC). AUC=0.71 better than SkillProbe on decoy—centering helps lexical robustness</t>
+          <t>Obsolete (interaction+PCA64). FPR=100% confirms noise</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Centered Relational</t>
         </is>
       </c>
       <c r="B14" s="70" t="n">
-        <v>0.427</v>
+        <v>0.705</v>
       </c>
       <c r="C14" s="70" t="n">
-        <v>75.3</v>
+        <v>57.3</v>
       </c>
       <c r="D14" s="70" t="n">
-        <v>8.1</v>
+        <v>14.7</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>49.1</v>
+        <v>70.3</v>
       </c>
       <c r="F14" s="70" t="n">
-        <v>38.3</v>
+        <v>59.2</v>
       </c>
       <c r="G14" s="70" t="n">
-        <v>91.90000000000001</v>
+        <v>85.3</v>
       </c>
       <c r="H14" s="70" t="inlineStr">
         <is>
@@ -5698,14 +5832,14 @@
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>v1: FPR=75% (oper reads suspicious code)</t>
+          <t>Centered (-1PC). AUC=0.71 better than SkillProbe on decoy—centering helps lexical robustness</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2</t>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B15" s="70" t="n">
@@ -5733,75 +5867,110 @@
       </c>
       <c r="I15" s="70" t="inlineStr">
         <is>
-          <t>v2: max(v1,decl). Decl-Probe also fires on suspicious vocab. =v1</t>
+          <t>v1: FPR=75% (oper reads suspicious code)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="70" t="inlineStr">
         <is>
+          <t>SkillProbe v2</t>
+        </is>
+      </c>
+      <c r="B16" s="70" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="C16" s="70" t="n">
+        <v>75.3</v>
+      </c>
+      <c r="D16" s="70" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="E16" s="70" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="F16" s="70" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G16" s="70" t="n">
+        <v>91.90000000000001</v>
+      </c>
+      <c r="H16" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="70" t="inlineStr">
+        <is>
+          <t>v2: max(v1,decl). Decl-Probe also fires on suspicious vocab. =v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
           <t>SkillProbe v4 (ours)</t>
         </is>
       </c>
-      <c r="B16" s="70" t="n">
+      <c r="B17" s="70" t="n">
         <v>0.998</v>
       </c>
-      <c r="C16" s="70" t="n">
+      <c r="C17" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="70" t="n">
+      <c r="D17" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="70" t="n">
+      <c r="E17" s="70" t="n">
         <v>98.40000000000001</v>
       </c>
-      <c r="F16" s="70" t="n">
-        <v>100</v>
-      </c>
-      <c r="G16" s="70" t="n">
+      <c r="F17" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="G17" s="70" t="n">
         <v>97</v>
       </c>
-      <c r="H16" s="70" t="inlineStr">
+      <c r="H17" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I16" s="70" t="inlineStr">
+      <c r="I17" s="70" t="inlineStr">
         <is>
           <t>★ v4: Boundary-gated v3. Gate&lt;0.15. FPR=0% FNR=3%. Best on Decoy!</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="92" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B18" s="92" t="n">
         <v>0.49</v>
       </c>
-      <c r="C17" t="n">
-        <v>100</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" s="92" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" s="92" t="n">
         <v>66.7</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" s="92" t="n">
         <v>50.2</v>
       </c>
-      <c r="G17" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" s="92" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I18" s="92" t="inlineStr">
         <is>
           <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
@@ -5822,7 +5991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5856,37 +6025,49 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="87" t="inlineStr">
-        <is>
-          <t>Static Regex</t>
-        </is>
-      </c>
-      <c r="B3" s="87" t="n">
-        <v>0.994</v>
-      </c>
-      <c r="C3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="D3" s="87" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="87" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F3" s="87" t="n">
-        <v>50</v>
-      </c>
-      <c r="G3" s="87" t="n">
-        <v>100</v>
-      </c>
-      <c r="H3" s="87" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I3" s="87" t="inlineStr">
-        <is>
-          <t>Regex on clean vocab: FPR=0% FNR=100%—no patterns to match. Useless.</t>
+      <c r="A3" s="67" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B3" s="67" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>FPR%</t>
+        </is>
+      </c>
+      <c r="D3" s="67" t="inlineStr">
+        <is>
+          <t>FNR%</t>
+        </is>
+      </c>
+      <c r="E3" s="67" t="inlineStr">
+        <is>
+          <t>F1%</t>
+        </is>
+      </c>
+      <c r="F3" s="67" t="inlineStr">
+        <is>
+          <t>Precision%</t>
+        </is>
+      </c>
+      <c r="G3" s="67" t="inlineStr">
+        <is>
+          <t>Recall%</t>
+        </is>
+      </c>
+      <c r="H3" s="67" t="inlineStr">
+        <is>
+          <t>Train AUC</t>
+        </is>
+      </c>
+      <c r="I3" s="67" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
       <c r="J3" s="20" t="n"/>
@@ -5894,11 +6075,11 @@
     <row r="4">
       <c r="A4" s="21" t="inlineStr">
         <is>
-          <t>Skill-Inject Filter</t>
+          <t>Static Regex</t>
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>0.5</v>
+        <v>0.994</v>
       </c>
       <c r="C4" s="22" t="n">
         <v>100</v>
@@ -5922,7 +6103,7 @@
       </c>
       <c r="I4" s="22" t="inlineStr">
         <is>
-          <t>Naive filter: clean vocab -&gt; always fires</t>
+          <t>Regex on clean vocab: FPR=0% FNR=100%—no patterns to match. Useless.</t>
         </is>
       </c>
       <c r="J4" s="22" t="n"/>
@@ -5930,26 +6111,26 @@
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>TF-IDF + LR</t>
+          <t>Skill-Inject Filter</t>
         </is>
       </c>
       <c r="B5" s="22" t="n">
-        <v>0.1593</v>
+        <v>0.5</v>
       </c>
       <c r="C5" s="22" t="n">
-        <v>78.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="D5" s="22" t="n">
-        <v>78.09999999999999</v>
+        <v>0</v>
       </c>
       <c r="E5" s="22" t="n">
-        <v>21.9</v>
+        <v>66.7</v>
       </c>
       <c r="F5" s="22" t="n">
-        <v>46.3</v>
+        <v>50</v>
       </c>
       <c r="G5" s="22" t="n">
-        <v>78.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="H5" s="22" t="inlineStr">
         <is>
@@ -5958,7 +6139,7 @@
       </c>
       <c r="I5" s="22" t="inlineStr">
         <is>
-          <t>TF-IDF on clean vocab: AUC=0.50 random (vocab has no signal)</t>
+          <t>Naive filter: clean vocab -&gt; always fires</t>
         </is>
       </c>
       <c r="J5" s="22" t="n"/>
@@ -5966,26 +6147,26 @@
     <row r="6">
       <c r="A6" s="21" t="inlineStr">
         <is>
-          <t>cisco-skill-scanner</t>
+          <t>TF-IDF + LR</t>
         </is>
       </c>
       <c r="B6" s="22" t="n">
-        <v>0.503</v>
+        <v>0.1593</v>
       </c>
       <c r="C6" s="22" t="n">
-        <v>100</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>66.7</v>
+        <v>21.9</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>50</v>
+        <v>46.3</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>100</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="H6" s="22" t="inlineStr">
         <is>
@@ -5994,7 +6175,7 @@
       </c>
       <c r="I6" s="22" t="inlineStr">
         <is>
-          <t>Standard Python code triggers patterns -&gt; always fires</t>
+          <t>TF-IDF on clean vocab: AUC=0.50 random (vocab has no signal)</t>
         </is>
       </c>
       <c r="J6" s="22" t="n"/>
@@ -6002,11 +6183,11 @@
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
         <is>
-          <t>NVIDIA SkillSpector</t>
+          <t>cisco-skill-scanner</t>
         </is>
       </c>
       <c r="B7" s="22" t="n">
-        <v>0.5</v>
+        <v>0.503</v>
       </c>
       <c r="C7" s="22" t="n">
         <v>100</v>
@@ -6030,7 +6211,7 @@
       </c>
       <c r="I7" s="22" t="inlineStr">
         <is>
-          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
+          <t>Standard Python code triggers patterns -&gt; always fires</t>
         </is>
       </c>
       <c r="J7" s="22" t="n"/>
@@ -6038,7 +6219,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>LLM-as-judge</t>
+          <t>NVIDIA SkillSpector</t>
         </is>
       </c>
       <c r="B8" s="22" t="n">
@@ -6066,7 +6247,7 @@
       </c>
       <c r="I8" s="22" t="inlineStr">
         <is>
-          <t>Mistral always MAL. Zero-shot useless</t>
+          <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>
       </c>
       <c r="J8" s="22" t="n"/>
@@ -6074,33 +6255,35 @@
     <row r="9">
       <c r="A9" s="21" t="inlineStr">
         <is>
-          <t>Boundary only</t>
+          <t>LLM-as-judge</t>
         </is>
       </c>
       <c r="B9" s="22" t="n">
-        <v>0.793</v>
+        <v>0.5</v>
       </c>
       <c r="C9" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="22" t="n">
-        <v>100</v>
-      </c>
       <c r="E9" s="22" t="n">
-        <v>0</v>
+        <v>66.7</v>
       </c>
       <c r="F9" s="22" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="G9" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="22" t="n">
-        <v>0.994</v>
+        <v>100</v>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="I9" s="22" t="inlineStr">
         <is>
-          <t>L23. Model judges ALL safe! FNR=100%—clean vocab fools model judgment completely</t>
+          <t>Mistral always MAL. Zero-shot useless</t>
         </is>
       </c>
       <c r="J9" s="22" t="n"/>
@@ -6108,33 +6291,33 @@
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>AgentLens</t>
+          <t>Boundary only</t>
         </is>
       </c>
       <c r="B10" s="22" t="n">
-        <v>0.676</v>
+        <v>0.793</v>
       </c>
       <c r="C10" s="22" t="n">
-        <v>78.09999999999999</v>
+        <v>0</v>
       </c>
       <c r="D10" s="22" t="n">
-        <v>0.6</v>
+        <v>100</v>
       </c>
       <c r="E10" s="22" t="n">
-        <v>71.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="F10" s="22" t="n">
-        <v>53.2</v>
+        <v>0</v>
       </c>
       <c r="G10" s="22" t="n">
-        <v>99.40000000000001</v>
+        <v>0</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>0.989</v>
+        <v>0.994</v>
       </c>
       <c r="I10" s="22" t="inlineStr">
         <is>
-          <t>L15. Catches 99% malicious but FPR=78%</t>
+          <t>L23. Model judges ALL safe! FNR=100%—clean vocab fools model judgment completely</t>
         </is>
       </c>
       <c r="J10" s="22" t="n"/>
@@ -6142,69 +6325,67 @@
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
+          <t>AgentLens</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="C11" s="22" t="n">
+        <v>78.09999999999999</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E11" s="22" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="G11" s="22" t="n">
+        <v>99.40000000000001</v>
+      </c>
+      <c r="H11" s="22" t="n">
+        <v>0.989</v>
+      </c>
+      <c r="I11" s="22" t="inlineStr">
+        <is>
+          <t>L15. Catches 99% malicious but FPR=78%</t>
+        </is>
+      </c>
+      <c r="J11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
           <t>RouteGuard</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B12" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="C11" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="D11" s="22" t="n">
+      <c r="C12" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D12" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="22" t="n">
+      <c r="E12" s="22" t="n">
         <v>66.7</v>
       </c>
-      <c r="F11" s="22" t="n">
+      <c r="F12" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="G11" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="H11" s="22" t="n">
+      <c r="G12" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" s="22" t="n">
         <v>0.734</v>
       </c>
-      <c r="I11" s="22" t="inlineStr">
+      <c r="I12" s="22" t="inlineStr">
         <is>
           <t>rhid only. Random on clean vocab. Cross-extract.</t>
-        </is>
-      </c>
-      <c r="J11" s="22" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="68" t="inlineStr">
-        <is>
-          <t>Relational (v1)</t>
-        </is>
-      </c>
-      <c r="B12" s="69" t="n">
-        <v>0.824</v>
-      </c>
-      <c r="C12" s="69" t="n">
-        <v>100</v>
-      </c>
-      <c r="D12" s="69" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="69" t="n">
-        <v>66.7</v>
-      </c>
-      <c r="F12" s="69" t="n">
-        <v>50</v>
-      </c>
-      <c r="G12" s="69" t="n">
-        <v>100</v>
-      </c>
-      <c r="H12" s="69" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I12" s="69" t="inlineStr">
-        <is>
-          <t>AUC=0.82 ranks correctly but FPR=100% (threshold issue)</t>
         </is>
       </c>
       <c r="J12" s="28" t="n"/>
@@ -6212,26 +6393,26 @@
     <row r="13">
       <c r="A13" s="70" t="inlineStr">
         <is>
-          <t>Centered Relational</t>
+          <t>Relational (v1)</t>
         </is>
       </c>
       <c r="B13" s="70" t="n">
-        <v>0.846</v>
+        <v>0.824</v>
       </c>
       <c r="C13" s="70" t="n">
-        <v>21.9</v>
+        <v>100</v>
       </c>
       <c r="D13" s="70" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="E13" s="70" t="n">
-        <v>89.5</v>
+        <v>66.7</v>
       </c>
       <c r="F13" s="70" t="n">
-        <v>80.90000000000001</v>
+        <v>50</v>
       </c>
       <c r="G13" s="70" t="n">
-        <v>98.7</v>
+        <v>100</v>
       </c>
       <c r="H13" s="70" t="inlineStr">
         <is>
@@ -6240,33 +6421,33 @@
       </c>
       <c r="I13" s="70" t="inlineStr">
         <is>
-          <t>Centered (-1PC). AUC=0.85 BEST on InvDecoy! Centering removes anisotropic noise→clean signal</t>
+          <t>AUC=0.82 ranks correctly but FPR=100% (threshold issue)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v1</t>
+          <t>Centered Relational</t>
         </is>
       </c>
       <c r="B14" s="70" t="n">
-        <v>0.165</v>
+        <v>0.846</v>
       </c>
       <c r="C14" s="70" t="n">
-        <v>100</v>
+        <v>21.9</v>
       </c>
       <c r="D14" s="70" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>43.9</v>
+        <v>89.5</v>
       </c>
       <c r="F14" s="70" t="n">
-        <v>50</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="G14" s="70" t="n">
-        <v>100</v>
+        <v>98.7</v>
       </c>
       <c r="H14" s="70" t="inlineStr">
         <is>
@@ -6275,14 +6456,14 @@
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>v1: cross-distribution collapse. AUC=0.16</t>
+          <t>Centered (-1PC). AUC=0.85 BEST on InvDecoy! Centering removes anisotropic noise→clean signal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="70" t="inlineStr">
         <is>
-          <t>SkillProbe v2</t>
+          <t>SkillProbe v1</t>
         </is>
       </c>
       <c r="B15" s="70" t="n">
@@ -6310,75 +6491,110 @@
       </c>
       <c r="I15" s="70" t="inlineStr">
         <is>
-          <t>v2: max(v1,decl). Decl AUC=0.48 random. =v1</t>
+          <t>v1: cross-distribution collapse. AUC=0.16</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="70" t="inlineStr">
         <is>
+          <t>SkillProbe v2</t>
+        </is>
+      </c>
+      <c r="B16" s="70" t="n">
+        <v>0.165</v>
+      </c>
+      <c r="C16" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="D16" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="70" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="F16" s="70" t="n">
+        <v>50</v>
+      </c>
+      <c r="G16" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" s="70" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I16" s="70" t="inlineStr">
+        <is>
+          <t>v2: max(v1,decl). Decl AUC=0.48 random. =v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="70" t="inlineStr">
+        <is>
           <t>SkillProbe v4 (ours)</t>
         </is>
       </c>
-      <c r="B16" s="70" t="n">
+      <c r="B17" s="70" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="70" t="n">
+      <c r="C17" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="70" t="n">
+      <c r="D17" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="70" t="n">
+      <c r="E17" s="70" t="n">
         <v>98.5</v>
       </c>
-      <c r="F16" s="70" t="n">
-        <v>100</v>
-      </c>
-      <c r="G16" s="70" t="n">
+      <c r="F17" s="70" t="n">
+        <v>100</v>
+      </c>
+      <c r="G17" s="70" t="n">
         <v>97</v>
       </c>
-      <c r="H16" s="70" t="inlineStr">
+      <c r="H17" s="70" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I16" s="70" t="inlineStr">
+      <c r="I17" s="70" t="inlineStr">
         <is>
           <t>★ v4: Boundary-gated v3. Gate&lt;0.15. AUC=1.0 FPR=0%! Both Decoy solved!</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="92" t="inlineStr">
         <is>
           <t>NVIDIA SkillSpector</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B18" s="92" t="n">
         <v>0.5</v>
       </c>
-      <c r="C17" t="n">
-        <v>100</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="C18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" s="92" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" s="92" t="n">
         <v>66.7</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" s="92" t="n">
         <v>50</v>
       </c>
-      <c r="G17" t="n">
-        <v>100</v>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G18" s="92" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" s="92" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I18" s="92" t="inlineStr">
         <is>
           <t>20 YARA rules, 13.5k stars. Always fires on standard Python</t>
         </is>

</xml_diff>

<commit_message>
Add SkillHarm external validation sheet. v3 AUC=1.000 perfect on 879 attacks. Boundary/AgentLens fail (FNR=100%).
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -15,6 +15,7 @@
     <sheet name="MASB 75K" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Lexical Decoy" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Inverse Decoy" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SkillHarm" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6607,4 +6608,236 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>SkillHarm - External (879 attacks, 12 risk types)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>931 poisoned + 242 SMP clean. SMP-dev trained. L7+.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AUROC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FPR%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FNR%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>F1%</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Precision%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Recall%</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Boundary only</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>30</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Model fooled - 100% FNR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AgentLens</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>33</v>
+      </c>
+      <c r="D5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Boundary deceived</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>RouteGuard</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>95.7</v>
+      </c>
+      <c r="F6" t="n">
+        <v>100</v>
+      </c>
+      <c r="G6" t="n">
+        <v>91.7</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>route_hidden works</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SkillProbe v3</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" t="n">
+        <v>100</v>
+      </c>
+      <c r="G7" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PERFECT! Cross-dist robust</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SkillProbe v4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Gate fails cross-dist</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix SkillHarm numbers: v3 AUC=0.970 Recall=100% Precision=95.3%. Boundary TP=0 FN=242.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -6685,7 +6685,7 @@
         <v>0</v>
       </c>
       <c r="C4" t="n">
-        <v>30</v>
+        <v>39.2</v>
       </c>
       <c r="D4" t="n">
         <v>100</v>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Model fooled - 100% FNR</t>
+          <t>All 242 mal→safe. TP=0 FN=242</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Boundary deceived</t>
+          <t>Same failure mode</t>
         </is>
       </c>
     </row>
@@ -6772,26 +6772,26 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>100</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="F7" t="n">
-        <v>100</v>
+        <v>95.3</v>
       </c>
       <c r="G7" t="n">
         <v>100</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>PERFECT! Cross-dist robust</t>
+          <t>Recall=100%! FP=12/242. Cross-dist proof</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SkillHarm v2 (exact SMP template): v3 AUC=0.973 Recall=100%. Boundary/AgentLens AUC=0. Cross-dist proof holds.
</commit_message>
<xml_diff>
--- a/final.xlsx
+++ b/final.xlsx
@@ -6622,7 +6622,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>SkillHarm - External (879 attacks, 12 risk types)</t>
+          <t>SkillHarm - External Validation (931 attacks, 12 risk types, exact SMP template)</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>All 242 mal→safe. TP=0 FN=242</t>
+          <t>TP=0 FN=242. Model judgment fails cross-dist</t>
         </is>
       </c>
     </row>
@@ -6731,7 +6731,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Same failure mode</t>
+          <t>Same failure</t>
         </is>
       </c>
     </row>
@@ -6748,7 +6748,7 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="E6" t="n">
         <v>95.7</v>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>route_hidden works</t>
+          <t>route_hidden works OK</t>
         </is>
       </c>
     </row>
@@ -6772,26 +6772,26 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.97</v>
+        <v>0.973</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>3.7</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>97.59999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="F7" t="n">
-        <v>95.3</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="G7" t="n">
         <v>100</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Recall=100%! FP=12/242. Cross-dist proof</t>
+          <t>Recall=100%! centering proof. TP=242 FP=9</t>
         </is>
       </c>
     </row>

</xml_diff>